<commit_message>
Daily screener update: 2026-08-24
</commit_message>
<xml_diff>
--- a/screener_history.xlsx
+++ b/screener_history.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G493"/>
+  <dimension ref="A1:G523"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -11754,6 +11754,768 @@
         </is>
       </c>
       <c r="C493" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="494">
+      <c r="A494" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="B494" t="inlineStr">
+        <is>
+          <t>ALOT</t>
+        </is>
+      </c>
+      <c r="C494" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D494" t="n">
+        <v>28.93</v>
+      </c>
+      <c r="E494" t="n">
+        <v>28.82</v>
+      </c>
+      <c r="F494" t="n">
+        <v>29.16</v>
+      </c>
+      <c r="G494" t="n">
+        <v>446</v>
+      </c>
+    </row>
+    <row r="495">
+      <c r="A495" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="B495" t="inlineStr">
+        <is>
+          <t>AZTA</t>
+        </is>
+      </c>
+      <c r="C495" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D495" t="n">
+        <v>37.49</v>
+      </c>
+      <c r="E495" t="n">
+        <v>31.9</v>
+      </c>
+      <c r="F495" t="n">
+        <v>48.67</v>
+      </c>
+      <c r="G495" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="496">
+      <c r="A496" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="B496" t="inlineStr">
+        <is>
+          <t>BFLY</t>
+        </is>
+      </c>
+      <c r="C496" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D496" t="n">
+        <v>9.789999999999999</v>
+      </c>
+      <c r="E496" t="n">
+        <v>8.359999999999999</v>
+      </c>
+      <c r="F496" t="n">
+        <v>12.65</v>
+      </c>
+      <c r="G496" t="n">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="497">
+      <c r="A497" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="B497" t="inlineStr">
+        <is>
+          <t>BNBX</t>
+        </is>
+      </c>
+      <c r="C497" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D497" t="n">
+        <v>0.18</v>
+      </c>
+      <c r="E497" t="n">
+        <v>0.13</v>
+      </c>
+      <c r="F497" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="G497" t="n">
+        <v>999</v>
+      </c>
+    </row>
+    <row r="498">
+      <c r="A498" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="B498" t="inlineStr">
+        <is>
+          <t>BYND</t>
+        </is>
+      </c>
+      <c r="C498" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D498" t="n">
+        <v>15.47</v>
+      </c>
+      <c r="E498" t="n">
+        <v>10.71</v>
+      </c>
+      <c r="F498" t="n">
+        <v>24.99</v>
+      </c>
+      <c r="G498" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="499">
+      <c r="A499" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="B499" t="inlineStr">
+        <is>
+          <t>CURX</t>
+        </is>
+      </c>
+      <c r="C499" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D499" t="n">
+        <v>6</v>
+      </c>
+      <c r="E499" t="n">
+        <v>3.84</v>
+      </c>
+      <c r="F499" t="n">
+        <v>10.32</v>
+      </c>
+      <c r="G499" t="n">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="500">
+      <c r="A500" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="B500" t="inlineStr">
+        <is>
+          <t>CXAI</t>
+        </is>
+      </c>
+      <c r="C500" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D500" t="n">
+        <v>9.449999999999999</v>
+      </c>
+      <c r="E500" t="n">
+        <v>3.44</v>
+      </c>
+      <c r="F500" t="n">
+        <v>21.46</v>
+      </c>
+      <c r="G500" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="501">
+      <c r="A501" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="B501" t="inlineStr">
+        <is>
+          <t>JUNS</t>
+        </is>
+      </c>
+      <c r="C501" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D501" t="n">
+        <v>11.2</v>
+      </c>
+      <c r="E501" t="n">
+        <v>4.56</v>
+      </c>
+      <c r="F501" t="n">
+        <v>24.48</v>
+      </c>
+      <c r="G501" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="502">
+      <c r="A502" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="B502" t="inlineStr">
+        <is>
+          <t>KIDZ</t>
+        </is>
+      </c>
+      <c r="C502" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D502" t="n">
+        <v>5.29</v>
+      </c>
+      <c r="E502" t="n">
+        <v>3.85</v>
+      </c>
+      <c r="F502" t="n">
+        <v>8.17</v>
+      </c>
+      <c r="G502" t="n">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="503">
+      <c r="A503" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="B503" t="inlineStr">
+        <is>
+          <t>LPSN</t>
+        </is>
+      </c>
+      <c r="C503" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D503" t="n">
+        <v>2.99</v>
+      </c>
+      <c r="E503" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="F503" t="n">
+        <v>3.97</v>
+      </c>
+      <c r="G503" t="n">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="504">
+      <c r="A504" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="B504" t="inlineStr">
+        <is>
+          <t>LUNG</t>
+        </is>
+      </c>
+      <c r="C504" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D504" t="n">
+        <v>2.48</v>
+      </c>
+      <c r="E504" t="n">
+        <v>2.14</v>
+      </c>
+      <c r="F504" t="n">
+        <v>3.17</v>
+      </c>
+      <c r="G504" t="n">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="505">
+      <c r="A505" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="B505" t="inlineStr">
+        <is>
+          <t>LVWR</t>
+        </is>
+      </c>
+      <c r="C505" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D505" t="n">
+        <v>1.43</v>
+      </c>
+      <c r="E505" t="n">
+        <v>1.06</v>
+      </c>
+      <c r="F505" t="n">
+        <v>2.17</v>
+      </c>
+      <c r="G505" t="n">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="506">
+      <c r="A506" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="B506" t="inlineStr">
+        <is>
+          <t>MYSZ</t>
+        </is>
+      </c>
+      <c r="C506" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D506" t="n">
+        <v>4.28</v>
+      </c>
+      <c r="E506" t="n">
+        <v>2.23</v>
+      </c>
+      <c r="F506" t="n">
+        <v>8.380000000000001</v>
+      </c>
+      <c r="G506" t="n">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="507">
+      <c r="A507" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="B507" t="inlineStr">
+        <is>
+          <t>NRDY</t>
+        </is>
+      </c>
+      <c r="C507" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D507" t="n">
+        <v>11.74</v>
+      </c>
+      <c r="E507" t="n">
+        <v>9.15</v>
+      </c>
+      <c r="F507" t="n">
+        <v>16.94</v>
+      </c>
+      <c r="G507" t="n">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="508">
+      <c r="A508" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="B508" t="inlineStr">
+        <is>
+          <t>OPAD</t>
+        </is>
+      </c>
+      <c r="C508" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D508" t="n">
+        <v>4.94</v>
+      </c>
+      <c r="E508" t="n">
+        <v>4.01</v>
+      </c>
+      <c r="F508" t="n">
+        <v>6.78</v>
+      </c>
+      <c r="G508" t="n">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="509">
+      <c r="A509" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="B509" t="inlineStr">
+        <is>
+          <t>PUBM</t>
+        </is>
+      </c>
+      <c r="C509" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D509" t="n">
+        <v>18.2</v>
+      </c>
+      <c r="E509" t="n">
+        <v>16.03</v>
+      </c>
+      <c r="F509" t="n">
+        <v>22.54</v>
+      </c>
+      <c r="G509" t="n">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="510">
+      <c r="A510" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="B510" t="inlineStr">
+        <is>
+          <t>REPL</t>
+        </is>
+      </c>
+      <c r="C510" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D510" t="n">
+        <v>15.7</v>
+      </c>
+      <c r="E510" t="n">
+        <v>13.2</v>
+      </c>
+      <c r="F510" t="n">
+        <v>20.72</v>
+      </c>
+      <c r="G510" t="n">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="511">
+      <c r="A511" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="B511" t="inlineStr">
+        <is>
+          <t>SGRP</t>
+        </is>
+      </c>
+      <c r="C511" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D511" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="E511" t="n">
+        <v>0.62</v>
+      </c>
+      <c r="F511" t="n">
+        <v>0.86</v>
+      </c>
+      <c r="G511" t="n">
+        <v>625</v>
+      </c>
+    </row>
+    <row r="512">
+      <c r="A512" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="B512" t="inlineStr">
+        <is>
+          <t>SMXT</t>
+        </is>
+      </c>
+      <c r="C512" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D512" t="n">
+        <v>4.9</v>
+      </c>
+      <c r="E512" t="n">
+        <v>3.42</v>
+      </c>
+      <c r="F512" t="n">
+        <v>7.87</v>
+      </c>
+      <c r="G512" t="n">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="513">
+      <c r="A513" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="B513" t="inlineStr">
+        <is>
+          <t>STIM</t>
+        </is>
+      </c>
+      <c r="C513" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D513" t="n">
+        <v>3.44</v>
+      </c>
+      <c r="E513" t="n">
+        <v>2.71</v>
+      </c>
+      <c r="F513" t="n">
+        <v>4.9</v>
+      </c>
+      <c r="G513" t="n">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="514">
+      <c r="A514" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="B514" t="inlineStr">
+        <is>
+          <t>TTRX</t>
+        </is>
+      </c>
+      <c r="C514" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D514" t="n">
+        <v>10.95</v>
+      </c>
+      <c r="E514" t="n">
+        <v>9.039999999999999</v>
+      </c>
+      <c r="F514" t="n">
+        <v>14.78</v>
+      </c>
+      <c r="G514" t="n">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="515">
+      <c r="A515" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="B515" t="inlineStr">
+        <is>
+          <t>ANTX</t>
+        </is>
+      </c>
+      <c r="C515" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="516">
+      <c r="A516" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="B516" t="inlineStr">
+        <is>
+          <t>DUKR</t>
+        </is>
+      </c>
+      <c r="C516" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="517">
+      <c r="A517" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="B517" t="inlineStr">
+        <is>
+          <t>FATN</t>
+        </is>
+      </c>
+      <c r="C517" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="518">
+      <c r="A518" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="B518" t="inlineStr">
+        <is>
+          <t>FBRX</t>
+        </is>
+      </c>
+      <c r="C518" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="519">
+      <c r="A519" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="B519" t="inlineStr">
+        <is>
+          <t>FIRY</t>
+        </is>
+      </c>
+      <c r="C519" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="520">
+      <c r="A520" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="B520" t="inlineStr">
+        <is>
+          <t>HZO</t>
+        </is>
+      </c>
+      <c r="C520" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="521">
+      <c r="A521" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="B521" t="inlineStr">
+        <is>
+          <t>LCUT</t>
+        </is>
+      </c>
+      <c r="C521" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="522">
+      <c r="A522" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="B522" t="inlineStr">
+        <is>
+          <t>NAVN</t>
+        </is>
+      </c>
+      <c r="C522" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="523">
+      <c r="A523" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="B523" t="inlineStr">
+        <is>
+          <t>QLYS</t>
+        </is>
+      </c>
+      <c r="C523" t="inlineStr">
         <is>
           <t>Dropped</t>
         </is>
@@ -11770,7 +12532,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G663"/>
+  <dimension ref="A1:G675"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -26992,6 +27754,318 @@
         </is>
       </c>
       <c r="C663" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="664">
+      <c r="A664" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="B664" t="inlineStr">
+        <is>
+          <t>APRE</t>
+        </is>
+      </c>
+      <c r="C664" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D664" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="E664" t="n">
+        <v>0.68</v>
+      </c>
+      <c r="F664" t="n">
+        <v>0.74</v>
+      </c>
+      <c r="G664" t="n">
+        <v>2512</v>
+      </c>
+    </row>
+    <row r="665">
+      <c r="A665" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="B665" t="inlineStr">
+        <is>
+          <t>CAPR</t>
+        </is>
+      </c>
+      <c r="C665" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D665" t="n">
+        <v>8.02</v>
+      </c>
+      <c r="E665" t="n">
+        <v>6.34</v>
+      </c>
+      <c r="F665" t="n">
+        <v>11.37</v>
+      </c>
+      <c r="G665" t="n">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="666">
+      <c r="A666" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="B666" t="inlineStr">
+        <is>
+          <t>DAIC</t>
+        </is>
+      </c>
+      <c r="C666" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D666" t="n">
+        <v>1.26</v>
+      </c>
+      <c r="E666" t="n">
+        <v>1.07</v>
+      </c>
+      <c r="F666" t="n">
+        <v>1.64</v>
+      </c>
+      <c r="G666" t="n">
+        <v>263</v>
+      </c>
+    </row>
+    <row r="667">
+      <c r="A667" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="B667" t="inlineStr">
+        <is>
+          <t>LUCY</t>
+        </is>
+      </c>
+      <c r="C667" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D667" t="n">
+        <v>1.02</v>
+      </c>
+      <c r="E667" t="n">
+        <v>0.88</v>
+      </c>
+      <c r="F667" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="G667" t="n">
+        <v>353</v>
+      </c>
+    </row>
+    <row r="668">
+      <c r="A668" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="B668" t="inlineStr">
+        <is>
+          <t>NSSC</t>
+        </is>
+      </c>
+      <c r="C668" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D668" t="n">
+        <v>51.5</v>
+      </c>
+      <c r="E668" t="n">
+        <v>36.38</v>
+      </c>
+      <c r="F668" t="n">
+        <v>81.73999999999999</v>
+      </c>
+      <c r="G668" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="669">
+      <c r="A669" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="B669" t="inlineStr">
+        <is>
+          <t>OLOX</t>
+        </is>
+      </c>
+      <c r="C669" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D669" t="n">
+        <v>2.42</v>
+      </c>
+      <c r="E669" t="n">
+        <v>1.98</v>
+      </c>
+      <c r="F669" t="n">
+        <v>3.3</v>
+      </c>
+      <c r="G669" t="n">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="670">
+      <c r="A670" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="B670" t="inlineStr">
+        <is>
+          <t>PUSA</t>
+        </is>
+      </c>
+      <c r="C670" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D670" t="n">
+        <v>4.02</v>
+      </c>
+      <c r="E670" t="n">
+        <v>3.75</v>
+      </c>
+      <c r="F670" t="n">
+        <v>4.56</v>
+      </c>
+      <c r="G670" t="n">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="671">
+      <c r="A671" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="B671" t="inlineStr">
+        <is>
+          <t>SDOT</t>
+        </is>
+      </c>
+      <c r="C671" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D671" t="n">
+        <v>24.33</v>
+      </c>
+      <c r="E671" t="n">
+        <v>21.26</v>
+      </c>
+      <c r="F671" t="n">
+        <v>30.47</v>
+      </c>
+      <c r="G671" t="n">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="672">
+      <c r="A672" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="B672" t="inlineStr">
+        <is>
+          <t>XPON</t>
+        </is>
+      </c>
+      <c r="C672" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D672" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="E672" t="n">
+        <v>6.02</v>
+      </c>
+      <c r="F672" t="n">
+        <v>14.66</v>
+      </c>
+      <c r="G672" t="n">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="673">
+      <c r="A673" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="B673" t="inlineStr">
+        <is>
+          <t>BIVI</t>
+        </is>
+      </c>
+      <c r="C673" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="674">
+      <c r="A674" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="B674" t="inlineStr">
+        <is>
+          <t>HOWL</t>
+        </is>
+      </c>
+      <c r="C674" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="675">
+      <c r="A675" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="B675" t="inlineStr">
+        <is>
+          <t>JUNS</t>
+        </is>
+      </c>
+      <c r="C675" t="inlineStr">
         <is>
           <t>Dropped</t>
         </is>
@@ -27008,7 +28082,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G19"/>
+  <dimension ref="A1:G20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -27462,6 +28536,35 @@
         </is>
       </c>
     </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>DAIC</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>1.07</v>
+      </c>
+      <c r="E20" t="n">
+        <v>3.13</v>
+      </c>
+      <c r="F20" t="n">
+        <v>-3.05</v>
+      </c>
+      <c r="G20" t="n">
+        <v>24</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily screener update: 2026-08-25
</commit_message>
<xml_diff>
--- a/screener_history.xlsx
+++ b/screener_history.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G523"/>
+  <dimension ref="A1:G544"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -12516,6 +12516,447 @@
         </is>
       </c>
       <c r="C523" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="524">
+      <c r="A524" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="B524" t="inlineStr">
+        <is>
+          <t>ALOY</t>
+        </is>
+      </c>
+      <c r="C524" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D524" t="n">
+        <v>15.35</v>
+      </c>
+      <c r="E524" t="n">
+        <v>10.93</v>
+      </c>
+      <c r="F524" t="n">
+        <v>24.19</v>
+      </c>
+      <c r="G524" t="n">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="525">
+      <c r="A525" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="B525" t="inlineStr">
+        <is>
+          <t>AMIX</t>
+        </is>
+      </c>
+      <c r="C525" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D525" t="n">
+        <v>9.99</v>
+      </c>
+      <c r="E525" t="n">
+        <v>4.97</v>
+      </c>
+      <c r="F525" t="n">
+        <v>20.03</v>
+      </c>
+      <c r="G525" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="526">
+      <c r="A526" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="B526" t="inlineStr">
+        <is>
+          <t>CJMB</t>
+        </is>
+      </c>
+      <c r="C526" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D526" t="n">
+        <v>3.24</v>
+      </c>
+      <c r="E526" t="n">
+        <v>1.83</v>
+      </c>
+      <c r="F526" t="n">
+        <v>6.06</v>
+      </c>
+      <c r="G526" t="n">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="527">
+      <c r="A527" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="B527" t="inlineStr">
+        <is>
+          <t>DELL</t>
+        </is>
+      </c>
+      <c r="C527" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D527" t="n">
+        <v>514</v>
+      </c>
+      <c r="E527" t="n">
+        <v>424</v>
+      </c>
+      <c r="F527" t="n">
+        <v>694</v>
+      </c>
+      <c r="G527" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="528">
+      <c r="A528" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="B528" t="inlineStr">
+        <is>
+          <t>HPE</t>
+        </is>
+      </c>
+      <c r="C528" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D528" t="n">
+        <v>63.44</v>
+      </c>
+      <c r="E528" t="n">
+        <v>51.3</v>
+      </c>
+      <c r="F528" t="n">
+        <v>87.72</v>
+      </c>
+      <c r="G528" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="529">
+      <c r="A529" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="B529" t="inlineStr">
+        <is>
+          <t>LCUT</t>
+        </is>
+      </c>
+      <c r="C529" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D529" t="n">
+        <v>10.17</v>
+      </c>
+      <c r="E529" t="n">
+        <v>8.800000000000001</v>
+      </c>
+      <c r="F529" t="n">
+        <v>12.91</v>
+      </c>
+      <c r="G529" t="n">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="530">
+      <c r="A530" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="B530" t="inlineStr">
+        <is>
+          <t>QNCX</t>
+        </is>
+      </c>
+      <c r="C530" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D530" t="n">
+        <v>35.41</v>
+      </c>
+      <c r="E530" t="n">
+        <v>30.04</v>
+      </c>
+      <c r="F530" t="n">
+        <v>46.15</v>
+      </c>
+      <c r="G530" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="531">
+      <c r="A531" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="B531" t="inlineStr">
+        <is>
+          <t>ALOT</t>
+        </is>
+      </c>
+      <c r="C531" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="532">
+      <c r="A532" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="B532" t="inlineStr">
+        <is>
+          <t>AZTA</t>
+        </is>
+      </c>
+      <c r="C532" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="533">
+      <c r="A533" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="B533" t="inlineStr">
+        <is>
+          <t>BNBX</t>
+        </is>
+      </c>
+      <c r="C533" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="534">
+      <c r="A534" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="B534" t="inlineStr">
+        <is>
+          <t>BWMN</t>
+        </is>
+      </c>
+      <c r="C534" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="535">
+      <c r="A535" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="B535" t="inlineStr">
+        <is>
+          <t>CIIT</t>
+        </is>
+      </c>
+      <c r="C535" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="536">
+      <c r="A536" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="B536" t="inlineStr">
+        <is>
+          <t>FWRD</t>
+        </is>
+      </c>
+      <c r="C536" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="537">
+      <c r="A537" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="B537" t="inlineStr">
+        <is>
+          <t>LUNG</t>
+        </is>
+      </c>
+      <c r="C537" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="538">
+      <c r="A538" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="B538" t="inlineStr">
+        <is>
+          <t>LVWR</t>
+        </is>
+      </c>
+      <c r="C538" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="539">
+      <c r="A539" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="B539" t="inlineStr">
+        <is>
+          <t>MBX</t>
+        </is>
+      </c>
+      <c r="C539" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="540">
+      <c r="A540" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="B540" t="inlineStr">
+        <is>
+          <t>OPAD</t>
+        </is>
+      </c>
+      <c r="C540" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="541">
+      <c r="A541" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="B541" t="inlineStr">
+        <is>
+          <t>PUBM</t>
+        </is>
+      </c>
+      <c r="C541" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="542">
+      <c r="A542" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="B542" t="inlineStr">
+        <is>
+          <t>REPL</t>
+        </is>
+      </c>
+      <c r="C542" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="543">
+      <c r="A543" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="B543" t="inlineStr">
+        <is>
+          <t>SGRP</t>
+        </is>
+      </c>
+      <c r="C543" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="544">
+      <c r="A544" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="B544" t="inlineStr">
+        <is>
+          <t>SMXT</t>
+        </is>
+      </c>
+      <c r="C544" t="inlineStr">
         <is>
           <t>Dropped</t>
         </is>
@@ -12532,7 +12973,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G675"/>
+  <dimension ref="A1:G687"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -28066,6 +28507,246 @@
         </is>
       </c>
       <c r="C675" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="676">
+      <c r="A676" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="B676" t="inlineStr">
+        <is>
+          <t>AMIX</t>
+        </is>
+      </c>
+      <c r="C676" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D676" t="n">
+        <v>8.300000000000001</v>
+      </c>
+      <c r="E676" t="n">
+        <v>5.37</v>
+      </c>
+      <c r="F676" t="n">
+        <v>14.16</v>
+      </c>
+      <c r="G676" t="n">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="677">
+      <c r="A677" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="B677" t="inlineStr">
+        <is>
+          <t>MAIR</t>
+        </is>
+      </c>
+      <c r="C677" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D677" t="n">
+        <v>29.44</v>
+      </c>
+      <c r="E677" t="n">
+        <v>27.11</v>
+      </c>
+      <c r="F677" t="n">
+        <v>34.1</v>
+      </c>
+      <c r="G677" t="n">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="678">
+      <c r="A678" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="B678" t="inlineStr">
+        <is>
+          <t>TENX</t>
+        </is>
+      </c>
+      <c r="C678" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D678" t="n">
+        <v>2.21</v>
+      </c>
+      <c r="E678" t="n">
+        <v>1.85</v>
+      </c>
+      <c r="F678" t="n">
+        <v>2.93</v>
+      </c>
+      <c r="G678" t="n">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="679">
+      <c r="A679" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="B679" t="inlineStr">
+        <is>
+          <t>APRE</t>
+        </is>
+      </c>
+      <c r="C679" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="680">
+      <c r="A680" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="B680" t="inlineStr">
+        <is>
+          <t>CAPR</t>
+        </is>
+      </c>
+      <c r="C680" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="681">
+      <c r="A681" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="B681" t="inlineStr">
+        <is>
+          <t>CYPH</t>
+        </is>
+      </c>
+      <c r="C681" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="682">
+      <c r="A682" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="B682" t="inlineStr">
+        <is>
+          <t>LUCY</t>
+        </is>
+      </c>
+      <c r="C682" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="683">
+      <c r="A683" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="B683" t="inlineStr">
+        <is>
+          <t>NSSC</t>
+        </is>
+      </c>
+      <c r="C683" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="684">
+      <c r="A684" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="B684" t="inlineStr">
+        <is>
+          <t>OLOX</t>
+        </is>
+      </c>
+      <c r="C684" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="685">
+      <c r="A685" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="B685" t="inlineStr">
+        <is>
+          <t>PUSA</t>
+        </is>
+      </c>
+      <c r="C685" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="686">
+      <c r="A686" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="B686" t="inlineStr">
+        <is>
+          <t>SDOT</t>
+        </is>
+      </c>
+      <c r="C686" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="687">
+      <c r="A687" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="B687" t="inlineStr">
+        <is>
+          <t>XPON</t>
+        </is>
+      </c>
+      <c r="C687" t="inlineStr">
         <is>
           <t>Dropped</t>
         </is>

</xml_diff>

<commit_message>
Daily screener update: 2026-08-27
</commit_message>
<xml_diff>
--- a/screener_history.xlsx
+++ b/screener_history.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G544"/>
+  <dimension ref="A1:G559"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -12957,6 +12957,357 @@
         </is>
       </c>
       <c r="C544" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="545">
+      <c r="A545" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="B545" t="inlineStr">
+        <is>
+          <t>ABSI</t>
+        </is>
+      </c>
+      <c r="C545" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D545" t="n">
+        <v>10.03</v>
+      </c>
+      <c r="E545" t="n">
+        <v>8.550000000000001</v>
+      </c>
+      <c r="F545" t="n">
+        <v>12.99</v>
+      </c>
+      <c r="G545" t="n">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="546">
+      <c r="A546" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="B546" t="inlineStr">
+        <is>
+          <t>BOXL</t>
+        </is>
+      </c>
+      <c r="C546" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D546" t="n">
+        <v>9.5</v>
+      </c>
+      <c r="E546" t="n">
+        <v>4.97</v>
+      </c>
+      <c r="F546" t="n">
+        <v>18.55</v>
+      </c>
+      <c r="G546" t="n">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="547">
+      <c r="A547" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="B547" t="inlineStr">
+        <is>
+          <t>CISS</t>
+        </is>
+      </c>
+      <c r="C547" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D547" t="n">
+        <v>4.9</v>
+      </c>
+      <c r="E547" t="n">
+        <v>2.24</v>
+      </c>
+      <c r="F547" t="n">
+        <v>10.22</v>
+      </c>
+      <c r="G547" t="n">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="548">
+      <c r="A548" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="B548" t="inlineStr">
+        <is>
+          <t>FWRD</t>
+        </is>
+      </c>
+      <c r="C548" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D548" t="n">
+        <v>20.57</v>
+      </c>
+      <c r="E548" t="n">
+        <v>17.15</v>
+      </c>
+      <c r="F548" t="n">
+        <v>27.41</v>
+      </c>
+      <c r="G548" t="n">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="549">
+      <c r="A549" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="B549" t="inlineStr">
+        <is>
+          <t>MBX</t>
+        </is>
+      </c>
+      <c r="C549" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D549" t="n">
+        <v>69.94</v>
+      </c>
+      <c r="E549" t="n">
+        <v>64</v>
+      </c>
+      <c r="F549" t="n">
+        <v>81.81999999999999</v>
+      </c>
+      <c r="G549" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="550">
+      <c r="A550" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="B550" t="inlineStr">
+        <is>
+          <t>PAYS</t>
+        </is>
+      </c>
+      <c r="C550" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D550" t="n">
+        <v>14.43</v>
+      </c>
+      <c r="E550" t="n">
+        <v>12.59</v>
+      </c>
+      <c r="F550" t="n">
+        <v>18.11</v>
+      </c>
+      <c r="G550" t="n">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="551">
+      <c r="A551" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="B551" t="inlineStr">
+        <is>
+          <t>RLYB</t>
+        </is>
+      </c>
+      <c r="C551" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D551" t="n">
+        <v>17.35</v>
+      </c>
+      <c r="E551" t="n">
+        <v>16.51</v>
+      </c>
+      <c r="F551" t="n">
+        <v>19.03</v>
+      </c>
+      <c r="G551" t="n">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="552">
+      <c r="A552" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="B552" t="inlineStr">
+        <is>
+          <t>SMXT</t>
+        </is>
+      </c>
+      <c r="C552" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D552" t="n">
+        <v>4.9</v>
+      </c>
+      <c r="E552" t="n">
+        <v>2.65</v>
+      </c>
+      <c r="F552" t="n">
+        <v>9.4</v>
+      </c>
+      <c r="G552" t="n">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="553">
+      <c r="A553" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="B553" t="inlineStr">
+        <is>
+          <t>ALOY</t>
+        </is>
+      </c>
+      <c r="C553" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="554">
+      <c r="A554" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="B554" t="inlineStr">
+        <is>
+          <t>AMIX</t>
+        </is>
+      </c>
+      <c r="C554" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="555">
+      <c r="A555" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="B555" t="inlineStr">
+        <is>
+          <t>BFLY</t>
+        </is>
+      </c>
+      <c r="C555" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="556">
+      <c r="A556" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="B556" t="inlineStr">
+        <is>
+          <t>DELL</t>
+        </is>
+      </c>
+      <c r="C556" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="557">
+      <c r="A557" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="B557" t="inlineStr">
+        <is>
+          <t>HPE</t>
+        </is>
+      </c>
+      <c r="C557" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="558">
+      <c r="A558" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="B558" t="inlineStr">
+        <is>
+          <t>LCUT</t>
+        </is>
+      </c>
+      <c r="C558" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="559">
+      <c r="A559" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="B559" t="inlineStr">
+        <is>
+          <t>LPSN</t>
+        </is>
+      </c>
+      <c r="C559" t="inlineStr">
         <is>
           <t>Dropped</t>
         </is>
@@ -12973,7 +13324,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G687"/>
+  <dimension ref="A1:G699"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -28747,6 +29098,318 @@
         </is>
       </c>
       <c r="C687" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="688">
+      <c r="A688" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="B688" t="inlineStr">
+        <is>
+          <t>ANF</t>
+        </is>
+      </c>
+      <c r="C688" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D688" t="n">
+        <v>141.98</v>
+      </c>
+      <c r="E688" t="n">
+        <v>130.24</v>
+      </c>
+      <c r="F688" t="n">
+        <v>165.47</v>
+      </c>
+      <c r="G688" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="689">
+      <c r="A689" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="B689" t="inlineStr">
+        <is>
+          <t>APRE</t>
+        </is>
+      </c>
+      <c r="C689" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D689" t="n">
+        <v>1.13</v>
+      </c>
+      <c r="E689" t="n">
+        <v>0.92</v>
+      </c>
+      <c r="F689" t="n">
+        <v>1.54</v>
+      </c>
+      <c r="G689" t="n">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="690">
+      <c r="A690" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="B690" t="inlineStr">
+        <is>
+          <t>MSS</t>
+        </is>
+      </c>
+      <c r="C690" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D690" t="n">
+        <v>2.24</v>
+      </c>
+      <c r="E690" t="n">
+        <v>1.57</v>
+      </c>
+      <c r="F690" t="n">
+        <v>3.58</v>
+      </c>
+      <c r="G690" t="n">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="691">
+      <c r="A691" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="B691" t="inlineStr">
+        <is>
+          <t>PLAB</t>
+        </is>
+      </c>
+      <c r="C691" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D691" t="n">
+        <v>37.91</v>
+      </c>
+      <c r="E691" t="n">
+        <v>29.86</v>
+      </c>
+      <c r="F691" t="n">
+        <v>54.01</v>
+      </c>
+      <c r="G691" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="692">
+      <c r="A692" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="B692" t="inlineStr">
+        <is>
+          <t>RDIB</t>
+        </is>
+      </c>
+      <c r="C692" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D692" t="n">
+        <v>13.38</v>
+      </c>
+      <c r="E692" t="n">
+        <v>12</v>
+      </c>
+      <c r="F692" t="n">
+        <v>16.14</v>
+      </c>
+      <c r="G692" t="n">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="693">
+      <c r="A693" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="B693" t="inlineStr">
+        <is>
+          <t>SMTK</t>
+        </is>
+      </c>
+      <c r="C693" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D693" t="n">
+        <v>4.47</v>
+      </c>
+      <c r="E693" t="n">
+        <v>3.83</v>
+      </c>
+      <c r="F693" t="n">
+        <v>5.77</v>
+      </c>
+      <c r="G693" t="n">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="694">
+      <c r="A694" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="B694" t="inlineStr">
+        <is>
+          <t>STRT</t>
+        </is>
+      </c>
+      <c r="C694" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D694" t="n">
+        <v>93</v>
+      </c>
+      <c r="E694" t="n">
+        <v>68.18000000000001</v>
+      </c>
+      <c r="F694" t="n">
+        <v>142.64</v>
+      </c>
+      <c r="G694" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="695">
+      <c r="A695" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="B695" t="inlineStr">
+        <is>
+          <t>TRUG</t>
+        </is>
+      </c>
+      <c r="C695" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D695" t="n">
+        <v>0.68</v>
+      </c>
+      <c r="E695" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="F695" t="n">
+        <v>0.84</v>
+      </c>
+      <c r="G695" t="n">
+        <v>627</v>
+      </c>
+    </row>
+    <row r="696">
+      <c r="A696" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="B696" t="inlineStr">
+        <is>
+          <t>XPON</t>
+        </is>
+      </c>
+      <c r="C696" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D696" t="n">
+        <v>6.58</v>
+      </c>
+      <c r="E696" t="n">
+        <v>6.3</v>
+      </c>
+      <c r="F696" t="n">
+        <v>7.15</v>
+      </c>
+      <c r="G696" t="n">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="697">
+      <c r="A697" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="B697" t="inlineStr">
+        <is>
+          <t>AMIX</t>
+        </is>
+      </c>
+      <c r="C697" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="698">
+      <c r="A698" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="B698" t="inlineStr">
+        <is>
+          <t>MAIR</t>
+        </is>
+      </c>
+      <c r="C698" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="699">
+      <c r="A699" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="B699" t="inlineStr">
+        <is>
+          <t>TENX</t>
+        </is>
+      </c>
+      <c r="C699" t="inlineStr">
         <is>
           <t>Dropped</t>
         </is>
@@ -28763,7 +29426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G20"/>
+  <dimension ref="A1:G21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -29246,6 +29909,35 @@
         <v>24</v>
       </c>
     </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>BRCC</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>8.31</v>
+      </c>
+      <c r="E21" t="n">
+        <v>9</v>
+      </c>
+      <c r="F21" t="n">
+        <v>6.93</v>
+      </c>
+      <c r="G21" t="n">
+        <v>72</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily screener update: 2026-08-28
</commit_message>
<xml_diff>
--- a/screener_history.xlsx
+++ b/screener_history.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G559"/>
+  <dimension ref="A1:G570"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -13308,6 +13308,265 @@
         </is>
       </c>
       <c r="C559" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="560">
+      <c r="A560" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="B560" t="inlineStr">
+        <is>
+          <t>ANTX</t>
+        </is>
+      </c>
+      <c r="C560" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D560" t="n">
+        <v>6.21</v>
+      </c>
+      <c r="E560" t="n">
+        <v>5.46</v>
+      </c>
+      <c r="F560" t="n">
+        <v>7.71</v>
+      </c>
+      <c r="G560" t="n">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="561">
+      <c r="A561" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="B561" t="inlineStr">
+        <is>
+          <t>APPS</t>
+        </is>
+      </c>
+      <c r="C561" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D561" t="n">
+        <v>12.9</v>
+      </c>
+      <c r="E561" t="n">
+        <v>10.43</v>
+      </c>
+      <c r="F561" t="n">
+        <v>17.84</v>
+      </c>
+      <c r="G561" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="562">
+      <c r="A562" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="B562" t="inlineStr">
+        <is>
+          <t>CYCN</t>
+        </is>
+      </c>
+      <c r="C562" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D562" t="n">
+        <v>4.47</v>
+      </c>
+      <c r="E562" t="n">
+        <v>3.73</v>
+      </c>
+      <c r="F562" t="n">
+        <v>5.94</v>
+      </c>
+      <c r="G562" t="n">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="563">
+      <c r="A563" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="B563" t="inlineStr">
+        <is>
+          <t>LCUT</t>
+        </is>
+      </c>
+      <c r="C563" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D563" t="n">
+        <v>10.17</v>
+      </c>
+      <c r="E563" t="n">
+        <v>8.800000000000001</v>
+      </c>
+      <c r="F563" t="n">
+        <v>12.91</v>
+      </c>
+      <c r="G563" t="n">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="564">
+      <c r="A564" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="B564" t="inlineStr">
+        <is>
+          <t>PEPG</t>
+        </is>
+      </c>
+      <c r="C564" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D564" t="n">
+        <v>3.57</v>
+      </c>
+      <c r="E564" t="n">
+        <v>2.85</v>
+      </c>
+      <c r="F564" t="n">
+        <v>5.01</v>
+      </c>
+      <c r="G564" t="n">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="565">
+      <c r="A565" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="B565" t="inlineStr">
+        <is>
+          <t>RRGB</t>
+        </is>
+      </c>
+      <c r="C565" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D565" t="n">
+        <v>10.71</v>
+      </c>
+      <c r="E565" t="n">
+        <v>9.19</v>
+      </c>
+      <c r="F565" t="n">
+        <v>13.75</v>
+      </c>
+      <c r="G565" t="n">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="566">
+      <c r="A566" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="B566" t="inlineStr">
+        <is>
+          <t>ABSI</t>
+        </is>
+      </c>
+      <c r="C566" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="567">
+      <c r="A567" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="B567" t="inlineStr">
+        <is>
+          <t>CISS</t>
+        </is>
+      </c>
+      <c r="C567" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="568">
+      <c r="A568" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="B568" t="inlineStr">
+        <is>
+          <t>FRD</t>
+        </is>
+      </c>
+      <c r="C568" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="569">
+      <c r="A569" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="B569" t="inlineStr">
+        <is>
+          <t>RLYB</t>
+        </is>
+      </c>
+      <c r="C569" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="570">
+      <c r="A570" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="B570" t="inlineStr">
+        <is>
+          <t>TTRX</t>
+        </is>
+      </c>
+      <c r="C570" t="inlineStr">
         <is>
           <t>Dropped</t>
         </is>
@@ -13324,7 +13583,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G699"/>
+  <dimension ref="A1:G720"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -29410,6 +29669,495 @@
         </is>
       </c>
       <c r="C699" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="700">
+      <c r="A700" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="B700" t="inlineStr">
+        <is>
+          <t>CELU</t>
+        </is>
+      </c>
+      <c r="C700" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D700" t="n">
+        <v>1.13</v>
+      </c>
+      <c r="E700" t="n">
+        <v>0.93</v>
+      </c>
+      <c r="F700" t="n">
+        <v>1.54</v>
+      </c>
+      <c r="G700" t="n">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="701">
+      <c r="A701" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="B701" t="inlineStr">
+        <is>
+          <t>CRM</t>
+        </is>
+      </c>
+      <c r="C701" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D701" t="n">
+        <v>235.8</v>
+      </c>
+      <c r="E701" t="n">
+        <v>230.05</v>
+      </c>
+      <c r="F701" t="n">
+        <v>247.29</v>
+      </c>
+      <c r="G701" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="702">
+      <c r="A702" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="B702" t="inlineStr">
+        <is>
+          <t>LTRX</t>
+        </is>
+      </c>
+      <c r="C702" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D702" t="n">
+        <v>7.07</v>
+      </c>
+      <c r="E702" t="n">
+        <v>5.8</v>
+      </c>
+      <c r="F702" t="n">
+        <v>9.609999999999999</v>
+      </c>
+      <c r="G702" t="n">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="703">
+      <c r="A703" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="B703" t="inlineStr">
+        <is>
+          <t>MERC</t>
+        </is>
+      </c>
+      <c r="C703" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D703" t="n">
+        <v>0.64</v>
+      </c>
+      <c r="E703" t="n">
+        <v>0.38</v>
+      </c>
+      <c r="F703" t="n">
+        <v>1.18</v>
+      </c>
+      <c r="G703" t="n">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="704">
+      <c r="A704" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="B704" t="inlineStr">
+        <is>
+          <t>NCPL</t>
+        </is>
+      </c>
+      <c r="C704" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D704" t="n">
+        <v>0.74</v>
+      </c>
+      <c r="E704" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="F704" t="n">
+        <v>1.22</v>
+      </c>
+      <c r="G704" t="n">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="705">
+      <c r="A705" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="B705" t="inlineStr">
+        <is>
+          <t>OBAI</t>
+        </is>
+      </c>
+      <c r="C705" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D705" t="n">
+        <v>0.37</v>
+      </c>
+      <c r="E705" t="n">
+        <v>0.32</v>
+      </c>
+      <c r="F705" t="n">
+        <v>0.47</v>
+      </c>
+      <c r="G705" t="n">
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="706">
+      <c r="A706" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="B706" t="inlineStr">
+        <is>
+          <t>OKTA</t>
+        </is>
+      </c>
+      <c r="C706" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D706" t="n">
+        <v>167.59</v>
+      </c>
+      <c r="E706" t="n">
+        <v>156.5</v>
+      </c>
+      <c r="F706" t="n">
+        <v>189.77</v>
+      </c>
+      <c r="G706" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="707">
+      <c r="A707" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="B707" t="inlineStr">
+        <is>
+          <t>PPCB</t>
+        </is>
+      </c>
+      <c r="C707" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D707" t="n">
+        <v>4.13</v>
+      </c>
+      <c r="E707" t="n">
+        <v>1.98</v>
+      </c>
+      <c r="F707" t="n">
+        <v>8.43</v>
+      </c>
+      <c r="G707" t="n">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="708">
+      <c r="A708" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="B708" t="inlineStr">
+        <is>
+          <t>VEEV</t>
+        </is>
+      </c>
+      <c r="C708" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D708" t="n">
+        <v>282.51</v>
+      </c>
+      <c r="E708" t="n">
+        <v>274.81</v>
+      </c>
+      <c r="F708" t="n">
+        <v>297.91</v>
+      </c>
+      <c r="G708" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="709">
+      <c r="A709" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="B709" t="inlineStr">
+        <is>
+          <t>VNCE</t>
+        </is>
+      </c>
+      <c r="C709" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D709" t="n">
+        <v>8.08</v>
+      </c>
+      <c r="E709" t="n">
+        <v>7.3</v>
+      </c>
+      <c r="F709" t="n">
+        <v>9.640000000000001</v>
+      </c>
+      <c r="G709" t="n">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="710">
+      <c r="A710" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="B710" t="inlineStr">
+        <is>
+          <t>WKSP</t>
+        </is>
+      </c>
+      <c r="C710" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D710" t="n">
+        <v>0.62</v>
+      </c>
+      <c r="E710" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="F710" t="n">
+        <v>0.66</v>
+      </c>
+      <c r="G710" t="n">
+        <v>2645</v>
+      </c>
+    </row>
+    <row r="711">
+      <c r="A711" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="B711" t="inlineStr">
+        <is>
+          <t>ANF</t>
+        </is>
+      </c>
+      <c r="C711" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="712">
+      <c r="A712" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="B712" t="inlineStr">
+        <is>
+          <t>APRE</t>
+        </is>
+      </c>
+      <c r="C712" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="713">
+      <c r="A713" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="B713" t="inlineStr">
+        <is>
+          <t>DAIC</t>
+        </is>
+      </c>
+      <c r="C713" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="714">
+      <c r="A714" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="B714" t="inlineStr">
+        <is>
+          <t>MSS</t>
+        </is>
+      </c>
+      <c r="C714" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="715">
+      <c r="A715" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="B715" t="inlineStr">
+        <is>
+          <t>PLAB</t>
+        </is>
+      </c>
+      <c r="C715" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="716">
+      <c r="A716" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="B716" t="inlineStr">
+        <is>
+          <t>RDIB</t>
+        </is>
+      </c>
+      <c r="C716" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="717">
+      <c r="A717" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="B717" t="inlineStr">
+        <is>
+          <t>SMTK</t>
+        </is>
+      </c>
+      <c r="C717" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="718">
+      <c r="A718" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="B718" t="inlineStr">
+        <is>
+          <t>STRT</t>
+        </is>
+      </c>
+      <c r="C718" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="719">
+      <c r="A719" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="B719" t="inlineStr">
+        <is>
+          <t>TRUG</t>
+        </is>
+      </c>
+      <c r="C719" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="720">
+      <c r="A720" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="B720" t="inlineStr">
+        <is>
+          <t>XPON</t>
+        </is>
+      </c>
+      <c r="C720" t="inlineStr">
         <is>
           <t>Dropped</t>
         </is>
@@ -29426,7 +30174,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G21"/>
+  <dimension ref="A1:G23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -29938,6 +30686,40 @@
         <v>72</v>
       </c>
     </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>BRCC</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>DAIC</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily screener update: 2026-08-29
</commit_message>
<xml_diff>
--- a/screener_history.xlsx
+++ b/screener_history.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G570"/>
+  <dimension ref="A1:G588"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -13567,6 +13567,432 @@
         </is>
       </c>
       <c r="C570" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="571">
+      <c r="A571" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
+        </is>
+      </c>
+      <c r="B571" t="inlineStr">
+        <is>
+          <t>AIFA</t>
+        </is>
+      </c>
+      <c r="C571" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D571" t="n">
+        <v>3.4</v>
+      </c>
+      <c r="E571" t="n">
+        <v>2.72</v>
+      </c>
+      <c r="F571" t="n">
+        <v>4.76</v>
+      </c>
+      <c r="G571" t="n">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="572">
+      <c r="A572" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
+        </is>
+      </c>
+      <c r="B572" t="inlineStr">
+        <is>
+          <t>ALOT</t>
+        </is>
+      </c>
+      <c r="C572" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D572" t="n">
+        <v>28.6</v>
+      </c>
+      <c r="E572" t="n">
+        <v>28.47</v>
+      </c>
+      <c r="F572" t="n">
+        <v>28.86</v>
+      </c>
+      <c r="G572" t="n">
+        <v>384</v>
+      </c>
+    </row>
+    <row r="573">
+      <c r="A573" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
+        </is>
+      </c>
+      <c r="B573" t="inlineStr">
+        <is>
+          <t>BOLD</t>
+        </is>
+      </c>
+      <c r="C573" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D573" t="n">
+        <v>3.16</v>
+      </c>
+      <c r="E573" t="n">
+        <v>2.71</v>
+      </c>
+      <c r="F573" t="n">
+        <v>4.07</v>
+      </c>
+      <c r="G573" t="n">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="574">
+      <c r="A574" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
+        </is>
+      </c>
+      <c r="B574" t="inlineStr">
+        <is>
+          <t>DUKR</t>
+        </is>
+      </c>
+      <c r="C574" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D574" t="n">
+        <v>5.87</v>
+      </c>
+      <c r="E574" t="n">
+        <v>5.22</v>
+      </c>
+      <c r="F574" t="n">
+        <v>7.16</v>
+      </c>
+      <c r="G574" t="n">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="575">
+      <c r="A575" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
+        </is>
+      </c>
+      <c r="B575" t="inlineStr">
+        <is>
+          <t>ETON</t>
+        </is>
+      </c>
+      <c r="C575" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D575" t="n">
+        <v>66.37</v>
+      </c>
+      <c r="E575" t="n">
+        <v>56.65</v>
+      </c>
+      <c r="F575" t="n">
+        <v>85.81</v>
+      </c>
+      <c r="G575" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="576">
+      <c r="A576" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
+        </is>
+      </c>
+      <c r="B576" t="inlineStr">
+        <is>
+          <t>FATN</t>
+        </is>
+      </c>
+      <c r="C576" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D576" t="n">
+        <v>6.44</v>
+      </c>
+      <c r="E576" t="n">
+        <v>5.8</v>
+      </c>
+      <c r="F576" t="n">
+        <v>7.72</v>
+      </c>
+      <c r="G576" t="n">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="577">
+      <c r="A577" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
+        </is>
+      </c>
+      <c r="B577" t="inlineStr">
+        <is>
+          <t>FRD</t>
+        </is>
+      </c>
+      <c r="C577" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D577" t="n">
+        <v>48.77</v>
+      </c>
+      <c r="E577" t="n">
+        <v>41.16</v>
+      </c>
+      <c r="F577" t="n">
+        <v>63.99</v>
+      </c>
+      <c r="G577" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="578">
+      <c r="A578" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
+        </is>
+      </c>
+      <c r="B578" t="inlineStr">
+        <is>
+          <t>OPAD</t>
+        </is>
+      </c>
+      <c r="C578" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D578" t="n">
+        <v>4.62</v>
+      </c>
+      <c r="E578" t="n">
+        <v>4.01</v>
+      </c>
+      <c r="F578" t="n">
+        <v>5.83</v>
+      </c>
+      <c r="G578" t="n">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="579">
+      <c r="A579" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
+        </is>
+      </c>
+      <c r="B579" t="inlineStr">
+        <is>
+          <t>SLS</t>
+        </is>
+      </c>
+      <c r="C579" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D579" t="n">
+        <v>15.67</v>
+      </c>
+      <c r="E579" t="n">
+        <v>12.39</v>
+      </c>
+      <c r="F579" t="n">
+        <v>22.23</v>
+      </c>
+      <c r="G579" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="580">
+      <c r="A580" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
+        </is>
+      </c>
+      <c r="B580" t="inlineStr">
+        <is>
+          <t>TKNO</t>
+        </is>
+      </c>
+      <c r="C580" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D580" t="n">
+        <v>7.68</v>
+      </c>
+      <c r="E580" t="n">
+        <v>6.65</v>
+      </c>
+      <c r="F580" t="n">
+        <v>9.74</v>
+      </c>
+      <c r="G580" t="n">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="581">
+      <c r="A581" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
+        </is>
+      </c>
+      <c r="B581" t="inlineStr">
+        <is>
+          <t>ANTX</t>
+        </is>
+      </c>
+      <c r="C581" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="582">
+      <c r="A582" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
+        </is>
+      </c>
+      <c r="B582" t="inlineStr">
+        <is>
+          <t>APPS</t>
+        </is>
+      </c>
+      <c r="C582" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="583">
+      <c r="A583" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
+        </is>
+      </c>
+      <c r="B583" t="inlineStr">
+        <is>
+          <t>CXAI</t>
+        </is>
+      </c>
+      <c r="C583" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="584">
+      <c r="A584" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
+        </is>
+      </c>
+      <c r="B584" t="inlineStr">
+        <is>
+          <t>CYCN</t>
+        </is>
+      </c>
+      <c r="C584" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="585">
+      <c r="A585" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
+        </is>
+      </c>
+      <c r="B585" t="inlineStr">
+        <is>
+          <t>FWRD</t>
+        </is>
+      </c>
+      <c r="C585" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="586">
+      <c r="A586" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
+        </is>
+      </c>
+      <c r="B586" t="inlineStr">
+        <is>
+          <t>JUNS</t>
+        </is>
+      </c>
+      <c r="C586" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="587">
+      <c r="A587" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
+        </is>
+      </c>
+      <c r="B587" t="inlineStr">
+        <is>
+          <t>MBX</t>
+        </is>
+      </c>
+      <c r="C587" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="588">
+      <c r="A588" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
+        </is>
+      </c>
+      <c r="B588" t="inlineStr">
+        <is>
+          <t>QNCX</t>
+        </is>
+      </c>
+      <c r="C588" t="inlineStr">
         <is>
           <t>Dropped</t>
         </is>
@@ -13583,7 +14009,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G720"/>
+  <dimension ref="A1:G738"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -30158,6 +30584,396 @@
         </is>
       </c>
       <c r="C720" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="721">
+      <c r="A721" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
+        </is>
+      </c>
+      <c r="B721" t="inlineStr">
+        <is>
+          <t>AEMD</t>
+        </is>
+      </c>
+      <c r="C721" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D721" t="n">
+        <v>3.07</v>
+      </c>
+      <c r="E721" t="n">
+        <v>2.44</v>
+      </c>
+      <c r="F721" t="n">
+        <v>4.33</v>
+      </c>
+      <c r="G721" t="n">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="722">
+      <c r="A722" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
+        </is>
+      </c>
+      <c r="B722" t="inlineStr">
+        <is>
+          <t>AFRM</t>
+        </is>
+      </c>
+      <c r="C722" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D722" t="n">
+        <v>90.44</v>
+      </c>
+      <c r="E722" t="n">
+        <v>77.59</v>
+      </c>
+      <c r="F722" t="n">
+        <v>116.14</v>
+      </c>
+      <c r="G722" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="723">
+      <c r="A723" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
+        </is>
+      </c>
+      <c r="B723" t="inlineStr">
+        <is>
+          <t>CYAB</t>
+        </is>
+      </c>
+      <c r="C723" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D723" t="n">
+        <v>0.38</v>
+      </c>
+      <c r="E723" t="n">
+        <v>0.32</v>
+      </c>
+      <c r="F723" t="n">
+        <v>0.51</v>
+      </c>
+      <c r="G723" t="n">
+        <v>825</v>
+      </c>
+    </row>
+    <row r="724">
+      <c r="A724" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
+        </is>
+      </c>
+      <c r="B724" t="inlineStr">
+        <is>
+          <t>FNGR</t>
+        </is>
+      </c>
+      <c r="C724" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D724" t="n">
+        <v>0.37</v>
+      </c>
+      <c r="E724" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="F724" t="n">
+        <v>0.51</v>
+      </c>
+      <c r="G724" t="n">
+        <v>724</v>
+      </c>
+    </row>
+    <row r="725">
+      <c r="A725" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
+        </is>
+      </c>
+      <c r="B725" t="inlineStr">
+        <is>
+          <t>GAP</t>
+        </is>
+      </c>
+      <c r="C725" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D725" t="n">
+        <v>25.8</v>
+      </c>
+      <c r="E725" t="n">
+        <v>23.33</v>
+      </c>
+      <c r="F725" t="n">
+        <v>30.74</v>
+      </c>
+      <c r="G725" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="726">
+      <c r="A726" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
+        </is>
+      </c>
+      <c r="B726" t="inlineStr">
+        <is>
+          <t>SOLS</t>
+        </is>
+      </c>
+      <c r="C726" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D726" t="n">
+        <v>66.90000000000001</v>
+      </c>
+      <c r="E726" t="n">
+        <v>63.13</v>
+      </c>
+      <c r="F726" t="n">
+        <v>74.44</v>
+      </c>
+      <c r="G726" t="n">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="727">
+      <c r="A727" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
+        </is>
+      </c>
+      <c r="B727" t="inlineStr">
+        <is>
+          <t>WHLR</t>
+        </is>
+      </c>
+      <c r="C727" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D727" t="n">
+        <v>1.55</v>
+      </c>
+      <c r="E727" t="n">
+        <v>0.9399999999999999</v>
+      </c>
+      <c r="F727" t="n">
+        <v>2.77</v>
+      </c>
+      <c r="G727" t="n">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="728">
+      <c r="A728" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
+        </is>
+      </c>
+      <c r="B728" t="inlineStr">
+        <is>
+          <t>CELU</t>
+        </is>
+      </c>
+      <c r="C728" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="729">
+      <c r="A729" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
+        </is>
+      </c>
+      <c r="B729" t="inlineStr">
+        <is>
+          <t>CRM</t>
+        </is>
+      </c>
+      <c r="C729" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="730">
+      <c r="A730" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
+        </is>
+      </c>
+      <c r="B730" t="inlineStr">
+        <is>
+          <t>LTRX</t>
+        </is>
+      </c>
+      <c r="C730" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="731">
+      <c r="A731" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
+        </is>
+      </c>
+      <c r="B731" t="inlineStr">
+        <is>
+          <t>MERC</t>
+        </is>
+      </c>
+      <c r="C731" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="732">
+      <c r="A732" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
+        </is>
+      </c>
+      <c r="B732" t="inlineStr">
+        <is>
+          <t>NCPL</t>
+        </is>
+      </c>
+      <c r="C732" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="733">
+      <c r="A733" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
+        </is>
+      </c>
+      <c r="B733" t="inlineStr">
+        <is>
+          <t>OBAI</t>
+        </is>
+      </c>
+      <c r="C733" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="734">
+      <c r="A734" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
+        </is>
+      </c>
+      <c r="B734" t="inlineStr">
+        <is>
+          <t>OKTA</t>
+        </is>
+      </c>
+      <c r="C734" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="735">
+      <c r="A735" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
+        </is>
+      </c>
+      <c r="B735" t="inlineStr">
+        <is>
+          <t>PPCB</t>
+        </is>
+      </c>
+      <c r="C735" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="736">
+      <c r="A736" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
+        </is>
+      </c>
+      <c r="B736" t="inlineStr">
+        <is>
+          <t>VEEV</t>
+        </is>
+      </c>
+      <c r="C736" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="737">
+      <c r="A737" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
+        </is>
+      </c>
+      <c r="B737" t="inlineStr">
+        <is>
+          <t>VNCE</t>
+        </is>
+      </c>
+      <c r="C737" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="738">
+      <c r="A738" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
+        </is>
+      </c>
+      <c r="B738" t="inlineStr">
+        <is>
+          <t>WKSP</t>
+        </is>
+      </c>
+      <c r="C738" t="inlineStr">
         <is>
           <t>Dropped</t>
         </is>

</xml_diff>

<commit_message>
Daily screener update: 2026-09-01
</commit_message>
<xml_diff>
--- a/screener_history.xlsx
+++ b/screener_history.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G588"/>
+  <dimension ref="A1:G604"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -13993,6 +13993,374 @@
         </is>
       </c>
       <c r="C588" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="589">
+      <c r="A589" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="B589" t="inlineStr">
+        <is>
+          <t>AGEN</t>
+        </is>
+      </c>
+      <c r="C589" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D589" t="n">
+        <v>8.73</v>
+      </c>
+      <c r="E589" t="n">
+        <v>7.08</v>
+      </c>
+      <c r="F589" t="n">
+        <v>12.03</v>
+      </c>
+      <c r="G589" t="n">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="590">
+      <c r="A590" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="B590" t="inlineStr">
+        <is>
+          <t>AGPU</t>
+        </is>
+      </c>
+      <c r="C590" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D590" t="n">
+        <v>11.73</v>
+      </c>
+      <c r="E590" t="n">
+        <v>9.289999999999999</v>
+      </c>
+      <c r="F590" t="n">
+        <v>16.61</v>
+      </c>
+      <c r="G590" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="591">
+      <c r="A591" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="B591" t="inlineStr">
+        <is>
+          <t>BWMN</t>
+        </is>
+      </c>
+      <c r="C591" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D591" t="n">
+        <v>42.64</v>
+      </c>
+      <c r="E591" t="n">
+        <v>42.31</v>
+      </c>
+      <c r="F591" t="n">
+        <v>43.3</v>
+      </c>
+      <c r="G591" t="n">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="592">
+      <c r="A592" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="B592" t="inlineStr">
+        <is>
+          <t>FTH</t>
+        </is>
+      </c>
+      <c r="C592" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D592" t="n">
+        <v>36</v>
+      </c>
+      <c r="E592" t="n">
+        <v>30.3</v>
+      </c>
+      <c r="F592" t="n">
+        <v>47.4</v>
+      </c>
+      <c r="G592" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="593">
+      <c r="A593" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="B593" t="inlineStr">
+        <is>
+          <t>HELP</t>
+        </is>
+      </c>
+      <c r="C593" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D593" t="n">
+        <v>14.35</v>
+      </c>
+      <c r="E593" t="n">
+        <v>11.17</v>
+      </c>
+      <c r="F593" t="n">
+        <v>20.71</v>
+      </c>
+      <c r="G593" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="594">
+      <c r="A594" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="B594" t="inlineStr">
+        <is>
+          <t>LEXX</t>
+        </is>
+      </c>
+      <c r="C594" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D594" t="n">
+        <v>12.89</v>
+      </c>
+      <c r="E594" t="n">
+        <v>10.18</v>
+      </c>
+      <c r="F594" t="n">
+        <v>18.3</v>
+      </c>
+      <c r="G594" t="n">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="595">
+      <c r="A595" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="B595" t="inlineStr">
+        <is>
+          <t>NAVN</t>
+        </is>
+      </c>
+      <c r="C595" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D595" t="n">
+        <v>30.88</v>
+      </c>
+      <c r="E595" t="n">
+        <v>28</v>
+      </c>
+      <c r="F595" t="n">
+        <v>36.64</v>
+      </c>
+      <c r="G595" t="n">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="596">
+      <c r="A596" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="B596" t="inlineStr">
+        <is>
+          <t>TTRX</t>
+        </is>
+      </c>
+      <c r="C596" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D596" t="n">
+        <v>10.27</v>
+      </c>
+      <c r="E596" t="n">
+        <v>9.039999999999999</v>
+      </c>
+      <c r="F596" t="n">
+        <v>12.74</v>
+      </c>
+      <c r="G596" t="n">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="597">
+      <c r="A597" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="B597" t="inlineStr">
+        <is>
+          <t>ALOT</t>
+        </is>
+      </c>
+      <c r="C597" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="598">
+      <c r="A598" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="B598" t="inlineStr">
+        <is>
+          <t>BOLD</t>
+        </is>
+      </c>
+      <c r="C598" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="599">
+      <c r="A599" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="B599" t="inlineStr">
+        <is>
+          <t>BOXL</t>
+        </is>
+      </c>
+      <c r="C599" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="600">
+      <c r="A600" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="B600" t="inlineStr">
+        <is>
+          <t>DUKR</t>
+        </is>
+      </c>
+      <c r="C600" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="601">
+      <c r="A601" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="B601" t="inlineStr">
+        <is>
+          <t>FRD</t>
+        </is>
+      </c>
+      <c r="C601" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="602">
+      <c r="A602" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="B602" t="inlineStr">
+        <is>
+          <t>OPAD</t>
+        </is>
+      </c>
+      <c r="C602" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="603">
+      <c r="A603" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="B603" t="inlineStr">
+        <is>
+          <t>PAYS</t>
+        </is>
+      </c>
+      <c r="C603" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="604">
+      <c r="A604" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="B604" t="inlineStr">
+        <is>
+          <t>RRGB</t>
+        </is>
+      </c>
+      <c r="C604" t="inlineStr">
         <is>
           <t>Dropped</t>
         </is>
@@ -14009,7 +14377,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G738"/>
+  <dimension ref="A1:G752"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -30974,6 +31342,328 @@
         </is>
       </c>
       <c r="C738" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="739">
+      <c r="A739" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="B739" t="inlineStr">
+        <is>
+          <t>AUID</t>
+        </is>
+      </c>
+      <c r="C739" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D739" t="n">
+        <v>0.58</v>
+      </c>
+      <c r="E739" t="n">
+        <v>0.41</v>
+      </c>
+      <c r="F739" t="n">
+        <v>0.93</v>
+      </c>
+      <c r="G739" t="n">
+        <v>290</v>
+      </c>
+    </row>
+    <row r="740">
+      <c r="A740" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="B740" t="inlineStr">
+        <is>
+          <t>FTFT</t>
+        </is>
+      </c>
+      <c r="C740" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D740" t="n">
+        <v>2.21</v>
+      </c>
+      <c r="E740" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="F740" t="n">
+        <v>3.43</v>
+      </c>
+      <c r="G740" t="n">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="741">
+      <c r="A741" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="B741" t="inlineStr">
+        <is>
+          <t>MOVE</t>
+        </is>
+      </c>
+      <c r="C741" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D741" t="n">
+        <v>15.09</v>
+      </c>
+      <c r="E741" t="n">
+        <v>10.72</v>
+      </c>
+      <c r="F741" t="n">
+        <v>23.83</v>
+      </c>
+      <c r="G741" t="n">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="742">
+      <c r="A742" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="B742" t="inlineStr">
+        <is>
+          <t>NCRA</t>
+        </is>
+      </c>
+      <c r="C742" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D742" t="n">
+        <v>2.44</v>
+      </c>
+      <c r="E742" t="n">
+        <v>2.23</v>
+      </c>
+      <c r="F742" t="n">
+        <v>2.85</v>
+      </c>
+      <c r="G742" t="n">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="743">
+      <c r="A743" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="B743" t="inlineStr">
+        <is>
+          <t>NEOV</t>
+        </is>
+      </c>
+      <c r="C743" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D743" t="n">
+        <v>4.04</v>
+      </c>
+      <c r="E743" t="n">
+        <v>3.82</v>
+      </c>
+      <c r="F743" t="n">
+        <v>4.47</v>
+      </c>
+      <c r="G743" t="n">
+        <v>229</v>
+      </c>
+    </row>
+    <row r="744">
+      <c r="A744" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="B744" t="inlineStr">
+        <is>
+          <t>SAIC</t>
+        </is>
+      </c>
+      <c r="C744" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D744" t="n">
+        <v>142.42</v>
+      </c>
+      <c r="E744" t="n">
+        <v>127.1</v>
+      </c>
+      <c r="F744" t="n">
+        <v>173.07</v>
+      </c>
+      <c r="G744" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="745">
+      <c r="A745" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="B745" t="inlineStr">
+        <is>
+          <t>VVOS</t>
+        </is>
+      </c>
+      <c r="C745" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D745" t="n">
+        <v>0.46</v>
+      </c>
+      <c r="E745" t="n">
+        <v>0.17</v>
+      </c>
+      <c r="F745" t="n">
+        <v>1.03</v>
+      </c>
+      <c r="G745" t="n">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="746">
+      <c r="A746" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="B746" t="inlineStr">
+        <is>
+          <t>AEMD</t>
+        </is>
+      </c>
+      <c r="C746" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="747">
+      <c r="A747" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="B747" t="inlineStr">
+        <is>
+          <t>AFRM</t>
+        </is>
+      </c>
+      <c r="C747" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="748">
+      <c r="A748" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="B748" t="inlineStr">
+        <is>
+          <t>CYAB</t>
+        </is>
+      </c>
+      <c r="C748" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="749">
+      <c r="A749" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="B749" t="inlineStr">
+        <is>
+          <t>FNGR</t>
+        </is>
+      </c>
+      <c r="C749" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="750">
+      <c r="A750" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="B750" t="inlineStr">
+        <is>
+          <t>GAP</t>
+        </is>
+      </c>
+      <c r="C750" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="751">
+      <c r="A751" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="B751" t="inlineStr">
+        <is>
+          <t>SOLS</t>
+        </is>
+      </c>
+      <c r="C751" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="752">
+      <c r="A752" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="B752" t="inlineStr">
+        <is>
+          <t>WHLR</t>
+        </is>
+      </c>
+      <c r="C752" t="inlineStr">
         <is>
           <t>Dropped</t>
         </is>
@@ -30990,7 +31680,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G23"/>
+  <dimension ref="A1:G24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -31536,6 +32226,35 @@
         </is>
       </c>
     </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>VBIO</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D24" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="E24" t="n">
+        <v>3.85</v>
+      </c>
+      <c r="F24" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="G24" t="n">
+        <v>47</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily screener update: 2026-09-02
</commit_message>
<xml_diff>
--- a/screener_history.xlsx
+++ b/screener_history.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G617"/>
+  <dimension ref="A1:G640"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -14642,6 +14642,541 @@
         </is>
       </c>
       <c r="C617" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="618">
+      <c r="A618" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B618" t="inlineStr">
+        <is>
+          <t>AGPU</t>
+        </is>
+      </c>
+      <c r="C618" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D618" t="n">
+        <v>11.73</v>
+      </c>
+      <c r="E618" t="n">
+        <v>9.07</v>
+      </c>
+      <c r="F618" t="n">
+        <v>17.05</v>
+      </c>
+      <c r="G618" t="n">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="619">
+      <c r="A619" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B619" t="inlineStr">
+        <is>
+          <t>AMLX</t>
+        </is>
+      </c>
+      <c r="C619" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D619" t="n">
+        <v>41.14</v>
+      </c>
+      <c r="E619" t="n">
+        <v>32.98</v>
+      </c>
+      <c r="F619" t="n">
+        <v>57.46</v>
+      </c>
+      <c r="G619" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="620">
+      <c r="A620" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B620" t="inlineStr">
+        <is>
+          <t>EVC</t>
+        </is>
+      </c>
+      <c r="C620" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D620" t="n">
+        <v>8.56</v>
+      </c>
+      <c r="E620" t="n">
+        <v>7.81</v>
+      </c>
+      <c r="F620" t="n">
+        <v>10.06</v>
+      </c>
+      <c r="G620" t="n">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="621">
+      <c r="A621" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B621" t="inlineStr">
+        <is>
+          <t>EXFY</t>
+        </is>
+      </c>
+      <c r="C621" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D621" t="n">
+        <v>2.78</v>
+      </c>
+      <c r="E621" t="n">
+        <v>2.32</v>
+      </c>
+      <c r="F621" t="n">
+        <v>3.7</v>
+      </c>
+      <c r="G621" t="n">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="622">
+      <c r="A622" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B622" t="inlineStr">
+        <is>
+          <t>GSHD</t>
+        </is>
+      </c>
+      <c r="C622" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D622" t="n">
+        <v>74.42</v>
+      </c>
+      <c r="E622" t="n">
+        <v>66.95999999999999</v>
+      </c>
+      <c r="F622" t="n">
+        <v>89.34</v>
+      </c>
+      <c r="G622" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="623">
+      <c r="A623" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B623" t="inlineStr">
+        <is>
+          <t>LCUT</t>
+        </is>
+      </c>
+      <c r="C623" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D623" t="n">
+        <v>9.630000000000001</v>
+      </c>
+      <c r="E623" t="n">
+        <v>8.800000000000001</v>
+      </c>
+      <c r="F623" t="n">
+        <v>11.29</v>
+      </c>
+      <c r="G623" t="n">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="624">
+      <c r="A624" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B624" t="inlineStr">
+        <is>
+          <t>MAN</t>
+        </is>
+      </c>
+      <c r="C624" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D624" t="n">
+        <v>63.88</v>
+      </c>
+      <c r="E624" t="n">
+        <v>59</v>
+      </c>
+      <c r="F624" t="n">
+        <v>73.64</v>
+      </c>
+      <c r="G624" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="625">
+      <c r="A625" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B625" t="inlineStr">
+        <is>
+          <t>PAYS</t>
+        </is>
+      </c>
+      <c r="C625" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D625" t="n">
+        <v>14.43</v>
+      </c>
+      <c r="E625" t="n">
+        <v>12.08</v>
+      </c>
+      <c r="F625" t="n">
+        <v>19.13</v>
+      </c>
+      <c r="G625" t="n">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="626">
+      <c r="A626" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B626" t="inlineStr">
+        <is>
+          <t>TWST</t>
+        </is>
+      </c>
+      <c r="C626" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D626" t="n">
+        <v>155.44</v>
+      </c>
+      <c r="E626" t="n">
+        <v>126.42</v>
+      </c>
+      <c r="F626" t="n">
+        <v>213.48</v>
+      </c>
+      <c r="G626" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="627">
+      <c r="A627" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B627" t="inlineStr">
+        <is>
+          <t>TXG</t>
+        </is>
+      </c>
+      <c r="C627" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D627" t="n">
+        <v>66.94</v>
+      </c>
+      <c r="E627" t="n">
+        <v>58.7</v>
+      </c>
+      <c r="F627" t="n">
+        <v>83.42</v>
+      </c>
+      <c r="G627" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="628">
+      <c r="A628" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B628" t="inlineStr">
+        <is>
+          <t>XNCR</t>
+        </is>
+      </c>
+      <c r="C628" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D628" t="n">
+        <v>30.61</v>
+      </c>
+      <c r="E628" t="n">
+        <v>25.81</v>
+      </c>
+      <c r="F628" t="n">
+        <v>40.22</v>
+      </c>
+      <c r="G628" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="629">
+      <c r="A629" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B629" t="inlineStr">
+        <is>
+          <t>ZSTK</t>
+        </is>
+      </c>
+      <c r="C629" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D629" t="n">
+        <v>6.9</v>
+      </c>
+      <c r="E629" t="n">
+        <v>4.12</v>
+      </c>
+      <c r="F629" t="n">
+        <v>12.46</v>
+      </c>
+      <c r="G629" t="n">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="630">
+      <c r="A630" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B630" t="inlineStr">
+        <is>
+          <t>BWMN</t>
+        </is>
+      </c>
+      <c r="C630" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="631">
+      <c r="A631" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B631" t="inlineStr">
+        <is>
+          <t>BYND</t>
+        </is>
+      </c>
+      <c r="C631" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="632">
+      <c r="A632" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B632" t="inlineStr">
+        <is>
+          <t>FATN</t>
+        </is>
+      </c>
+      <c r="C632" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="633">
+      <c r="A633" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B633" t="inlineStr">
+        <is>
+          <t>KIDZ</t>
+        </is>
+      </c>
+      <c r="C633" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="634">
+      <c r="A634" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B634" t="inlineStr">
+        <is>
+          <t>LNSR</t>
+        </is>
+      </c>
+      <c r="C634" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="635">
+      <c r="A635" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B635" t="inlineStr">
+        <is>
+          <t>MU</t>
+        </is>
+      </c>
+      <c r="C635" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="636">
+      <c r="A636" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B636" t="inlineStr">
+        <is>
+          <t>SLS</t>
+        </is>
+      </c>
+      <c r="C636" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="637">
+      <c r="A637" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B637" t="inlineStr">
+        <is>
+          <t>SNDK</t>
+        </is>
+      </c>
+      <c r="C637" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="638">
+      <c r="A638" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B638" t="inlineStr">
+        <is>
+          <t>STIM</t>
+        </is>
+      </c>
+      <c r="C638" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="639">
+      <c r="A639" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B639" t="inlineStr">
+        <is>
+          <t>TKNO</t>
+        </is>
+      </c>
+      <c r="C639" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="640">
+      <c r="A640" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B640" t="inlineStr">
+        <is>
+          <t>VREX</t>
+        </is>
+      </c>
+      <c r="C640" t="inlineStr">
         <is>
           <t>Dropped</t>
         </is>
@@ -14658,7 +15193,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G766"/>
+  <dimension ref="A1:G778"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -32267,6 +32802,282 @@
         </is>
       </c>
       <c r="C766" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="767">
+      <c r="A767" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B767" t="inlineStr">
+        <is>
+          <t>DAKT</t>
+        </is>
+      </c>
+      <c r="C767" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D767" t="n">
+        <v>21.59</v>
+      </c>
+      <c r="E767" t="n">
+        <v>18.99</v>
+      </c>
+      <c r="F767" t="n">
+        <v>26.8</v>
+      </c>
+      <c r="G767" t="n">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="768">
+      <c r="A768" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B768" t="inlineStr">
+        <is>
+          <t>DH</t>
+        </is>
+      </c>
+      <c r="C768" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D768" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="E768" t="n">
+        <v>1.02</v>
+      </c>
+      <c r="F768" t="n">
+        <v>1.26</v>
+      </c>
+      <c r="G768" t="n">
+        <v>624</v>
+      </c>
+    </row>
+    <row r="769">
+      <c r="A769" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B769" t="inlineStr">
+        <is>
+          <t>GTLB</t>
+        </is>
+      </c>
+      <c r="C769" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D769" t="n">
+        <v>55.55</v>
+      </c>
+      <c r="E769" t="n">
+        <v>49.11</v>
+      </c>
+      <c r="F769" t="n">
+        <v>68.43000000000001</v>
+      </c>
+      <c r="G769" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="770">
+      <c r="A770" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B770" t="inlineStr">
+        <is>
+          <t>LHAI</t>
+        </is>
+      </c>
+      <c r="C770" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D770" t="n">
+        <v>1.26</v>
+      </c>
+      <c r="E770" t="n">
+        <v>0.96</v>
+      </c>
+      <c r="F770" t="n">
+        <v>1.86</v>
+      </c>
+      <c r="G770" t="n">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="771">
+      <c r="A771" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B771" t="inlineStr">
+        <is>
+          <t>SPWH</t>
+        </is>
+      </c>
+      <c r="C771" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D771" t="n">
+        <v>1.36</v>
+      </c>
+      <c r="E771" t="n">
+        <v>1.21</v>
+      </c>
+      <c r="F771" t="n">
+        <v>1.66</v>
+      </c>
+      <c r="G771" t="n">
+        <v>333</v>
+      </c>
+    </row>
+    <row r="772">
+      <c r="A772" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B772" t="inlineStr">
+        <is>
+          <t>VIVK</t>
+        </is>
+      </c>
+      <c r="C772" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D772" t="n">
+        <v>1.14</v>
+      </c>
+      <c r="E772" t="n">
+        <v>0.87</v>
+      </c>
+      <c r="F772" t="n">
+        <v>1.69</v>
+      </c>
+      <c r="G772" t="n">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="773">
+      <c r="A773" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B773" t="inlineStr">
+        <is>
+          <t>FLYE</t>
+        </is>
+      </c>
+      <c r="C773" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="774">
+      <c r="A774" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B774" t="inlineStr">
+        <is>
+          <t>GPRO</t>
+        </is>
+      </c>
+      <c r="C774" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="775">
+      <c r="A775" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B775" t="inlineStr">
+        <is>
+          <t>LIDR</t>
+        </is>
+      </c>
+      <c r="C775" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="776">
+      <c r="A776" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B776" t="inlineStr">
+        <is>
+          <t>PXS</t>
+        </is>
+      </c>
+      <c r="C776" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="777">
+      <c r="A777" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B777" t="inlineStr">
+        <is>
+          <t>SST</t>
+        </is>
+      </c>
+      <c r="C777" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="778">
+      <c r="A778" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B778" t="inlineStr">
+        <is>
+          <t>VSTD</t>
+        </is>
+      </c>
+      <c r="C778" t="inlineStr">
         <is>
           <t>Dropped</t>
         </is>
@@ -32283,7 +33094,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G25"/>
+  <dimension ref="A1:G26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -32875,6 +33686,35 @@
         </is>
       </c>
     </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>ARTL</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D26" t="n">
+        <v>6.27</v>
+      </c>
+      <c r="E26" t="n">
+        <v>6.71</v>
+      </c>
+      <c r="F26" t="n">
+        <v>5.39</v>
+      </c>
+      <c r="G26" t="n">
+        <v>114</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily screener update: 2026-09-03
</commit_message>
<xml_diff>
--- a/screener_history.xlsx
+++ b/screener_history.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G640"/>
+  <dimension ref="A1:G655"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -15177,6 +15177,345 @@
         </is>
       </c>
       <c r="C640" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="641">
+      <c r="A641" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="B641" t="inlineStr">
+        <is>
+          <t>CADL</t>
+        </is>
+      </c>
+      <c r="C641" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D641" t="n">
+        <v>14</v>
+      </c>
+      <c r="E641" t="n">
+        <v>12.38</v>
+      </c>
+      <c r="F641" t="n">
+        <v>17.24</v>
+      </c>
+      <c r="G641" t="n">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="642">
+      <c r="A642" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="B642" t="inlineStr">
+        <is>
+          <t>CRNX</t>
+        </is>
+      </c>
+      <c r="C642" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D642" t="n">
+        <v>85.01000000000001</v>
+      </c>
+      <c r="E642" t="n">
+        <v>83.8</v>
+      </c>
+      <c r="F642" t="n">
+        <v>87.43000000000001</v>
+      </c>
+      <c r="G642" t="n">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="643">
+      <c r="A643" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="B643" t="inlineStr">
+        <is>
+          <t>DUKR</t>
+        </is>
+      </c>
+      <c r="C643" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D643" t="n">
+        <v>5.82</v>
+      </c>
+      <c r="E643" t="n">
+        <v>5.31</v>
+      </c>
+      <c r="F643" t="n">
+        <v>6.85</v>
+      </c>
+      <c r="G643" t="n">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="644">
+      <c r="A644" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="B644" t="inlineStr">
+        <is>
+          <t>KIDZ</t>
+        </is>
+      </c>
+      <c r="C644" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D644" t="n">
+        <v>5.26</v>
+      </c>
+      <c r="E644" t="n">
+        <v>3.35</v>
+      </c>
+      <c r="F644" t="n">
+        <v>9.08</v>
+      </c>
+      <c r="G644" t="n">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="645">
+      <c r="A645" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="B645" t="inlineStr">
+        <is>
+          <t>RCMT</t>
+        </is>
+      </c>
+      <c r="C645" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D645" t="n">
+        <v>43.09</v>
+      </c>
+      <c r="E645" t="n">
+        <v>40.2</v>
+      </c>
+      <c r="F645" t="n">
+        <v>48.87</v>
+      </c>
+      <c r="G645" t="n">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="646">
+      <c r="A646" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="B646" t="inlineStr">
+        <is>
+          <t>SLS</t>
+        </is>
+      </c>
+      <c r="C646" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D646" t="n">
+        <v>15.67</v>
+      </c>
+      <c r="E646" t="n">
+        <v>12.64</v>
+      </c>
+      <c r="F646" t="n">
+        <v>21.73</v>
+      </c>
+      <c r="G646" t="n">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="647">
+      <c r="A647" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="B647" t="inlineStr">
+        <is>
+          <t>TKNO</t>
+        </is>
+      </c>
+      <c r="C647" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D647" t="n">
+        <v>7.64</v>
+      </c>
+      <c r="E647" t="n">
+        <v>6.85</v>
+      </c>
+      <c r="F647" t="n">
+        <v>9.220000000000001</v>
+      </c>
+      <c r="G647" t="n">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="648">
+      <c r="A648" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="B648" t="inlineStr">
+        <is>
+          <t>CJMB</t>
+        </is>
+      </c>
+      <c r="C648" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="649">
+      <c r="A649" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="B649" t="inlineStr">
+        <is>
+          <t>EVC</t>
+        </is>
+      </c>
+      <c r="C649" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="650">
+      <c r="A650" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="B650" t="inlineStr">
+        <is>
+          <t>GSHD</t>
+        </is>
+      </c>
+      <c r="C650" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="651">
+      <c r="A651" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="B651" t="inlineStr">
+        <is>
+          <t>LCUT</t>
+        </is>
+      </c>
+      <c r="C651" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="652">
+      <c r="A652" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="B652" t="inlineStr">
+        <is>
+          <t>PAYS</t>
+        </is>
+      </c>
+      <c r="C652" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="653">
+      <c r="A653" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="B653" t="inlineStr">
+        <is>
+          <t>TTRX</t>
+        </is>
+      </c>
+      <c r="C653" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="654">
+      <c r="A654" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="B654" t="inlineStr">
+        <is>
+          <t>TWST</t>
+        </is>
+      </c>
+      <c r="C654" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="655">
+      <c r="A655" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="B655" t="inlineStr">
+        <is>
+          <t>TXG</t>
+        </is>
+      </c>
+      <c r="C655" t="inlineStr">
         <is>
           <t>Dropped</t>
         </is>
@@ -15193,7 +15532,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G778"/>
+  <dimension ref="A1:G792"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -33078,6 +33417,340 @@
         </is>
       </c>
       <c r="C778" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="779">
+      <c r="A779" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="B779" t="inlineStr">
+        <is>
+          <t>BTAI</t>
+        </is>
+      </c>
+      <c r="C779" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D779" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="E779" t="n">
+        <v>0.11</v>
+      </c>
+      <c r="F779" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="G779" t="n">
+        <v>4201</v>
+      </c>
+    </row>
+    <row r="780">
+      <c r="A780" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="B780" t="inlineStr">
+        <is>
+          <t>CHPT</t>
+        </is>
+      </c>
+      <c r="C780" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D780" t="n">
+        <v>7.65</v>
+      </c>
+      <c r="E780" t="n">
+        <v>6.71</v>
+      </c>
+      <c r="F780" t="n">
+        <v>9.529999999999999</v>
+      </c>
+      <c r="G780" t="n">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="781">
+      <c r="A781" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="B781" t="inlineStr">
+        <is>
+          <t>DLTH</t>
+        </is>
+      </c>
+      <c r="C781" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D781" t="n">
+        <v>4.28</v>
+      </c>
+      <c r="E781" t="n">
+        <v>3.8</v>
+      </c>
+      <c r="F781" t="n">
+        <v>5.24</v>
+      </c>
+      <c r="G781" t="n">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="782">
+      <c r="A782" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="B782" t="inlineStr">
+        <is>
+          <t>GIPR</t>
+        </is>
+      </c>
+      <c r="C782" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D782" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="E782" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="F782" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="G782" t="n">
+        <v>335</v>
+      </c>
+    </row>
+    <row r="783">
+      <c r="A783" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="B783" t="inlineStr">
+        <is>
+          <t>SID</t>
+        </is>
+      </c>
+      <c r="C783" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D783" t="n">
+        <v>1.37</v>
+      </c>
+      <c r="E783" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="F783" t="n">
+        <v>1.69</v>
+      </c>
+      <c r="G783" t="n">
+        <v>303</v>
+      </c>
+    </row>
+    <row r="784">
+      <c r="A784" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="B784" t="inlineStr">
+        <is>
+          <t>SNOW</t>
+        </is>
+      </c>
+      <c r="C784" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D784" t="n">
+        <v>384.56</v>
+      </c>
+      <c r="E784" t="n">
+        <v>355.47</v>
+      </c>
+      <c r="F784" t="n">
+        <v>442.74</v>
+      </c>
+      <c r="G784" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="785">
+      <c r="A785" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="B785" t="inlineStr">
+        <is>
+          <t>TLYS</t>
+        </is>
+      </c>
+      <c r="C785" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D785" t="n">
+        <v>6.25</v>
+      </c>
+      <c r="E785" t="n">
+        <v>4</v>
+      </c>
+      <c r="F785" t="n">
+        <v>10.75</v>
+      </c>
+      <c r="G785" t="n">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="786">
+      <c r="A786" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="B786" t="inlineStr">
+        <is>
+          <t>WOOF</t>
+        </is>
+      </c>
+      <c r="C786" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D786" t="n">
+        <v>3.22</v>
+      </c>
+      <c r="E786" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="F786" t="n">
+        <v>4.66</v>
+      </c>
+      <c r="G786" t="n">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="787">
+      <c r="A787" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="B787" t="inlineStr">
+        <is>
+          <t>DAKT</t>
+        </is>
+      </c>
+      <c r="C787" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="788">
+      <c r="A788" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="B788" t="inlineStr">
+        <is>
+          <t>DH</t>
+        </is>
+      </c>
+      <c r="C788" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="789">
+      <c r="A789" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="B789" t="inlineStr">
+        <is>
+          <t>GTLB</t>
+        </is>
+      </c>
+      <c r="C789" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="790">
+      <c r="A790" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="B790" t="inlineStr">
+        <is>
+          <t>LHAI</t>
+        </is>
+      </c>
+      <c r="C790" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="791">
+      <c r="A791" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="B791" t="inlineStr">
+        <is>
+          <t>SPWH</t>
+        </is>
+      </c>
+      <c r="C791" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="792">
+      <c r="A792" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="B792" t="inlineStr">
+        <is>
+          <t>VIVK</t>
+        </is>
+      </c>
+      <c r="C792" t="inlineStr">
         <is>
           <t>Dropped</t>
         </is>
@@ -33094,7 +33767,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G26"/>
+  <dimension ref="A1:G27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -33715,6 +34388,23 @@
         <v>114</v>
       </c>
     </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>ARTL</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily screener update: 2026-09-04
</commit_message>
<xml_diff>
--- a/screener_history.xlsx
+++ b/screener_history.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G655"/>
+  <dimension ref="A1:G674"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -15516,6 +15516,413 @@
         </is>
       </c>
       <c r="C655" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="656">
+      <c r="A656" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="B656" t="inlineStr">
+        <is>
+          <t>ASTC</t>
+        </is>
+      </c>
+      <c r="C656" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D656" t="n">
+        <v>7.89</v>
+      </c>
+      <c r="E656" t="n">
+        <v>6.8</v>
+      </c>
+      <c r="F656" t="n">
+        <v>10.07</v>
+      </c>
+      <c r="G656" t="n">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="657">
+      <c r="A657" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="B657" t="inlineStr">
+        <is>
+          <t>AVAH</t>
+        </is>
+      </c>
+      <c r="C657" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D657" t="n">
+        <v>14</v>
+      </c>
+      <c r="E657" t="n">
+        <v>12.97</v>
+      </c>
+      <c r="F657" t="n">
+        <v>16.06</v>
+      </c>
+      <c r="G657" t="n">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="658">
+      <c r="A658" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="B658" t="inlineStr">
+        <is>
+          <t>BYND</t>
+        </is>
+      </c>
+      <c r="C658" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D658" t="n">
+        <v>15.02</v>
+      </c>
+      <c r="E658" t="n">
+        <v>11.04</v>
+      </c>
+      <c r="F658" t="n">
+        <v>22.98</v>
+      </c>
+      <c r="G658" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="659">
+      <c r="A659" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="B659" t="inlineStr">
+        <is>
+          <t>HTFL</t>
+        </is>
+      </c>
+      <c r="C659" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D659" t="n">
+        <v>51.78</v>
+      </c>
+      <c r="E659" t="n">
+        <v>47.13</v>
+      </c>
+      <c r="F659" t="n">
+        <v>61.07</v>
+      </c>
+      <c r="G659" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="660">
+      <c r="A660" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="B660" t="inlineStr">
+        <is>
+          <t>MRNA</t>
+        </is>
+      </c>
+      <c r="C660" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D660" t="n">
+        <v>161.37</v>
+      </c>
+      <c r="E660" t="n">
+        <v>130</v>
+      </c>
+      <c r="F660" t="n">
+        <v>224.11</v>
+      </c>
+      <c r="G660" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="661">
+      <c r="A661" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="B661" t="inlineStr">
+        <is>
+          <t>OABI</t>
+        </is>
+      </c>
+      <c r="C661" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D661" t="n">
+        <v>5.43</v>
+      </c>
+      <c r="E661" t="n">
+        <v>4.2</v>
+      </c>
+      <c r="F661" t="n">
+        <v>7.89</v>
+      </c>
+      <c r="G661" t="n">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="662">
+      <c r="A662" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="B662" t="inlineStr">
+        <is>
+          <t>PEPG</t>
+        </is>
+      </c>
+      <c r="C662" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D662" t="n">
+        <v>3.57</v>
+      </c>
+      <c r="E662" t="n">
+        <v>2.91</v>
+      </c>
+      <c r="F662" t="n">
+        <v>4.89</v>
+      </c>
+      <c r="G662" t="n">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="663">
+      <c r="A663" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="B663" t="inlineStr">
+        <is>
+          <t>AGPU</t>
+        </is>
+      </c>
+      <c r="C663" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="664">
+      <c r="A664" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="B664" t="inlineStr">
+        <is>
+          <t>AIFA</t>
+        </is>
+      </c>
+      <c r="C664" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="665">
+      <c r="A665" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="B665" t="inlineStr">
+        <is>
+          <t>CURX</t>
+        </is>
+      </c>
+      <c r="C665" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="666">
+      <c r="A666" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="B666" t="inlineStr">
+        <is>
+          <t>DUKR</t>
+        </is>
+      </c>
+      <c r="C666" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="667">
+      <c r="A667" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="B667" t="inlineStr">
+        <is>
+          <t>EXFY</t>
+        </is>
+      </c>
+      <c r="C667" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="668">
+      <c r="A668" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="B668" t="inlineStr">
+        <is>
+          <t>HELP</t>
+        </is>
+      </c>
+      <c r="C668" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="669">
+      <c r="A669" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="B669" t="inlineStr">
+        <is>
+          <t>KIDZ</t>
+        </is>
+      </c>
+      <c r="C669" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="670">
+      <c r="A670" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="B670" t="inlineStr">
+        <is>
+          <t>MAN</t>
+        </is>
+      </c>
+      <c r="C670" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="671">
+      <c r="A671" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="B671" t="inlineStr">
+        <is>
+          <t>MYSZ</t>
+        </is>
+      </c>
+      <c r="C671" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="672">
+      <c r="A672" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="B672" t="inlineStr">
+        <is>
+          <t>RCMT</t>
+        </is>
+      </c>
+      <c r="C672" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="673">
+      <c r="A673" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="B673" t="inlineStr">
+        <is>
+          <t>SLS</t>
+        </is>
+      </c>
+      <c r="C673" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="674">
+      <c r="A674" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="B674" t="inlineStr">
+        <is>
+          <t>TKNO</t>
+        </is>
+      </c>
+      <c r="C674" t="inlineStr">
         <is>
           <t>Dropped</t>
         </is>
@@ -15532,7 +15939,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G792"/>
+  <dimension ref="A1:G807"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -33751,6 +34158,333 @@
         </is>
       </c>
       <c r="C792" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="793">
+      <c r="A793" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="B793" t="inlineStr">
+        <is>
+          <t>AOUT</t>
+        </is>
+      </c>
+      <c r="C793" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D793" t="n">
+        <v>13.76</v>
+      </c>
+      <c r="E793" t="n">
+        <v>12.76</v>
+      </c>
+      <c r="F793" t="n">
+        <v>15.76</v>
+      </c>
+      <c r="G793" t="n">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="794">
+      <c r="A794" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="B794" t="inlineStr">
+        <is>
+          <t>BBCP</t>
+        </is>
+      </c>
+      <c r="C794" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D794" t="n">
+        <v>10.95</v>
+      </c>
+      <c r="E794" t="n">
+        <v>9.69</v>
+      </c>
+      <c r="F794" t="n">
+        <v>13.47</v>
+      </c>
+      <c r="G794" t="n">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="795">
+      <c r="A795" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="B795" t="inlineStr">
+        <is>
+          <t>CURV</t>
+        </is>
+      </c>
+      <c r="C795" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D795" t="n">
+        <v>2.58</v>
+      </c>
+      <c r="E795" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="F795" t="n">
+        <v>2.94</v>
+      </c>
+      <c r="G795" t="n">
+        <v>277</v>
+      </c>
+    </row>
+    <row r="796">
+      <c r="A796" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="B796" t="inlineStr">
+        <is>
+          <t>IOT</t>
+        </is>
+      </c>
+      <c r="C796" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D796" t="n">
+        <v>45.12</v>
+      </c>
+      <c r="E796" t="n">
+        <v>39.32</v>
+      </c>
+      <c r="F796" t="n">
+        <v>56.72</v>
+      </c>
+      <c r="G796" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="797">
+      <c r="A797" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="B797" t="inlineStr">
+        <is>
+          <t>MTEX</t>
+        </is>
+      </c>
+      <c r="C797" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D797" t="n">
+        <v>8.050000000000001</v>
+      </c>
+      <c r="E797" t="n">
+        <v>7.39</v>
+      </c>
+      <c r="F797" t="n">
+        <v>9.359999999999999</v>
+      </c>
+      <c r="G797" t="n">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="798">
+      <c r="A798" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="B798" t="inlineStr">
+        <is>
+          <t>SWBI</t>
+        </is>
+      </c>
+      <c r="C798" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D798" t="n">
+        <v>14.06</v>
+      </c>
+      <c r="E798" t="n">
+        <v>12.12</v>
+      </c>
+      <c r="F798" t="n">
+        <v>17.94</v>
+      </c>
+      <c r="G798" t="n">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="799">
+      <c r="A799" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="B799" t="inlineStr">
+        <is>
+          <t>BIAF</t>
+        </is>
+      </c>
+      <c r="C799" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="800">
+      <c r="A800" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="B800" t="inlineStr">
+        <is>
+          <t>BTAI</t>
+        </is>
+      </c>
+      <c r="C800" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="801">
+      <c r="A801" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="B801" t="inlineStr">
+        <is>
+          <t>CHPT</t>
+        </is>
+      </c>
+      <c r="C801" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="802">
+      <c r="A802" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="B802" t="inlineStr">
+        <is>
+          <t>DLTH</t>
+        </is>
+      </c>
+      <c r="C802" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="803">
+      <c r="A803" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="B803" t="inlineStr">
+        <is>
+          <t>GIPR</t>
+        </is>
+      </c>
+      <c r="C803" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="804">
+      <c r="A804" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="B804" t="inlineStr">
+        <is>
+          <t>SID</t>
+        </is>
+      </c>
+      <c r="C804" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="805">
+      <c r="A805" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="B805" t="inlineStr">
+        <is>
+          <t>SNOW</t>
+        </is>
+      </c>
+      <c r="C805" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="806">
+      <c r="A806" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="B806" t="inlineStr">
+        <is>
+          <t>TLYS</t>
+        </is>
+      </c>
+      <c r="C806" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="807">
+      <c r="A807" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="B807" t="inlineStr">
+        <is>
+          <t>WOOF</t>
+        </is>
+      </c>
+      <c r="C807" t="inlineStr">
         <is>
           <t>Dropped</t>
         </is>

</xml_diff>

<commit_message>
Daily screener update: 2026-09-07
</commit_message>
<xml_diff>
--- a/screener_history.xlsx
+++ b/screener_history.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G674"/>
+  <dimension ref="A1:G685"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -15923,6 +15923,289 @@
         </is>
       </c>
       <c r="C674" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="675">
+      <c r="A675" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="B675" t="inlineStr">
+        <is>
+          <t>APGE</t>
+        </is>
+      </c>
+      <c r="C675" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D675" t="n">
+        <v>134.32</v>
+      </c>
+      <c r="E675" t="n">
+        <v>133.13</v>
+      </c>
+      <c r="F675" t="n">
+        <v>136.7</v>
+      </c>
+      <c r="G675" t="n">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="676">
+      <c r="A676" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="B676" t="inlineStr">
+        <is>
+          <t>BWMN</t>
+        </is>
+      </c>
+      <c r="C676" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D676" t="n">
+        <v>43.13</v>
+      </c>
+      <c r="E676" t="n">
+        <v>42.43</v>
+      </c>
+      <c r="F676" t="n">
+        <v>44.54</v>
+      </c>
+      <c r="G676" t="n">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="677">
+      <c r="A677" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="B677" t="inlineStr">
+        <is>
+          <t>GLBS</t>
+        </is>
+      </c>
+      <c r="C677" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D677" t="n">
+        <v>3.9</v>
+      </c>
+      <c r="E677" t="n">
+        <v>3.49</v>
+      </c>
+      <c r="F677" t="n">
+        <v>4.72</v>
+      </c>
+      <c r="G677" t="n">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="678">
+      <c r="A678" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="B678" t="inlineStr">
+        <is>
+          <t>OMER</t>
+        </is>
+      </c>
+      <c r="C678" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D678" t="n">
+        <v>19.65</v>
+      </c>
+      <c r="E678" t="n">
+        <v>18</v>
+      </c>
+      <c r="F678" t="n">
+        <v>22.95</v>
+      </c>
+      <c r="G678" t="n">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="679">
+      <c r="A679" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="B679" t="inlineStr">
+        <is>
+          <t>RCMT</t>
+        </is>
+      </c>
+      <c r="C679" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D679" t="n">
+        <v>43.09</v>
+      </c>
+      <c r="E679" t="n">
+        <v>40.2</v>
+      </c>
+      <c r="F679" t="n">
+        <v>48.87</v>
+      </c>
+      <c r="G679" t="n">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="680">
+      <c r="A680" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="B680" t="inlineStr">
+        <is>
+          <t>TVTX</t>
+        </is>
+      </c>
+      <c r="C680" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D680" t="n">
+        <v>68.03</v>
+      </c>
+      <c r="E680" t="n">
+        <v>63.71</v>
+      </c>
+      <c r="F680" t="n">
+        <v>76.67</v>
+      </c>
+      <c r="G680" t="n">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="681">
+      <c r="A681" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="B681" t="inlineStr">
+        <is>
+          <t>USIO</t>
+        </is>
+      </c>
+      <c r="C681" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D681" t="n">
+        <v>3.06</v>
+      </c>
+      <c r="E681" t="n">
+        <v>2.63</v>
+      </c>
+      <c r="F681" t="n">
+        <v>3.92</v>
+      </c>
+      <c r="G681" t="n">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="682">
+      <c r="A682" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="B682" t="inlineStr">
+        <is>
+          <t>VREX</t>
+        </is>
+      </c>
+      <c r="C682" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D682" t="n">
+        <v>18.54</v>
+      </c>
+      <c r="E682" t="n">
+        <v>18.45</v>
+      </c>
+      <c r="F682" t="n">
+        <v>18.72</v>
+      </c>
+      <c r="G682" t="n">
+        <v>555</v>
+      </c>
+    </row>
+    <row r="683">
+      <c r="A683" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="B683" t="inlineStr">
+        <is>
+          <t>BYND</t>
+        </is>
+      </c>
+      <c r="C683" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="684">
+      <c r="A684" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="B684" t="inlineStr">
+        <is>
+          <t>CSAI</t>
+        </is>
+      </c>
+      <c r="C684" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="685">
+      <c r="A685" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="B685" t="inlineStr">
+        <is>
+          <t>NRDY</t>
+        </is>
+      </c>
+      <c r="C685" t="inlineStr">
         <is>
           <t>Dropped</t>
         </is>

</xml_diff>

<commit_message>
Daily screener update: 2026-09-08
</commit_message>
<xml_diff>
--- a/screener_history.xlsx
+++ b/screener_history.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G685"/>
+  <dimension ref="A1:G706"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -16206,6 +16206,531 @@
         </is>
       </c>
       <c r="C685" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="686">
+      <c r="A686" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B686" t="inlineStr">
+        <is>
+          <t>AIFA</t>
+        </is>
+      </c>
+      <c r="C686" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D686" t="n">
+        <v>3.34</v>
+      </c>
+      <c r="E686" t="n">
+        <v>2.72</v>
+      </c>
+      <c r="F686" t="n">
+        <v>4.57</v>
+      </c>
+      <c r="G686" t="n">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="687">
+      <c r="A687" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B687" t="inlineStr">
+        <is>
+          <t>ANRO</t>
+        </is>
+      </c>
+      <c r="C687" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D687" t="n">
+        <v>37.48</v>
+      </c>
+      <c r="E687" t="n">
+        <v>33.98</v>
+      </c>
+      <c r="F687" t="n">
+        <v>44.48</v>
+      </c>
+      <c r="G687" t="n">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="688">
+      <c r="A688" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B688" t="inlineStr">
+        <is>
+          <t>BIVI</t>
+        </is>
+      </c>
+      <c r="C688" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D688" t="n">
+        <v>2.49</v>
+      </c>
+      <c r="E688" t="n">
+        <v>1.93</v>
+      </c>
+      <c r="F688" t="n">
+        <v>3.61</v>
+      </c>
+      <c r="G688" t="n">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="689">
+      <c r="A689" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B689" t="inlineStr">
+        <is>
+          <t>ELF</t>
+        </is>
+      </c>
+      <c r="C689" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D689" t="n">
+        <v>110.04</v>
+      </c>
+      <c r="E689" t="n">
+        <v>102.39</v>
+      </c>
+      <c r="F689" t="n">
+        <v>125.33</v>
+      </c>
+      <c r="G689" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="690">
+      <c r="A690" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B690" t="inlineStr">
+        <is>
+          <t>HHS</t>
+        </is>
+      </c>
+      <c r="C690" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D690" t="n">
+        <v>4.4</v>
+      </c>
+      <c r="E690" t="n">
+        <v>3.94</v>
+      </c>
+      <c r="F690" t="n">
+        <v>5.32</v>
+      </c>
+      <c r="G690" t="n">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="691">
+      <c r="A691" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B691" t="inlineStr">
+        <is>
+          <t>LNSR</t>
+        </is>
+      </c>
+      <c r="C691" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D691" t="n">
+        <v>9.25</v>
+      </c>
+      <c r="E691" t="n">
+        <v>8.210000000000001</v>
+      </c>
+      <c r="F691" t="n">
+        <v>11.33</v>
+      </c>
+      <c r="G691" t="n">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="692">
+      <c r="A692" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B692" t="inlineStr">
+        <is>
+          <t>NVCT</t>
+        </is>
+      </c>
+      <c r="C692" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D692" t="n">
+        <v>25.94</v>
+      </c>
+      <c r="E692" t="n">
+        <v>22.57</v>
+      </c>
+      <c r="F692" t="n">
+        <v>32.68</v>
+      </c>
+      <c r="G692" t="n">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="693">
+      <c r="A693" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B693" t="inlineStr">
+        <is>
+          <t>PLSE</t>
+        </is>
+      </c>
+      <c r="C693" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D693" t="n">
+        <v>55.37</v>
+      </c>
+      <c r="E693" t="n">
+        <v>47.01</v>
+      </c>
+      <c r="F693" t="n">
+        <v>72.09</v>
+      </c>
+      <c r="G693" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="694">
+      <c r="A694" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B694" t="inlineStr">
+        <is>
+          <t>RCEL</t>
+        </is>
+      </c>
+      <c r="C694" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D694" t="n">
+        <v>11.39</v>
+      </c>
+      <c r="E694" t="n">
+        <v>9.84</v>
+      </c>
+      <c r="F694" t="n">
+        <v>14.49</v>
+      </c>
+      <c r="G694" t="n">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="695">
+      <c r="A695" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B695" t="inlineStr">
+        <is>
+          <t>SENS</t>
+        </is>
+      </c>
+      <c r="C695" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D695" t="n">
+        <v>10.15</v>
+      </c>
+      <c r="E695" t="n">
+        <v>8.970000000000001</v>
+      </c>
+      <c r="F695" t="n">
+        <v>12.51</v>
+      </c>
+      <c r="G695" t="n">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="696">
+      <c r="A696" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B696" t="inlineStr">
+        <is>
+          <t>SGHT</t>
+        </is>
+      </c>
+      <c r="C696" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D696" t="n">
+        <v>8.789999999999999</v>
+      </c>
+      <c r="E696" t="n">
+        <v>7.82</v>
+      </c>
+      <c r="F696" t="n">
+        <v>10.73</v>
+      </c>
+      <c r="G696" t="n">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="697">
+      <c r="A697" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B697" t="inlineStr">
+        <is>
+          <t>STIM</t>
+        </is>
+      </c>
+      <c r="C697" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D697" t="n">
+        <v>3.04</v>
+      </c>
+      <c r="E697" t="n">
+        <v>2.67</v>
+      </c>
+      <c r="F697" t="n">
+        <v>3.78</v>
+      </c>
+      <c r="G697" t="n">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="698">
+      <c r="A698" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B698" t="inlineStr">
+        <is>
+          <t>TMCI</t>
+        </is>
+      </c>
+      <c r="C698" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D698" t="n">
+        <v>5.01</v>
+      </c>
+      <c r="E698" t="n">
+        <v>4.41</v>
+      </c>
+      <c r="F698" t="n">
+        <v>6.22</v>
+      </c>
+      <c r="G698" t="n">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="699">
+      <c r="A699" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B699" t="inlineStr">
+        <is>
+          <t>UTZ</t>
+        </is>
+      </c>
+      <c r="C699" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D699" t="n">
+        <v>14.27</v>
+      </c>
+      <c r="E699" t="n">
+        <v>14.18</v>
+      </c>
+      <c r="F699" t="n">
+        <v>14.45</v>
+      </c>
+      <c r="G699" t="n">
+        <v>555</v>
+      </c>
+    </row>
+    <row r="700">
+      <c r="A700" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B700" t="inlineStr">
+        <is>
+          <t>ASTC</t>
+        </is>
+      </c>
+      <c r="C700" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="701">
+      <c r="A701" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B701" t="inlineStr">
+        <is>
+          <t>GLBS</t>
+        </is>
+      </c>
+      <c r="C701" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="702">
+      <c r="A702" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B702" t="inlineStr">
+        <is>
+          <t>OMER</t>
+        </is>
+      </c>
+      <c r="C702" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="703">
+      <c r="A703" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B703" t="inlineStr">
+        <is>
+          <t>PEPG</t>
+        </is>
+      </c>
+      <c r="C703" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="704">
+      <c r="A704" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B704" t="inlineStr">
+        <is>
+          <t>TVTX</t>
+        </is>
+      </c>
+      <c r="C704" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="705">
+      <c r="A705" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B705" t="inlineStr">
+        <is>
+          <t>USIO</t>
+        </is>
+      </c>
+      <c r="C705" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="706">
+      <c r="A706" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B706" t="inlineStr">
+        <is>
+          <t>XNCR</t>
+        </is>
+      </c>
+      <c r="C706" t="inlineStr">
         <is>
           <t>Dropped</t>
         </is>
@@ -16222,7 +16747,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G807"/>
+  <dimension ref="A1:G819"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -34768,6 +35293,282 @@
         </is>
       </c>
       <c r="C807" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="808">
+      <c r="A808" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B808" t="inlineStr">
+        <is>
+          <t>BJDX</t>
+        </is>
+      </c>
+      <c r="C808" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D808" t="n">
+        <v>1.04</v>
+      </c>
+      <c r="E808" t="n">
+        <v>0.91</v>
+      </c>
+      <c r="F808" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="G808" t="n">
+        <v>391</v>
+      </c>
+    </row>
+    <row r="809">
+      <c r="A809" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B809" t="inlineStr">
+        <is>
+          <t>BNC</t>
+        </is>
+      </c>
+      <c r="C809" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D809" t="n">
+        <v>5.39</v>
+      </c>
+      <c r="E809" t="n">
+        <v>4.51</v>
+      </c>
+      <c r="F809" t="n">
+        <v>7.15</v>
+      </c>
+      <c r="G809" t="n">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="810">
+      <c r="A810" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B810" t="inlineStr">
+        <is>
+          <t>EAF</t>
+        </is>
+      </c>
+      <c r="C810" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D810" t="n">
+        <v>7.47</v>
+      </c>
+      <c r="E810" t="n">
+        <v>6.27</v>
+      </c>
+      <c r="F810" t="n">
+        <v>9.869999999999999</v>
+      </c>
+      <c r="G810" t="n">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="811">
+      <c r="A811" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B811" t="inlineStr">
+        <is>
+          <t>ISPC</t>
+        </is>
+      </c>
+      <c r="C811" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D811" t="n">
+        <v>1.94</v>
+      </c>
+      <c r="E811" t="n">
+        <v>1.55</v>
+      </c>
+      <c r="F811" t="n">
+        <v>2.72</v>
+      </c>
+      <c r="G811" t="n">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="812">
+      <c r="A812" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B812" t="inlineStr">
+        <is>
+          <t>MOBX</t>
+        </is>
+      </c>
+      <c r="C812" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D812" t="n">
+        <v>1.19</v>
+      </c>
+      <c r="E812" t="n">
+        <v>1.11</v>
+      </c>
+      <c r="F812" t="n">
+        <v>1.35</v>
+      </c>
+      <c r="G812" t="n">
+        <v>624</v>
+      </c>
+    </row>
+    <row r="813">
+      <c r="A813" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B813" t="inlineStr">
+        <is>
+          <t>PDSB</t>
+        </is>
+      </c>
+      <c r="C813" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D813" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="E813" t="n">
+        <v>0.26</v>
+      </c>
+      <c r="F813" t="n">
+        <v>1.44</v>
+      </c>
+      <c r="G813" t="n">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="814">
+      <c r="A814" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B814" t="inlineStr">
+        <is>
+          <t>AOUT</t>
+        </is>
+      </c>
+      <c r="C814" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="815">
+      <c r="A815" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B815" t="inlineStr">
+        <is>
+          <t>BBCP</t>
+        </is>
+      </c>
+      <c r="C815" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="816">
+      <c r="A816" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B816" t="inlineStr">
+        <is>
+          <t>CURV</t>
+        </is>
+      </c>
+      <c r="C816" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="817">
+      <c r="A817" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B817" t="inlineStr">
+        <is>
+          <t>IOT</t>
+        </is>
+      </c>
+      <c r="C817" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="818">
+      <c r="A818" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B818" t="inlineStr">
+        <is>
+          <t>MTEX</t>
+        </is>
+      </c>
+      <c r="C818" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="819">
+      <c r="A819" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B819" t="inlineStr">
+        <is>
+          <t>SWBI</t>
+        </is>
+      </c>
+      <c r="C819" t="inlineStr">
         <is>
           <t>Dropped</t>
         </is>

</xml_diff>

<commit_message>
Daily screener update: 2026-09-09
</commit_message>
<xml_diff>
--- a/screener_history.xlsx
+++ b/screener_history.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G706"/>
+  <dimension ref="A1:G731"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -16731,6 +16731,575 @@
         </is>
       </c>
       <c r="C706" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="707">
+      <c r="A707" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B707" t="inlineStr">
+        <is>
+          <t>ADIL</t>
+        </is>
+      </c>
+      <c r="C707" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D707" t="n">
+        <v>7.2</v>
+      </c>
+      <c r="E707" t="n">
+        <v>5.3</v>
+      </c>
+      <c r="F707" t="n">
+        <v>11</v>
+      </c>
+      <c r="G707" t="n">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="708">
+      <c r="A708" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B708" t="inlineStr">
+        <is>
+          <t>ARCT</t>
+        </is>
+      </c>
+      <c r="C708" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D708" t="n">
+        <v>17.75</v>
+      </c>
+      <c r="E708" t="n">
+        <v>14</v>
+      </c>
+      <c r="F708" t="n">
+        <v>25.25</v>
+      </c>
+      <c r="G708" t="n">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="709">
+      <c r="A709" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B709" t="inlineStr">
+        <is>
+          <t>DAIC</t>
+        </is>
+      </c>
+      <c r="C709" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D709" t="n">
+        <v>6.69</v>
+      </c>
+      <c r="E709" t="n">
+        <v>2.78</v>
+      </c>
+      <c r="F709" t="n">
+        <v>14.51</v>
+      </c>
+      <c r="G709" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="710">
+      <c r="A710" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B710" t="inlineStr">
+        <is>
+          <t>FIRY</t>
+        </is>
+      </c>
+      <c r="C710" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D710" t="n">
+        <v>10.4</v>
+      </c>
+      <c r="E710" t="n">
+        <v>9.52</v>
+      </c>
+      <c r="F710" t="n">
+        <v>12.16</v>
+      </c>
+      <c r="G710" t="n">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="711">
+      <c r="A711" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B711" t="inlineStr">
+        <is>
+          <t>FORR</t>
+        </is>
+      </c>
+      <c r="C711" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D711" t="n">
+        <v>12.75</v>
+      </c>
+      <c r="E711" t="n">
+        <v>11.69</v>
+      </c>
+      <c r="F711" t="n">
+        <v>14.87</v>
+      </c>
+      <c r="G711" t="n">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="712">
+      <c r="A712" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B712" t="inlineStr">
+        <is>
+          <t>HOWL</t>
+        </is>
+      </c>
+      <c r="C712" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D712" t="n">
+        <v>1.05</v>
+      </c>
+      <c r="E712" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="F712" t="n">
+        <v>1.35</v>
+      </c>
+      <c r="G712" t="n">
+        <v>328</v>
+      </c>
+    </row>
+    <row r="713">
+      <c r="A713" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B713" t="inlineStr">
+        <is>
+          <t>HWH</t>
+        </is>
+      </c>
+      <c r="C713" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D713" t="n">
+        <v>2.02</v>
+      </c>
+      <c r="E713" t="n">
+        <v>1.72</v>
+      </c>
+      <c r="F713" t="n">
+        <v>2.62</v>
+      </c>
+      <c r="G713" t="n">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="714">
+      <c r="A714" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B714" t="inlineStr">
+        <is>
+          <t>HZO</t>
+        </is>
+      </c>
+      <c r="C714" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D714" t="n">
+        <v>52.28</v>
+      </c>
+      <c r="E714" t="n">
+        <v>52.08</v>
+      </c>
+      <c r="F714" t="n">
+        <v>52.68</v>
+      </c>
+      <c r="G714" t="n">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="715">
+      <c r="A715" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B715" t="inlineStr">
+        <is>
+          <t>INO</t>
+        </is>
+      </c>
+      <c r="C715" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D715" t="n">
+        <v>1.45</v>
+      </c>
+      <c r="E715" t="n">
+        <v>1.22</v>
+      </c>
+      <c r="F715" t="n">
+        <v>1.91</v>
+      </c>
+      <c r="G715" t="n">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="716">
+      <c r="A716" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B716" t="inlineStr">
+        <is>
+          <t>PMTS</t>
+        </is>
+      </c>
+      <c r="C716" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D716" t="n">
+        <v>29.57</v>
+      </c>
+      <c r="E716" t="n">
+        <v>27.56</v>
+      </c>
+      <c r="F716" t="n">
+        <v>33.58</v>
+      </c>
+      <c r="G716" t="n">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="717">
+      <c r="A717" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B717" t="inlineStr">
+        <is>
+          <t>PURR</t>
+        </is>
+      </c>
+      <c r="C717" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D717" t="n">
+        <v>14.14</v>
+      </c>
+      <c r="E717" t="n">
+        <v>10.93</v>
+      </c>
+      <c r="F717" t="n">
+        <v>20.56</v>
+      </c>
+      <c r="G717" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="718">
+      <c r="A718" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B718" t="inlineStr">
+        <is>
+          <t>TKNO</t>
+        </is>
+      </c>
+      <c r="C718" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D718" t="n">
+        <v>7.64</v>
+      </c>
+      <c r="E718" t="n">
+        <v>6.77</v>
+      </c>
+      <c r="F718" t="n">
+        <v>9.390000000000001</v>
+      </c>
+      <c r="G718" t="n">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="719">
+      <c r="A719" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B719" t="inlineStr">
+        <is>
+          <t>ANRO</t>
+        </is>
+      </c>
+      <c r="C719" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="720">
+      <c r="A720" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B720" t="inlineStr">
+        <is>
+          <t>AVAH</t>
+        </is>
+      </c>
+      <c r="C720" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="721">
+      <c r="A721" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B721" t="inlineStr">
+        <is>
+          <t>CADL</t>
+        </is>
+      </c>
+      <c r="C721" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="722">
+      <c r="A722" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B722" t="inlineStr">
+        <is>
+          <t>ELF</t>
+        </is>
+      </c>
+      <c r="C722" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="723">
+      <c r="A723" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B723" t="inlineStr">
+        <is>
+          <t>LNSR</t>
+        </is>
+      </c>
+      <c r="C723" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="724">
+      <c r="A724" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B724" t="inlineStr">
+        <is>
+          <t>NVCT</t>
+        </is>
+      </c>
+      <c r="C724" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="725">
+      <c r="A725" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B725" t="inlineStr">
+        <is>
+          <t>OABI</t>
+        </is>
+      </c>
+      <c r="C725" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="726">
+      <c r="A726" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B726" t="inlineStr">
+        <is>
+          <t>PLSE</t>
+        </is>
+      </c>
+      <c r="C726" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="727">
+      <c r="A727" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B727" t="inlineStr">
+        <is>
+          <t>RCMT</t>
+        </is>
+      </c>
+      <c r="C727" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="728">
+      <c r="A728" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B728" t="inlineStr">
+        <is>
+          <t>SENS</t>
+        </is>
+      </c>
+      <c r="C728" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="729">
+      <c r="A729" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B729" t="inlineStr">
+        <is>
+          <t>STIM</t>
+        </is>
+      </c>
+      <c r="C729" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="730">
+      <c r="A730" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B730" t="inlineStr">
+        <is>
+          <t>TMCI</t>
+        </is>
+      </c>
+      <c r="C730" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="731">
+      <c r="A731" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B731" t="inlineStr">
+        <is>
+          <t>ZSTK</t>
+        </is>
+      </c>
+      <c r="C731" t="inlineStr">
         <is>
           <t>Dropped</t>
         </is>
@@ -16747,7 +17316,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G819"/>
+  <dimension ref="A1:G831"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -35569,6 +36138,282 @@
         </is>
       </c>
       <c r="C819" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="820">
+      <c r="A820" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B820" t="inlineStr">
+        <is>
+          <t>BIAF</t>
+        </is>
+      </c>
+      <c r="C820" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D820" t="n">
+        <v>12.21</v>
+      </c>
+      <c r="E820" t="n">
+        <v>10.09</v>
+      </c>
+      <c r="F820" t="n">
+        <v>16.45</v>
+      </c>
+      <c r="G820" t="n">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="821">
+      <c r="A821" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B821" t="inlineStr">
+        <is>
+          <t>INNV</t>
+        </is>
+      </c>
+      <c r="C821" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D821" t="n">
+        <v>11.7</v>
+      </c>
+      <c r="E821" t="n">
+        <v>10.93</v>
+      </c>
+      <c r="F821" t="n">
+        <v>13.24</v>
+      </c>
+      <c r="G821" t="n">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="822">
+      <c r="A822" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B822" t="inlineStr">
+        <is>
+          <t>IRD</t>
+        </is>
+      </c>
+      <c r="C822" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D822" t="n">
+        <v>6.55</v>
+      </c>
+      <c r="E822" t="n">
+        <v>5.32</v>
+      </c>
+      <c r="F822" t="n">
+        <v>9.01</v>
+      </c>
+      <c r="G822" t="n">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="823">
+      <c r="A823" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B823" t="inlineStr">
+        <is>
+          <t>JILL</t>
+        </is>
+      </c>
+      <c r="C823" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D823" t="n">
+        <v>23.48</v>
+      </c>
+      <c r="E823" t="n">
+        <v>20.89</v>
+      </c>
+      <c r="F823" t="n">
+        <v>28.65</v>
+      </c>
+      <c r="G823" t="n">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="824">
+      <c r="A824" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B824" t="inlineStr">
+        <is>
+          <t>OLB</t>
+        </is>
+      </c>
+      <c r="C824" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D824" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="E824" t="n">
+        <v>0.31</v>
+      </c>
+      <c r="F824" t="n">
+        <v>0.59</v>
+      </c>
+      <c r="G824" t="n">
+        <v>535</v>
+      </c>
+    </row>
+    <row r="825">
+      <c r="A825" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B825" t="inlineStr">
+        <is>
+          <t>SUNE</t>
+        </is>
+      </c>
+      <c r="C825" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D825" t="n">
+        <v>3.07</v>
+      </c>
+      <c r="E825" t="n">
+        <v>2.93</v>
+      </c>
+      <c r="F825" t="n">
+        <v>3.35</v>
+      </c>
+      <c r="G825" t="n">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="826">
+      <c r="A826" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B826" t="inlineStr">
+        <is>
+          <t>BJDX</t>
+        </is>
+      </c>
+      <c r="C826" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="827">
+      <c r="A827" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B827" t="inlineStr">
+        <is>
+          <t>BNC</t>
+        </is>
+      </c>
+      <c r="C827" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="828">
+      <c r="A828" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B828" t="inlineStr">
+        <is>
+          <t>EAF</t>
+        </is>
+      </c>
+      <c r="C828" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="829">
+      <c r="A829" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B829" t="inlineStr">
+        <is>
+          <t>ISPC</t>
+        </is>
+      </c>
+      <c r="C829" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="830">
+      <c r="A830" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B830" t="inlineStr">
+        <is>
+          <t>MOBX</t>
+        </is>
+      </c>
+      <c r="C830" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="831">
+      <c r="A831" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B831" t="inlineStr">
+        <is>
+          <t>PDSB</t>
+        </is>
+      </c>
+      <c r="C831" t="inlineStr">
         <is>
           <t>Dropped</t>
         </is>
@@ -35585,7 +36430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G27"/>
+  <dimension ref="A1:G28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -36223,6 +37068,35 @@
         </is>
       </c>
     </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>LRHC</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D28" t="n">
+        <v>2.82</v>
+      </c>
+      <c r="E28" t="n">
+        <v>2.93</v>
+      </c>
+      <c r="F28" t="n">
+        <v>2.6</v>
+      </c>
+      <c r="G28" t="n">
+        <v>454</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily screener update: 2026-09-10
</commit_message>
<xml_diff>
--- a/screener_history.xlsx
+++ b/screener_history.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G731"/>
+  <dimension ref="A1:G761"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -17300,6 +17300,708 @@
         </is>
       </c>
       <c r="C731" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="732">
+      <c r="A732" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B732" t="inlineStr">
+        <is>
+          <t>AMR</t>
+        </is>
+      </c>
+      <c r="C732" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D732" t="n">
+        <v>242.5</v>
+      </c>
+      <c r="E732" t="n">
+        <v>212.21</v>
+      </c>
+      <c r="F732" t="n">
+        <v>303.08</v>
+      </c>
+      <c r="G732" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="733">
+      <c r="A733" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B733" t="inlineStr">
+        <is>
+          <t>ANDG</t>
+        </is>
+      </c>
+      <c r="C733" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D733" t="n">
+        <v>57.62</v>
+      </c>
+      <c r="E733" t="n">
+        <v>52.9</v>
+      </c>
+      <c r="F733" t="n">
+        <v>67.06999999999999</v>
+      </c>
+      <c r="G733" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="734">
+      <c r="A734" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B734" t="inlineStr">
+        <is>
+          <t>ANF</t>
+        </is>
+      </c>
+      <c r="C734" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D734" t="n">
+        <v>155.22</v>
+      </c>
+      <c r="E734" t="n">
+        <v>136.17</v>
+      </c>
+      <c r="F734" t="n">
+        <v>193.32</v>
+      </c>
+      <c r="G734" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="735">
+      <c r="A735" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B735" t="inlineStr">
+        <is>
+          <t>CHYM</t>
+        </is>
+      </c>
+      <c r="C735" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D735" t="n">
+        <v>35.55</v>
+      </c>
+      <c r="E735" t="n">
+        <v>31.52</v>
+      </c>
+      <c r="F735" t="n">
+        <v>43.61</v>
+      </c>
+      <c r="G735" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="736">
+      <c r="A736" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B736" t="inlineStr">
+        <is>
+          <t>DFDV</t>
+        </is>
+      </c>
+      <c r="C736" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D736" t="n">
+        <v>6.21</v>
+      </c>
+      <c r="E736" t="n">
+        <v>4.8</v>
+      </c>
+      <c r="F736" t="n">
+        <v>9.029999999999999</v>
+      </c>
+      <c r="G736" t="n">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="737">
+      <c r="A737" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B737" t="inlineStr">
+        <is>
+          <t>FRD</t>
+        </is>
+      </c>
+      <c r="C737" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D737" t="n">
+        <v>46.49</v>
+      </c>
+      <c r="E737" t="n">
+        <v>42.47</v>
+      </c>
+      <c r="F737" t="n">
+        <v>54.53</v>
+      </c>
+      <c r="G737" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="738">
+      <c r="A738" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B738" t="inlineStr">
+        <is>
+          <t>IOVA</t>
+        </is>
+      </c>
+      <c r="C738" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D738" t="n">
+        <v>8.91</v>
+      </c>
+      <c r="E738" t="n">
+        <v>7.66</v>
+      </c>
+      <c r="F738" t="n">
+        <v>11.41</v>
+      </c>
+      <c r="G738" t="n">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="739">
+      <c r="A739" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B739" t="inlineStr">
+        <is>
+          <t>NEOV</t>
+        </is>
+      </c>
+      <c r="C739" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D739" t="n">
+        <v>4.35</v>
+      </c>
+      <c r="E739" t="n">
+        <v>3.33</v>
+      </c>
+      <c r="F739" t="n">
+        <v>6.39</v>
+      </c>
+      <c r="G739" t="n">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="740">
+      <c r="A740" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B740" t="inlineStr">
+        <is>
+          <t>NXPL</t>
+        </is>
+      </c>
+      <c r="C740" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D740" t="n">
+        <v>9.94</v>
+      </c>
+      <c r="E740" t="n">
+        <v>8.699999999999999</v>
+      </c>
+      <c r="F740" t="n">
+        <v>12.42</v>
+      </c>
+      <c r="G740" t="n">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="741">
+      <c r="A741" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B741" t="inlineStr">
+        <is>
+          <t>OMER</t>
+        </is>
+      </c>
+      <c r="C741" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D741" t="n">
+        <v>19.62</v>
+      </c>
+      <c r="E741" t="n">
+        <v>18</v>
+      </c>
+      <c r="F741" t="n">
+        <v>22.86</v>
+      </c>
+      <c r="G741" t="n">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="742">
+      <c r="A742" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B742" t="inlineStr">
+        <is>
+          <t>PEPG</t>
+        </is>
+      </c>
+      <c r="C742" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D742" t="n">
+        <v>3.48</v>
+      </c>
+      <c r="E742" t="n">
+        <v>2.91</v>
+      </c>
+      <c r="F742" t="n">
+        <v>4.62</v>
+      </c>
+      <c r="G742" t="n">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="743">
+      <c r="A743" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B743" t="inlineStr">
+        <is>
+          <t>PESI</t>
+        </is>
+      </c>
+      <c r="C743" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D743" t="n">
+        <v>19.49</v>
+      </c>
+      <c r="E743" t="n">
+        <v>17.64</v>
+      </c>
+      <c r="F743" t="n">
+        <v>23.19</v>
+      </c>
+      <c r="G743" t="n">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="744">
+      <c r="A744" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B744" t="inlineStr">
+        <is>
+          <t>QMCO</t>
+        </is>
+      </c>
+      <c r="C744" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D744" t="n">
+        <v>25.75</v>
+      </c>
+      <c r="E744" t="n">
+        <v>21.41</v>
+      </c>
+      <c r="F744" t="n">
+        <v>34.43</v>
+      </c>
+      <c r="G744" t="n">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="745">
+      <c r="A745" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B745" t="inlineStr">
+        <is>
+          <t>SLS</t>
+        </is>
+      </c>
+      <c r="C745" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D745" t="n">
+        <v>15.56</v>
+      </c>
+      <c r="E745" t="n">
+        <v>12.64</v>
+      </c>
+      <c r="F745" t="n">
+        <v>21.4</v>
+      </c>
+      <c r="G745" t="n">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="746">
+      <c r="A746" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B746" t="inlineStr">
+        <is>
+          <t>VIA</t>
+        </is>
+      </c>
+      <c r="C746" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D746" t="n">
+        <v>29.11</v>
+      </c>
+      <c r="E746" t="n">
+        <v>25.68</v>
+      </c>
+      <c r="F746" t="n">
+        <v>35.97</v>
+      </c>
+      <c r="G746" t="n">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="747">
+      <c r="A747" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B747" t="inlineStr">
+        <is>
+          <t>ZSTK</t>
+        </is>
+      </c>
+      <c r="C747" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D747" t="n">
+        <v>6.8</v>
+      </c>
+      <c r="E747" t="n">
+        <v>4.01</v>
+      </c>
+      <c r="F747" t="n">
+        <v>12.37</v>
+      </c>
+      <c r="G747" t="n">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="748">
+      <c r="A748" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B748" t="inlineStr">
+        <is>
+          <t>ADIL</t>
+        </is>
+      </c>
+      <c r="C748" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="749">
+      <c r="A749" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B749" t="inlineStr">
+        <is>
+          <t>AIFA</t>
+        </is>
+      </c>
+      <c r="C749" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="750">
+      <c r="A750" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B750" t="inlineStr">
+        <is>
+          <t>AMLX</t>
+        </is>
+      </c>
+      <c r="C750" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="751">
+      <c r="A751" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B751" t="inlineStr">
+        <is>
+          <t>BIVI</t>
+        </is>
+      </c>
+      <c r="C751" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="752">
+      <c r="A752" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B752" t="inlineStr">
+        <is>
+          <t>BOXL</t>
+        </is>
+      </c>
+      <c r="C752" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="753">
+      <c r="A753" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B753" t="inlineStr">
+        <is>
+          <t>BWMN</t>
+        </is>
+      </c>
+      <c r="C753" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="754">
+      <c r="A754" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B754" t="inlineStr">
+        <is>
+          <t>FIRY</t>
+        </is>
+      </c>
+      <c r="C754" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="755">
+      <c r="A755" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B755" t="inlineStr">
+        <is>
+          <t>FORR</t>
+        </is>
+      </c>
+      <c r="C755" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="756">
+      <c r="A756" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B756" t="inlineStr">
+        <is>
+          <t>HOWL</t>
+        </is>
+      </c>
+      <c r="C756" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="757">
+      <c r="A757" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B757" t="inlineStr">
+        <is>
+          <t>HWH</t>
+        </is>
+      </c>
+      <c r="C757" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="758">
+      <c r="A758" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B758" t="inlineStr">
+        <is>
+          <t>HZO</t>
+        </is>
+      </c>
+      <c r="C758" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="759">
+      <c r="A759" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B759" t="inlineStr">
+        <is>
+          <t>PMTS</t>
+        </is>
+      </c>
+      <c r="C759" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="760">
+      <c r="A760" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B760" t="inlineStr">
+        <is>
+          <t>TKNO</t>
+        </is>
+      </c>
+      <c r="C760" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="761">
+      <c r="A761" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B761" t="inlineStr">
+        <is>
+          <t>UTZ</t>
+        </is>
+      </c>
+      <c r="C761" t="inlineStr">
         <is>
           <t>Dropped</t>
         </is>
@@ -17316,7 +18018,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G831"/>
+  <dimension ref="A1:G842"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -36414,6 +37116,253 @@
         </is>
       </c>
       <c r="C831" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="832">
+      <c r="A832" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B832" t="inlineStr">
+        <is>
+          <t>CMRC</t>
+        </is>
+      </c>
+      <c r="C832" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D832" t="n">
+        <v>3.03</v>
+      </c>
+      <c r="E832" t="n">
+        <v>2.82</v>
+      </c>
+      <c r="F832" t="n">
+        <v>3.45</v>
+      </c>
+      <c r="G832" t="n">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="833">
+      <c r="A833" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B833" t="inlineStr">
+        <is>
+          <t>IPDN</t>
+        </is>
+      </c>
+      <c r="C833" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D833" t="n">
+        <v>0.18</v>
+      </c>
+      <c r="E833" t="n">
+        <v>0.14</v>
+      </c>
+      <c r="F833" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="G833" t="n">
+        <v>1052</v>
+      </c>
+    </row>
+    <row r="834">
+      <c r="A834" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B834" t="inlineStr">
+        <is>
+          <t>SKYQ</t>
+        </is>
+      </c>
+      <c r="C834" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D834" t="n">
+        <v>3.25</v>
+      </c>
+      <c r="E834" t="n">
+        <v>2.98</v>
+      </c>
+      <c r="F834" t="n">
+        <v>3.79</v>
+      </c>
+      <c r="G834" t="n">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="835">
+      <c r="A835" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B835" t="inlineStr">
+        <is>
+          <t>SNYR</t>
+        </is>
+      </c>
+      <c r="C835" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D835" t="n">
+        <v>0.13</v>
+      </c>
+      <c r="E835" t="n">
+        <v>0.09</v>
+      </c>
+      <c r="F835" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="G835" t="n">
+        <v>1436</v>
+      </c>
+    </row>
+    <row r="836">
+      <c r="A836" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B836" t="inlineStr">
+        <is>
+          <t>TNON</t>
+        </is>
+      </c>
+      <c r="C836" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D836" t="n">
+        <v>4.89</v>
+      </c>
+      <c r="E836" t="n">
+        <v>3.96</v>
+      </c>
+      <c r="F836" t="n">
+        <v>6.75</v>
+      </c>
+      <c r="G836" t="n">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="837">
+      <c r="A837" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B837" t="inlineStr">
+        <is>
+          <t>BIAF</t>
+        </is>
+      </c>
+      <c r="C837" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="838">
+      <c r="A838" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B838" t="inlineStr">
+        <is>
+          <t>INNV</t>
+        </is>
+      </c>
+      <c r="C838" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="839">
+      <c r="A839" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B839" t="inlineStr">
+        <is>
+          <t>IRD</t>
+        </is>
+      </c>
+      <c r="C839" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="840">
+      <c r="A840" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B840" t="inlineStr">
+        <is>
+          <t>JILL</t>
+        </is>
+      </c>
+      <c r="C840" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="841">
+      <c r="A841" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B841" t="inlineStr">
+        <is>
+          <t>OLB</t>
+        </is>
+      </c>
+      <c r="C841" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="842">
+      <c r="A842" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B842" t="inlineStr">
+        <is>
+          <t>SUNE</t>
+        </is>
+      </c>
+      <c r="C842" t="inlineStr">
         <is>
           <t>Dropped</t>
         </is>
@@ -36430,7 +37379,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G28"/>
+  <dimension ref="A1:G30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -37097,6 +38046,52 @@
         <v>454</v>
       </c>
     </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>BRTX</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D29" t="n">
+        <v>2.81</v>
+      </c>
+      <c r="E29" t="n">
+        <v>2.82</v>
+      </c>
+      <c r="F29" t="n">
+        <v>2.79</v>
+      </c>
+      <c r="G29" t="n">
+        <v>5000</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>LRHC</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily screener update: 2026-09-11
</commit_message>
<xml_diff>
--- a/screener_history.xlsx
+++ b/screener_history.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G761"/>
+  <dimension ref="A1:G790"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -18002,6 +18002,607 @@
         </is>
       </c>
       <c r="C761" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="762">
+      <c r="A762" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B762" t="inlineStr">
+        <is>
+          <t>BIVI</t>
+        </is>
+      </c>
+      <c r="C762" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D762" t="n">
+        <v>2.49</v>
+      </c>
+      <c r="E762" t="n">
+        <v>1.89</v>
+      </c>
+      <c r="F762" t="n">
+        <v>3.69</v>
+      </c>
+      <c r="G762" t="n">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="763">
+      <c r="A763" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B763" t="inlineStr">
+        <is>
+          <t>CELU</t>
+        </is>
+      </c>
+      <c r="C763" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D763" t="n">
+        <v>2.2</v>
+      </c>
+      <c r="E763" t="n">
+        <v>1.37</v>
+      </c>
+      <c r="F763" t="n">
+        <v>3.86</v>
+      </c>
+      <c r="G763" t="n">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="764">
+      <c r="A764" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B764" t="inlineStr">
+        <is>
+          <t>FIRY</t>
+        </is>
+      </c>
+      <c r="C764" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D764" t="n">
+        <v>10.2</v>
+      </c>
+      <c r="E764" t="n">
+        <v>9.5</v>
+      </c>
+      <c r="F764" t="n">
+        <v>11.6</v>
+      </c>
+      <c r="G764" t="n">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="765">
+      <c r="A765" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B765" t="inlineStr">
+        <is>
+          <t>GNLN</t>
+        </is>
+      </c>
+      <c r="C765" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D765" t="n">
+        <v>3.34</v>
+      </c>
+      <c r="E765" t="n">
+        <v>2.58</v>
+      </c>
+      <c r="F765" t="n">
+        <v>4.86</v>
+      </c>
+      <c r="G765" t="n">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="766">
+      <c r="A766" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B766" t="inlineStr">
+        <is>
+          <t>HOWL</t>
+        </is>
+      </c>
+      <c r="C766" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D766" t="n">
+        <v>1.03</v>
+      </c>
+      <c r="E766" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="F766" t="n">
+        <v>1.29</v>
+      </c>
+      <c r="G766" t="n">
+        <v>384</v>
+      </c>
+    </row>
+    <row r="767">
+      <c r="A767" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B767" t="inlineStr">
+        <is>
+          <t>PSNL</t>
+        </is>
+      </c>
+      <c r="C767" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D767" t="n">
+        <v>17.38</v>
+      </c>
+      <c r="E767" t="n">
+        <v>16</v>
+      </c>
+      <c r="F767" t="n">
+        <v>20.13</v>
+      </c>
+      <c r="G767" t="n">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="768">
+      <c r="A768" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B768" t="inlineStr">
+        <is>
+          <t>RCMT</t>
+        </is>
+      </c>
+      <c r="C768" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D768" t="n">
+        <v>43.09</v>
+      </c>
+      <c r="E768" t="n">
+        <v>38.93</v>
+      </c>
+      <c r="F768" t="n">
+        <v>51.41</v>
+      </c>
+      <c r="G768" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="769">
+      <c r="A769" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B769" t="inlineStr">
+        <is>
+          <t>TEAM</t>
+        </is>
+      </c>
+      <c r="C769" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D769" t="n">
+        <v>198.6</v>
+      </c>
+      <c r="E769" t="n">
+        <v>174.21</v>
+      </c>
+      <c r="F769" t="n">
+        <v>247.38</v>
+      </c>
+      <c r="G769" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="770">
+      <c r="A770" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B770" t="inlineStr">
+        <is>
+          <t>WEAV</t>
+        </is>
+      </c>
+      <c r="C770" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D770" t="n">
+        <v>7.36</v>
+      </c>
+      <c r="E770" t="n">
+        <v>7.29</v>
+      </c>
+      <c r="F770" t="n">
+        <v>7.5</v>
+      </c>
+      <c r="G770" t="n">
+        <v>714</v>
+      </c>
+    </row>
+    <row r="771">
+      <c r="A771" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B771" t="inlineStr">
+        <is>
+          <t>AMR</t>
+        </is>
+      </c>
+      <c r="C771" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="772">
+      <c r="A772" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B772" t="inlineStr">
+        <is>
+          <t>ANDG</t>
+        </is>
+      </c>
+      <c r="C772" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="773">
+      <c r="A773" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B773" t="inlineStr">
+        <is>
+          <t>ANF</t>
+        </is>
+      </c>
+      <c r="C773" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="774">
+      <c r="A774" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B774" t="inlineStr">
+        <is>
+          <t>ARCT</t>
+        </is>
+      </c>
+      <c r="C774" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="775">
+      <c r="A775" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B775" t="inlineStr">
+        <is>
+          <t>BOLD</t>
+        </is>
+      </c>
+      <c r="C775" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="776">
+      <c r="A776" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B776" t="inlineStr">
+        <is>
+          <t>CHYM</t>
+        </is>
+      </c>
+      <c r="C776" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="777">
+      <c r="A777" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B777" t="inlineStr">
+        <is>
+          <t>CRNX</t>
+        </is>
+      </c>
+      <c r="C777" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="778">
+      <c r="A778" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B778" t="inlineStr">
+        <is>
+          <t>DAIC</t>
+        </is>
+      </c>
+      <c r="C778" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="779">
+      <c r="A779" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B779" t="inlineStr">
+        <is>
+          <t>ETON</t>
+        </is>
+      </c>
+      <c r="C779" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="780">
+      <c r="A780" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B780" t="inlineStr">
+        <is>
+          <t>FRD</t>
+        </is>
+      </c>
+      <c r="C780" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="781">
+      <c r="A781" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B781" t="inlineStr">
+        <is>
+          <t>HTFL</t>
+        </is>
+      </c>
+      <c r="C781" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="782">
+      <c r="A782" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B782" t="inlineStr">
+        <is>
+          <t>IOVA</t>
+        </is>
+      </c>
+      <c r="C782" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="783">
+      <c r="A783" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B783" t="inlineStr">
+        <is>
+          <t>NEOV</t>
+        </is>
+      </c>
+      <c r="C783" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="784">
+      <c r="A784" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B784" t="inlineStr">
+        <is>
+          <t>NXPL</t>
+        </is>
+      </c>
+      <c r="C784" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="785">
+      <c r="A785" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B785" t="inlineStr">
+        <is>
+          <t>PEPG</t>
+        </is>
+      </c>
+      <c r="C785" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="786">
+      <c r="A786" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B786" t="inlineStr">
+        <is>
+          <t>PESI</t>
+        </is>
+      </c>
+      <c r="C786" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="787">
+      <c r="A787" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B787" t="inlineStr">
+        <is>
+          <t>QMCO</t>
+        </is>
+      </c>
+      <c r="C787" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="788">
+      <c r="A788" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B788" t="inlineStr">
+        <is>
+          <t>SGHT</t>
+        </is>
+      </c>
+      <c r="C788" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="789">
+      <c r="A789" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B789" t="inlineStr">
+        <is>
+          <t>SLS</t>
+        </is>
+      </c>
+      <c r="C789" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="790">
+      <c r="A790" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B790" t="inlineStr">
+        <is>
+          <t>VIA</t>
+        </is>
+      </c>
+      <c r="C790" t="inlineStr">
         <is>
           <t>Dropped</t>
         </is>
@@ -18018,7 +18619,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G842"/>
+  <dimension ref="A1:G852"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -37363,6 +37964,248 @@
         </is>
       </c>
       <c r="C842" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="843">
+      <c r="A843" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B843" t="inlineStr">
+        <is>
+          <t>ACVA</t>
+        </is>
+      </c>
+      <c r="C843" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D843" t="n">
+        <v>10.46</v>
+      </c>
+      <c r="E843" t="n">
+        <v>10.41</v>
+      </c>
+      <c r="F843" t="n">
+        <v>10.56</v>
+      </c>
+      <c r="G843" t="n">
+        <v>999</v>
+      </c>
+    </row>
+    <row r="844">
+      <c r="A844" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B844" t="inlineStr">
+        <is>
+          <t>AENT</t>
+        </is>
+      </c>
+      <c r="C844" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D844" t="n">
+        <v>7.62</v>
+      </c>
+      <c r="E844" t="n">
+        <v>6.14</v>
+      </c>
+      <c r="F844" t="n">
+        <v>10.58</v>
+      </c>
+      <c r="G844" t="n">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="845">
+      <c r="A845" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B845" t="inlineStr">
+        <is>
+          <t>FEIM</t>
+        </is>
+      </c>
+      <c r="C845" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D845" t="n">
+        <v>84.34999999999999</v>
+      </c>
+      <c r="E845" t="n">
+        <v>78.31999999999999</v>
+      </c>
+      <c r="F845" t="n">
+        <v>96.41</v>
+      </c>
+      <c r="G845" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="846">
+      <c r="A846" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B846" t="inlineStr">
+        <is>
+          <t>FTFT</t>
+        </is>
+      </c>
+      <c r="C846" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D846" t="n">
+        <v>3.35</v>
+      </c>
+      <c r="E846" t="n">
+        <v>2.66</v>
+      </c>
+      <c r="F846" t="n">
+        <v>4.73</v>
+      </c>
+      <c r="G846" t="n">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="847">
+      <c r="A847" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B847" t="inlineStr">
+        <is>
+          <t>SURG</t>
+        </is>
+      </c>
+      <c r="C847" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D847" t="n">
+        <v>0.21</v>
+      </c>
+      <c r="E847" t="n">
+        <v>0.17</v>
+      </c>
+      <c r="F847" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="G847" t="n">
+        <v>1424</v>
+      </c>
+    </row>
+    <row r="848">
+      <c r="A848" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B848" t="inlineStr">
+        <is>
+          <t>TRUG</t>
+        </is>
+      </c>
+      <c r="C848" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D848" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="E848" t="n">
+        <v>0.47</v>
+      </c>
+      <c r="F848" t="n">
+        <v>0.5600000000000001</v>
+      </c>
+      <c r="G848" t="n">
+        <v>1602</v>
+      </c>
+    </row>
+    <row r="849">
+      <c r="A849" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B849" t="inlineStr">
+        <is>
+          <t>CMRC</t>
+        </is>
+      </c>
+      <c r="C849" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="850">
+      <c r="A850" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B850" t="inlineStr">
+        <is>
+          <t>IPDN</t>
+        </is>
+      </c>
+      <c r="C850" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="851">
+      <c r="A851" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B851" t="inlineStr">
+        <is>
+          <t>SKYQ</t>
+        </is>
+      </c>
+      <c r="C851" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="852">
+      <c r="A852" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B852" t="inlineStr">
+        <is>
+          <t>SNYR</t>
+        </is>
+      </c>
+      <c r="C852" t="inlineStr">
         <is>
           <t>Dropped</t>
         </is>
@@ -37379,7 +38222,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G30"/>
+  <dimension ref="A1:G33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -38092,6 +38935,81 @@
         </is>
       </c>
     </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>CTSO</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D31" t="n">
+        <v>6.5</v>
+      </c>
+      <c r="E31" t="n">
+        <v>6.61</v>
+      </c>
+      <c r="F31" t="n">
+        <v>6.27</v>
+      </c>
+      <c r="G31" t="n">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>GTBP</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D32" t="n">
+        <v>6.59</v>
+      </c>
+      <c r="E32" t="n">
+        <v>8.82</v>
+      </c>
+      <c r="F32" t="n">
+        <v>2.13</v>
+      </c>
+      <c r="G32" t="n">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>BRTX</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily screener update: 2026-09-15
</commit_message>
<xml_diff>
--- a/screener_history.xlsx
+++ b/screener_history.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G790"/>
+  <dimension ref="A1:G813"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -18603,6 +18603,457 @@
         </is>
       </c>
       <c r="C790" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="791">
+      <c r="A791" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B791" t="inlineStr">
+        <is>
+          <t>AMLX</t>
+        </is>
+      </c>
+      <c r="C791" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D791" t="n">
+        <v>35.47</v>
+      </c>
+      <c r="E791" t="n">
+        <v>31.37</v>
+      </c>
+      <c r="F791" t="n">
+        <v>43.68</v>
+      </c>
+      <c r="G791" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="792">
+      <c r="A792" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B792" t="inlineStr">
+        <is>
+          <t>BMEA</t>
+        </is>
+      </c>
+      <c r="C792" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D792" t="n">
+        <v>2.07</v>
+      </c>
+      <c r="E792" t="n">
+        <v>1.66</v>
+      </c>
+      <c r="F792" t="n">
+        <v>2.89</v>
+      </c>
+      <c r="G792" t="n">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="793">
+      <c r="A793" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B793" t="inlineStr">
+        <is>
+          <t>BOLD</t>
+        </is>
+      </c>
+      <c r="C793" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D793" t="n">
+        <v>2.94</v>
+      </c>
+      <c r="E793" t="n">
+        <v>2.76</v>
+      </c>
+      <c r="F793" t="n">
+        <v>3.3</v>
+      </c>
+      <c r="G793" t="n">
+        <v>277</v>
+      </c>
+    </row>
+    <row r="794">
+      <c r="A794" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B794" t="inlineStr">
+        <is>
+          <t>CAPR</t>
+        </is>
+      </c>
+      <c r="C794" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D794" t="n">
+        <v>11</v>
+      </c>
+      <c r="E794" t="n">
+        <v>8.18</v>
+      </c>
+      <c r="F794" t="n">
+        <v>16.64</v>
+      </c>
+      <c r="G794" t="n">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="795">
+      <c r="A795" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B795" t="inlineStr">
+        <is>
+          <t>CJMB</t>
+        </is>
+      </c>
+      <c r="C795" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D795" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="E795" t="n">
+        <v>2</v>
+      </c>
+      <c r="F795" t="n">
+        <v>3.2</v>
+      </c>
+      <c r="G795" t="n">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="796">
+      <c r="A796" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B796" t="inlineStr">
+        <is>
+          <t>APGE</t>
+        </is>
+      </c>
+      <c r="C796" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="797">
+      <c r="A797" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B797" t="inlineStr">
+        <is>
+          <t>BIVI</t>
+        </is>
+      </c>
+      <c r="C797" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="798">
+      <c r="A798" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B798" t="inlineStr">
+        <is>
+          <t>DFDV</t>
+        </is>
+      </c>
+      <c r="C798" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="799">
+      <c r="A799" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B799" t="inlineStr">
+        <is>
+          <t>FIRY</t>
+        </is>
+      </c>
+      <c r="C799" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="800">
+      <c r="A800" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B800" t="inlineStr">
+        <is>
+          <t>GNLN</t>
+        </is>
+      </c>
+      <c r="C800" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="801">
+      <c r="A801" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B801" t="inlineStr">
+        <is>
+          <t>HHS</t>
+        </is>
+      </c>
+      <c r="C801" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="802">
+      <c r="A802" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B802" t="inlineStr">
+        <is>
+          <t>HOWL</t>
+        </is>
+      </c>
+      <c r="C802" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="803">
+      <c r="A803" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B803" t="inlineStr">
+        <is>
+          <t>INO</t>
+        </is>
+      </c>
+      <c r="C803" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="804">
+      <c r="A804" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B804" t="inlineStr">
+        <is>
+          <t>MRNA</t>
+        </is>
+      </c>
+      <c r="C804" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="805">
+      <c r="A805" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B805" t="inlineStr">
+        <is>
+          <t>OMER</t>
+        </is>
+      </c>
+      <c r="C805" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="806">
+      <c r="A806" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B806" t="inlineStr">
+        <is>
+          <t>PSNL</t>
+        </is>
+      </c>
+      <c r="C806" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="807">
+      <c r="A807" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B807" t="inlineStr">
+        <is>
+          <t>PURR</t>
+        </is>
+      </c>
+      <c r="C807" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="808">
+      <c r="A808" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B808" t="inlineStr">
+        <is>
+          <t>RCEL</t>
+        </is>
+      </c>
+      <c r="C808" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="809">
+      <c r="A809" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B809" t="inlineStr">
+        <is>
+          <t>RCMT</t>
+        </is>
+      </c>
+      <c r="C809" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="810">
+      <c r="A810" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B810" t="inlineStr">
+        <is>
+          <t>TEAM</t>
+        </is>
+      </c>
+      <c r="C810" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="811">
+      <c r="A811" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B811" t="inlineStr">
+        <is>
+          <t>VREX</t>
+        </is>
+      </c>
+      <c r="C811" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="812">
+      <c r="A812" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B812" t="inlineStr">
+        <is>
+          <t>WEAV</t>
+        </is>
+      </c>
+      <c r="C812" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="813">
+      <c r="A813" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B813" t="inlineStr">
+        <is>
+          <t>ZSTK</t>
+        </is>
+      </c>
+      <c r="C813" t="inlineStr">
         <is>
           <t>Dropped</t>
         </is>
@@ -18619,7 +19070,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G852"/>
+  <dimension ref="A1:G861"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -38206,6 +38657,195 @@
         </is>
       </c>
       <c r="C852" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="853">
+      <c r="A853" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B853" t="inlineStr">
+        <is>
+          <t>ELMT</t>
+        </is>
+      </c>
+      <c r="C853" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D853" t="n">
+        <v>23.11</v>
+      </c>
+      <c r="E853" t="n">
+        <v>20.22</v>
+      </c>
+      <c r="F853" t="n">
+        <v>28.89</v>
+      </c>
+      <c r="G853" t="n">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="854">
+      <c r="A854" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B854" t="inlineStr">
+        <is>
+          <t>OPENL</t>
+        </is>
+      </c>
+      <c r="C854" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D854" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="E854" t="n">
+        <v>0.09</v>
+      </c>
+      <c r="F854" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="G854" t="n">
+        <v>5000</v>
+      </c>
+    </row>
+    <row r="855">
+      <c r="A855" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B855" t="inlineStr">
+        <is>
+          <t>VNCE</t>
+        </is>
+      </c>
+      <c r="C855" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D855" t="n">
+        <v>6.68</v>
+      </c>
+      <c r="E855" t="n">
+        <v>5.53</v>
+      </c>
+      <c r="F855" t="n">
+        <v>8.98</v>
+      </c>
+      <c r="G855" t="n">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="856">
+      <c r="A856" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B856" t="inlineStr">
+        <is>
+          <t>ACVA</t>
+        </is>
+      </c>
+      <c r="C856" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="857">
+      <c r="A857" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B857" t="inlineStr">
+        <is>
+          <t>AENT</t>
+        </is>
+      </c>
+      <c r="C857" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="858">
+      <c r="A858" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B858" t="inlineStr">
+        <is>
+          <t>FEIM</t>
+        </is>
+      </c>
+      <c r="C858" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="859">
+      <c r="A859" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B859" t="inlineStr">
+        <is>
+          <t>SURG</t>
+        </is>
+      </c>
+      <c r="C859" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="860">
+      <c r="A860" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B860" t="inlineStr">
+        <is>
+          <t>TNON</t>
+        </is>
+      </c>
+      <c r="C860" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="861">
+      <c r="A861" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B861" t="inlineStr">
+        <is>
+          <t>TRUG</t>
+        </is>
+      </c>
+      <c r="C861" t="inlineStr">
         <is>
           <t>Dropped</t>
         </is>
@@ -38222,7 +38862,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G33"/>
+  <dimension ref="A1:G36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -39010,6 +39650,69 @@
         </is>
       </c>
     </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>ALP</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D34" t="n">
+        <v>4.16</v>
+      </c>
+      <c r="E34" t="n">
+        <v>4.39</v>
+      </c>
+      <c r="F34" t="n">
+        <v>3.72</v>
+      </c>
+      <c r="G34" t="n">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>CTSO</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>GTBP</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily screener update: 2026-09-16
</commit_message>
<xml_diff>
--- a/screener_history.xlsx
+++ b/screener_history.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G835"/>
+  <dimension ref="A1:G857"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -19644,6 +19644,476 @@
         </is>
       </c>
       <c r="C835" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="836">
+      <c r="A836" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B836" t="inlineStr">
+        <is>
+          <t>CAST</t>
+        </is>
+      </c>
+      <c r="C836" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D836" t="n">
+        <v>1.55</v>
+      </c>
+      <c r="E836" t="n">
+        <v>1.24</v>
+      </c>
+      <c r="F836" t="n">
+        <v>2.17</v>
+      </c>
+      <c r="G836" t="n">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="837">
+      <c r="A837" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B837" t="inlineStr">
+        <is>
+          <t>CJMB</t>
+        </is>
+      </c>
+      <c r="C837" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D837" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="E837" t="n">
+        <v>2</v>
+      </c>
+      <c r="F837" t="n">
+        <v>3.2</v>
+      </c>
+      <c r="G837" t="n">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="838">
+      <c r="A838" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B838" t="inlineStr">
+        <is>
+          <t>DH</t>
+        </is>
+      </c>
+      <c r="C838" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D838" t="n">
+        <v>1.22</v>
+      </c>
+      <c r="E838" t="n">
+        <v>0.96</v>
+      </c>
+      <c r="F838" t="n">
+        <v>1.74</v>
+      </c>
+      <c r="G838" t="n">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="839">
+      <c r="A839" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B839" t="inlineStr">
+        <is>
+          <t>GOAI</t>
+        </is>
+      </c>
+      <c r="C839" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D839" t="n">
+        <v>3.08</v>
+      </c>
+      <c r="E839" t="n">
+        <v>2.49</v>
+      </c>
+      <c r="F839" t="n">
+        <v>4.26</v>
+      </c>
+      <c r="G839" t="n">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="840">
+      <c r="A840" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B840" t="inlineStr">
+        <is>
+          <t>GPRO</t>
+        </is>
+      </c>
+      <c r="C840" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D840" t="n">
+        <v>2.05</v>
+      </c>
+      <c r="E840" t="n">
+        <v>1.18</v>
+      </c>
+      <c r="F840" t="n">
+        <v>3.79</v>
+      </c>
+      <c r="G840" t="n">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="841">
+      <c r="A841" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B841" t="inlineStr">
+        <is>
+          <t>MSTR</t>
+        </is>
+      </c>
+      <c r="C841" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D841" t="n">
+        <v>144.92</v>
+      </c>
+      <c r="E841" t="n">
+        <v>121.38</v>
+      </c>
+      <c r="F841" t="n">
+        <v>192</v>
+      </c>
+      <c r="G841" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="842">
+      <c r="A842" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B842" t="inlineStr">
+        <is>
+          <t>SID</t>
+        </is>
+      </c>
+      <c r="C842" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D842" t="n">
+        <v>1.38</v>
+      </c>
+      <c r="E842" t="n">
+        <v>1.14</v>
+      </c>
+      <c r="F842" t="n">
+        <v>1.86</v>
+      </c>
+      <c r="G842" t="n">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="843">
+      <c r="A843" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B843" t="inlineStr">
+        <is>
+          <t>VIA</t>
+        </is>
+      </c>
+      <c r="C843" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D843" t="n">
+        <v>28.76</v>
+      </c>
+      <c r="E843" t="n">
+        <v>25.41</v>
+      </c>
+      <c r="F843" t="n">
+        <v>35.46</v>
+      </c>
+      <c r="G843" t="n">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="844">
+      <c r="A844" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B844" t="inlineStr">
+        <is>
+          <t>ANDG</t>
+        </is>
+      </c>
+      <c r="C844" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="845">
+      <c r="A845" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B845" t="inlineStr">
+        <is>
+          <t>BB</t>
+        </is>
+      </c>
+      <c r="C845" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="846">
+      <c r="A846" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B846" t="inlineStr">
+        <is>
+          <t>BMEA</t>
+        </is>
+      </c>
+      <c r="C846" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="847">
+      <c r="A847" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B847" t="inlineStr">
+        <is>
+          <t>EMAT</t>
+        </is>
+      </c>
+      <c r="C847" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="848">
+      <c r="A848" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B848" t="inlineStr">
+        <is>
+          <t>FWDI</t>
+        </is>
+      </c>
+      <c r="C848" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="849">
+      <c r="A849" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B849" t="inlineStr">
+        <is>
+          <t>GNLN</t>
+        </is>
+      </c>
+      <c r="C849" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="850">
+      <c r="A850" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B850" t="inlineStr">
+        <is>
+          <t>HUM</t>
+        </is>
+      </c>
+      <c r="C850" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="851">
+      <c r="A851" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B851" t="inlineStr">
+        <is>
+          <t>QMCO</t>
+        </is>
+      </c>
+      <c r="C851" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="852">
+      <c r="A852" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B852" t="inlineStr">
+        <is>
+          <t>RCEL</t>
+        </is>
+      </c>
+      <c r="C852" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="853">
+      <c r="A853" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B853" t="inlineStr">
+        <is>
+          <t>RCMT</t>
+        </is>
+      </c>
+      <c r="C853" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="854">
+      <c r="A854" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B854" t="inlineStr">
+        <is>
+          <t>RDI</t>
+        </is>
+      </c>
+      <c r="C854" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="855">
+      <c r="A855" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B855" t="inlineStr">
+        <is>
+          <t>UPXI</t>
+        </is>
+      </c>
+      <c r="C855" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="856">
+      <c r="A856" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B856" t="inlineStr">
+        <is>
+          <t>XHLD</t>
+        </is>
+      </c>
+      <c r="C856" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="857">
+      <c r="A857" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B857" t="inlineStr">
+        <is>
+          <t>ZSTK</t>
+        </is>
+      </c>
+      <c r="C857" t="inlineStr">
         <is>
           <t>Dropped</t>
         </is>
@@ -19660,7 +20130,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G870"/>
+  <dimension ref="A1:G879"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -39649,6 +40119,219 @@
         </is>
       </c>
       <c r="C870" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="871">
+      <c r="A871" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B871" t="inlineStr">
+        <is>
+          <t>BENF</t>
+        </is>
+      </c>
+      <c r="C871" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D871" t="n">
+        <v>0.83</v>
+      </c>
+      <c r="E871" t="n">
+        <v>0.66</v>
+      </c>
+      <c r="F871" t="n">
+        <v>1.16</v>
+      </c>
+      <c r="G871" t="n">
+        <v>302</v>
+      </c>
+    </row>
+    <row r="872">
+      <c r="A872" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B872" t="inlineStr">
+        <is>
+          <t>CYPH</t>
+        </is>
+      </c>
+      <c r="C872" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D872" t="n">
+        <v>2.47</v>
+      </c>
+      <c r="E872" t="n">
+        <v>2.3</v>
+      </c>
+      <c r="F872" t="n">
+        <v>2.82</v>
+      </c>
+      <c r="G872" t="n">
+        <v>285</v>
+      </c>
+    </row>
+    <row r="873">
+      <c r="A873" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B873" t="inlineStr">
+        <is>
+          <t>SNYR</t>
+        </is>
+      </c>
+      <c r="C873" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D873" t="n">
+        <v>0.14</v>
+      </c>
+      <c r="E873" t="n">
+        <v>0.13</v>
+      </c>
+      <c r="F873" t="n">
+        <v>0.17</v>
+      </c>
+      <c r="G873" t="n">
+        <v>3424</v>
+      </c>
+    </row>
+    <row r="874">
+      <c r="A874" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B874" t="inlineStr">
+        <is>
+          <t>TPST</t>
+        </is>
+      </c>
+      <c r="C874" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D874" t="n">
+        <v>1.15</v>
+      </c>
+      <c r="E874" t="n">
+        <v>0.97</v>
+      </c>
+      <c r="F874" t="n">
+        <v>1.51</v>
+      </c>
+      <c r="G874" t="n">
+        <v>273</v>
+      </c>
+    </row>
+    <row r="875">
+      <c r="A875" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B875" t="inlineStr">
+        <is>
+          <t>VWAV</t>
+        </is>
+      </c>
+      <c r="C875" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D875" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="E875" t="n">
+        <v>0.36</v>
+      </c>
+      <c r="F875" t="n">
+        <v>1.08</v>
+      </c>
+      <c r="G875" t="n">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="876">
+      <c r="A876" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B876" t="inlineStr">
+        <is>
+          <t>MYSZ</t>
+        </is>
+      </c>
+      <c r="C876" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="877">
+      <c r="A877" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B877" t="inlineStr">
+        <is>
+          <t>TRUG</t>
+        </is>
+      </c>
+      <c r="C877" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="878">
+      <c r="A878" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B878" t="inlineStr">
+        <is>
+          <t>VEEA</t>
+        </is>
+      </c>
+      <c r="C878" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="879">
+      <c r="A879" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B879" t="inlineStr">
+        <is>
+          <t>VRA</t>
+        </is>
+      </c>
+      <c r="C879" t="inlineStr">
         <is>
           <t>Dropped</t>
         </is>
@@ -39665,7 +40348,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G38"/>
+  <dimension ref="A1:G39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -40562,6 +41245,23 @@
         </is>
       </c>
     </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>NFE</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily screener update: 2026-09-17
</commit_message>
<xml_diff>
--- a/screener_history.xlsx
+++ b/screener_history.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G857"/>
+  <dimension ref="A1:G874"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -20114,6 +20114,367 @@
         </is>
       </c>
       <c r="C857" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="858">
+      <c r="A858" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B858" t="inlineStr">
+        <is>
+          <t>FWDI</t>
+        </is>
+      </c>
+      <c r="C858" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D858" t="n">
+        <v>7.14</v>
+      </c>
+      <c r="E858" t="n">
+        <v>5.76</v>
+      </c>
+      <c r="F858" t="n">
+        <v>9.9</v>
+      </c>
+      <c r="G858" t="n">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="859">
+      <c r="A859" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B859" t="inlineStr">
+        <is>
+          <t>PLSE</t>
+        </is>
+      </c>
+      <c r="C859" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D859" t="n">
+        <v>58.9</v>
+      </c>
+      <c r="E859" t="n">
+        <v>47.7</v>
+      </c>
+      <c r="F859" t="n">
+        <v>81.3</v>
+      </c>
+      <c r="G859" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="860">
+      <c r="A860" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B860" t="inlineStr">
+        <is>
+          <t>RDIB</t>
+        </is>
+      </c>
+      <c r="C860" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D860" t="n">
+        <v>19.32</v>
+      </c>
+      <c r="E860" t="n">
+        <v>12.83</v>
+      </c>
+      <c r="F860" t="n">
+        <v>32.29</v>
+      </c>
+      <c r="G860" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="861">
+      <c r="A861" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B861" t="inlineStr">
+        <is>
+          <t>RNXT</t>
+        </is>
+      </c>
+      <c r="C861" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D861" t="n">
+        <v>2.54</v>
+      </c>
+      <c r="E861" t="n">
+        <v>1.55</v>
+      </c>
+      <c r="F861" t="n">
+        <v>4.52</v>
+      </c>
+      <c r="G861" t="n">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="862">
+      <c r="A862" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B862" t="inlineStr">
+        <is>
+          <t>VSTM</t>
+        </is>
+      </c>
+      <c r="C862" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D862" t="n">
+        <v>8.539999999999999</v>
+      </c>
+      <c r="E862" t="n">
+        <v>7.2</v>
+      </c>
+      <c r="F862" t="n">
+        <v>11.22</v>
+      </c>
+      <c r="G862" t="n">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="863">
+      <c r="A863" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B863" t="inlineStr">
+        <is>
+          <t>ZSTK</t>
+        </is>
+      </c>
+      <c r="C863" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D863" t="n">
+        <v>5.21</v>
+      </c>
+      <c r="E863" t="n">
+        <v>4.01</v>
+      </c>
+      <c r="F863" t="n">
+        <v>7.61</v>
+      </c>
+      <c r="G863" t="n">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="864">
+      <c r="A864" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B864" t="inlineStr">
+        <is>
+          <t>AMLX</t>
+        </is>
+      </c>
+      <c r="C864" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="865">
+      <c r="A865" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B865" t="inlineStr">
+        <is>
+          <t>CAST</t>
+        </is>
+      </c>
+      <c r="C865" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="866">
+      <c r="A866" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B866" t="inlineStr">
+        <is>
+          <t>CJMB</t>
+        </is>
+      </c>
+      <c r="C866" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="867">
+      <c r="A867" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B867" t="inlineStr">
+        <is>
+          <t>GOAI</t>
+        </is>
+      </c>
+      <c r="C867" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="868">
+      <c r="A868" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B868" t="inlineStr">
+        <is>
+          <t>MRNA</t>
+        </is>
+      </c>
+      <c r="C868" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="869">
+      <c r="A869" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B869" t="inlineStr">
+        <is>
+          <t>MSTR</t>
+        </is>
+      </c>
+      <c r="C869" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="870">
+      <c r="A870" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B870" t="inlineStr">
+        <is>
+          <t>PESI</t>
+        </is>
+      </c>
+      <c r="C870" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="871">
+      <c r="A871" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B871" t="inlineStr">
+        <is>
+          <t>PURR</t>
+        </is>
+      </c>
+      <c r="C871" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="872">
+      <c r="A872" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B872" t="inlineStr">
+        <is>
+          <t>SID</t>
+        </is>
+      </c>
+      <c r="C872" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="873">
+      <c r="A873" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B873" t="inlineStr">
+        <is>
+          <t>VIA</t>
+        </is>
+      </c>
+      <c r="C873" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="874">
+      <c r="A874" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B874" t="inlineStr">
+        <is>
+          <t>WEAV</t>
+        </is>
+      </c>
+      <c r="C874" t="inlineStr">
         <is>
           <t>Dropped</t>
         </is>
@@ -20130,7 +20491,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G879"/>
+  <dimension ref="A1:G897"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -40332,6 +40693,456 @@
         </is>
       </c>
       <c r="C879" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="880">
+      <c r="A880" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B880" t="inlineStr">
+        <is>
+          <t>AEMD</t>
+        </is>
+      </c>
+      <c r="C880" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D880" t="n">
+        <v>9.5</v>
+      </c>
+      <c r="E880" t="n">
+        <v>6.01</v>
+      </c>
+      <c r="F880" t="n">
+        <v>16.48</v>
+      </c>
+      <c r="G880" t="n">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="881">
+      <c r="A881" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B881" t="inlineStr">
+        <is>
+          <t>BIAF</t>
+        </is>
+      </c>
+      <c r="C881" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D881" t="n">
+        <v>7.41</v>
+      </c>
+      <c r="E881" t="n">
+        <v>6.45</v>
+      </c>
+      <c r="F881" t="n">
+        <v>9.32</v>
+      </c>
+      <c r="G881" t="n">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="882">
+      <c r="A882" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B882" t="inlineStr">
+        <is>
+          <t>CTNT</t>
+        </is>
+      </c>
+      <c r="C882" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D882" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="E882" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="F882" t="n">
+        <v>0.17</v>
+      </c>
+      <c r="G882" t="n">
+        <v>1196</v>
+      </c>
+    </row>
+    <row r="883">
+      <c r="A883" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B883" t="inlineStr">
+        <is>
+          <t>DAIC</t>
+        </is>
+      </c>
+      <c r="C883" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D883" t="n">
+        <v>4.75</v>
+      </c>
+      <c r="E883" t="n">
+        <v>3.98</v>
+      </c>
+      <c r="F883" t="n">
+        <v>6.29</v>
+      </c>
+      <c r="G883" t="n">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="884">
+      <c r="A884" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B884" t="inlineStr">
+        <is>
+          <t>GLOO</t>
+        </is>
+      </c>
+      <c r="C884" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D884" t="n">
+        <v>5</v>
+      </c>
+      <c r="E884" t="n">
+        <v>4.43</v>
+      </c>
+      <c r="F884" t="n">
+        <v>6.14</v>
+      </c>
+      <c r="G884" t="n">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="885">
+      <c r="A885" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B885" t="inlineStr">
+        <is>
+          <t>GNRC</t>
+        </is>
+      </c>
+      <c r="C885" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D885" t="n">
+        <v>231.89</v>
+      </c>
+      <c r="E885" t="n">
+        <v>202.26</v>
+      </c>
+      <c r="F885" t="n">
+        <v>291.14</v>
+      </c>
+      <c r="G885" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="886">
+      <c r="A886" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B886" t="inlineStr">
+        <is>
+          <t>LSTA</t>
+        </is>
+      </c>
+      <c r="C886" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D886" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="E886" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="F886" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="G886" t="n">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="887">
+      <c r="A887" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B887" t="inlineStr">
+        <is>
+          <t>MNOV</t>
+        </is>
+      </c>
+      <c r="C887" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D887" t="n">
+        <v>3.08</v>
+      </c>
+      <c r="E887" t="n">
+        <v>2.83</v>
+      </c>
+      <c r="F887" t="n">
+        <v>3.58</v>
+      </c>
+      <c r="G887" t="n">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="888">
+      <c r="A888" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B888" t="inlineStr">
+        <is>
+          <t>RTB</t>
+        </is>
+      </c>
+      <c r="C888" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D888" t="n">
+        <v>11.2</v>
+      </c>
+      <c r="E888" t="n">
+        <v>8.27</v>
+      </c>
+      <c r="F888" t="n">
+        <v>17.06</v>
+      </c>
+      <c r="G888" t="n">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="889">
+      <c r="A889" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B889" t="inlineStr">
+        <is>
+          <t>SDST</t>
+        </is>
+      </c>
+      <c r="C889" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D889" t="n">
+        <v>0.26</v>
+      </c>
+      <c r="E889" t="n">
+        <v>0.21</v>
+      </c>
+      <c r="F889" t="n">
+        <v>0.37</v>
+      </c>
+      <c r="G889" t="n">
+        <v>959</v>
+      </c>
+    </row>
+    <row r="890">
+      <c r="A890" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B890" t="inlineStr">
+        <is>
+          <t>SRFM</t>
+        </is>
+      </c>
+      <c r="C890" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D890" t="n">
+        <v>0.59</v>
+      </c>
+      <c r="E890" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="F890" t="n">
+        <v>0.6899999999999999</v>
+      </c>
+      <c r="G890" t="n">
+        <v>1051</v>
+      </c>
+    </row>
+    <row r="891">
+      <c r="A891" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B891" t="inlineStr">
+        <is>
+          <t>SURG</t>
+        </is>
+      </c>
+      <c r="C891" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D891" t="n">
+        <v>0.19</v>
+      </c>
+      <c r="E891" t="n">
+        <v>0.14</v>
+      </c>
+      <c r="F891" t="n">
+        <v>0.29</v>
+      </c>
+      <c r="G891" t="n">
+        <v>1006</v>
+      </c>
+    </row>
+    <row r="892">
+      <c r="A892" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B892" t="inlineStr">
+        <is>
+          <t>BENF</t>
+        </is>
+      </c>
+      <c r="C892" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="893">
+      <c r="A893" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B893" t="inlineStr">
+        <is>
+          <t>CYPH</t>
+        </is>
+      </c>
+      <c r="C893" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="894">
+      <c r="A894" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B894" t="inlineStr">
+        <is>
+          <t>PDSB</t>
+        </is>
+      </c>
+      <c r="C894" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="895">
+      <c r="A895" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B895" t="inlineStr">
+        <is>
+          <t>SNYR</t>
+        </is>
+      </c>
+      <c r="C895" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="896">
+      <c r="A896" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B896" t="inlineStr">
+        <is>
+          <t>TPST</t>
+        </is>
+      </c>
+      <c r="C896" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="897">
+      <c r="A897" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B897" t="inlineStr">
+        <is>
+          <t>VWAV</t>
+        </is>
+      </c>
+      <c r="C897" t="inlineStr">
         <is>
           <t>Dropped</t>
         </is>
@@ -40348,7 +41159,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G39"/>
+  <dimension ref="A1:G40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -41262,6 +42073,35 @@
         </is>
       </c>
     </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>NXXT</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D40" t="n">
+        <v>1.13</v>
+      </c>
+      <c r="E40" t="n">
+        <v>1.25</v>
+      </c>
+      <c r="F40" t="n">
+        <v>0.89</v>
+      </c>
+      <c r="G40" t="n">
+        <v>416</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily screener update: 2026-09-18
</commit_message>
<xml_diff>
--- a/screener_history.xlsx
+++ b/screener_history.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G874"/>
+  <dimension ref="A1:G881"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -20475,6 +20475,173 @@
         </is>
       </c>
       <c r="C874" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="875">
+      <c r="A875" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B875" t="inlineStr">
+        <is>
+          <t>AVAH</t>
+        </is>
+      </c>
+      <c r="C875" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D875" t="n">
+        <v>14.71</v>
+      </c>
+      <c r="E875" t="n">
+        <v>13.38</v>
+      </c>
+      <c r="F875" t="n">
+        <v>17.37</v>
+      </c>
+      <c r="G875" t="n">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="876">
+      <c r="A876" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B876" t="inlineStr">
+        <is>
+          <t>FATN</t>
+        </is>
+      </c>
+      <c r="C876" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D876" t="n">
+        <v>6.19</v>
+      </c>
+      <c r="E876" t="n">
+        <v>5.44</v>
+      </c>
+      <c r="F876" t="n">
+        <v>7.69</v>
+      </c>
+      <c r="G876" t="n">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="877">
+      <c r="A877" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B877" t="inlineStr">
+        <is>
+          <t>OSCR</t>
+        </is>
+      </c>
+      <c r="C877" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D877" t="n">
+        <v>34.48</v>
+      </c>
+      <c r="E877" t="n">
+        <v>30.44</v>
+      </c>
+      <c r="F877" t="n">
+        <v>42.56</v>
+      </c>
+      <c r="G877" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="878">
+      <c r="A878" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B878" t="inlineStr">
+        <is>
+          <t>UTZ</t>
+        </is>
+      </c>
+      <c r="C878" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D878" t="n">
+        <v>14.33</v>
+      </c>
+      <c r="E878" t="n">
+        <v>14.2</v>
+      </c>
+      <c r="F878" t="n">
+        <v>14.59</v>
+      </c>
+      <c r="G878" t="n">
+        <v>384</v>
+      </c>
+    </row>
+    <row r="879">
+      <c r="A879" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B879" t="inlineStr">
+        <is>
+          <t>FWDI</t>
+        </is>
+      </c>
+      <c r="C879" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="880">
+      <c r="A880" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B880" t="inlineStr">
+        <is>
+          <t>PLSE</t>
+        </is>
+      </c>
+      <c r="C880" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="881">
+      <c r="A881" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B881" t="inlineStr">
+        <is>
+          <t>RNXT</t>
+        </is>
+      </c>
+      <c r="C881" t="inlineStr">
         <is>
           <t>Dropped</t>
         </is>
@@ -20491,7 +20658,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G897"/>
+  <dimension ref="A1:G917"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -41143,6 +41310,454 @@
         </is>
       </c>
       <c r="C897" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="898">
+      <c r="A898" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B898" t="inlineStr">
+        <is>
+          <t>BENF</t>
+        </is>
+      </c>
+      <c r="C898" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D898" t="n">
+        <v>0.76</v>
+      </c>
+      <c r="E898" t="n">
+        <v>0.54</v>
+      </c>
+      <c r="F898" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="G898" t="n">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="899">
+      <c r="A899" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B899" t="inlineStr">
+        <is>
+          <t>DSP</t>
+        </is>
+      </c>
+      <c r="C899" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D899" t="n">
+        <v>11.95</v>
+      </c>
+      <c r="E899" t="n">
+        <v>11.23</v>
+      </c>
+      <c r="F899" t="n">
+        <v>13.39</v>
+      </c>
+      <c r="G899" t="n">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="900">
+      <c r="A900" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B900" t="inlineStr">
+        <is>
+          <t>FTCI</t>
+        </is>
+      </c>
+      <c r="C900" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D900" t="n">
+        <v>2.54</v>
+      </c>
+      <c r="E900" t="n">
+        <v>2.28</v>
+      </c>
+      <c r="F900" t="n">
+        <v>3.06</v>
+      </c>
+      <c r="G900" t="n">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="901">
+      <c r="A901" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B901" t="inlineStr">
+        <is>
+          <t>GIPR</t>
+        </is>
+      </c>
+      <c r="C901" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D901" t="n">
+        <v>1.56</v>
+      </c>
+      <c r="E901" t="n">
+        <v>0.67</v>
+      </c>
+      <c r="F901" t="n">
+        <v>3.33</v>
+      </c>
+      <c r="G901" t="n">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="902">
+      <c r="A902" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B902" t="inlineStr">
+        <is>
+          <t>NCPL</t>
+        </is>
+      </c>
+      <c r="C902" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D902" t="n">
+        <v>0.76</v>
+      </c>
+      <c r="E902" t="n">
+        <v>0.68</v>
+      </c>
+      <c r="F902" t="n">
+        <v>0.92</v>
+      </c>
+      <c r="G902" t="n">
+        <v>603</v>
+      </c>
+    </row>
+    <row r="903">
+      <c r="A903" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B903" t="inlineStr">
+        <is>
+          <t>SVRN</t>
+        </is>
+      </c>
+      <c r="C903" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D903" t="n">
+        <v>17.96</v>
+      </c>
+      <c r="E903" t="n">
+        <v>16.6</v>
+      </c>
+      <c r="F903" t="n">
+        <v>20.68</v>
+      </c>
+      <c r="G903" t="n">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="904">
+      <c r="A904" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B904" t="inlineStr">
+        <is>
+          <t>TRUG</t>
+        </is>
+      </c>
+      <c r="C904" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D904" t="n">
+        <v>0.52</v>
+      </c>
+      <c r="E904" t="n">
+        <v>0.46</v>
+      </c>
+      <c r="F904" t="n">
+        <v>0.64</v>
+      </c>
+      <c r="G904" t="n">
+        <v>806</v>
+      </c>
+    </row>
+    <row r="905">
+      <c r="A905" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B905" t="inlineStr">
+        <is>
+          <t>USDE</t>
+        </is>
+      </c>
+      <c r="C905" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D905" t="n">
+        <v>9.52</v>
+      </c>
+      <c r="E905" t="n">
+        <v>8.51</v>
+      </c>
+      <c r="F905" t="n">
+        <v>11.54</v>
+      </c>
+      <c r="G905" t="n">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="906">
+      <c r="A906" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B906" t="inlineStr">
+        <is>
+          <t>VRME</t>
+        </is>
+      </c>
+      <c r="C906" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D906" t="n">
+        <v>0.86</v>
+      </c>
+      <c r="E906" t="n">
+        <v>0.67</v>
+      </c>
+      <c r="F906" t="n">
+        <v>1.24</v>
+      </c>
+      <c r="G906" t="n">
+        <v>263</v>
+      </c>
+    </row>
+    <row r="907">
+      <c r="A907" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B907" t="inlineStr">
+        <is>
+          <t>AEMD</t>
+        </is>
+      </c>
+      <c r="C907" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="908">
+      <c r="A908" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B908" t="inlineStr">
+        <is>
+          <t>BIAF</t>
+        </is>
+      </c>
+      <c r="C908" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="909">
+      <c r="A909" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B909" t="inlineStr">
+        <is>
+          <t>DAIC</t>
+        </is>
+      </c>
+      <c r="C909" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="910">
+      <c r="A910" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B910" t="inlineStr">
+        <is>
+          <t>GLOO</t>
+        </is>
+      </c>
+      <c r="C910" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="911">
+      <c r="A911" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B911" t="inlineStr">
+        <is>
+          <t>GNRC</t>
+        </is>
+      </c>
+      <c r="C911" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="912">
+      <c r="A912" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B912" t="inlineStr">
+        <is>
+          <t>LSTA</t>
+        </is>
+      </c>
+      <c r="C912" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="913">
+      <c r="A913" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B913" t="inlineStr">
+        <is>
+          <t>MNOV</t>
+        </is>
+      </c>
+      <c r="C913" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="914">
+      <c r="A914" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B914" t="inlineStr">
+        <is>
+          <t>RTB</t>
+        </is>
+      </c>
+      <c r="C914" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="915">
+      <c r="A915" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B915" t="inlineStr">
+        <is>
+          <t>SDST</t>
+        </is>
+      </c>
+      <c r="C915" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="916">
+      <c r="A916" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B916" t="inlineStr">
+        <is>
+          <t>SRFM</t>
+        </is>
+      </c>
+      <c r="C916" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="917">
+      <c r="A917" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B917" t="inlineStr">
+        <is>
+          <t>SURG</t>
+        </is>
+      </c>
+      <c r="C917" t="inlineStr">
         <is>
           <t>Dropped</t>
         </is>
@@ -41159,7 +41774,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G40"/>
+  <dimension ref="A1:G41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -42102,6 +42717,23 @@
         <v>416</v>
       </c>
     </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>NXXT</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily screener update: 2026-09-22
</commit_message>
<xml_diff>
--- a/screener_history.xlsx
+++ b/screener_history.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G881"/>
+  <dimension ref="A1:G892"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -20642,6 +20642,205 @@
         </is>
       </c>
       <c r="C881" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="882">
+      <c r="A882" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="B882" t="inlineStr">
+        <is>
+          <t>BIO-B</t>
+        </is>
+      </c>
+      <c r="C882" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D882" t="n">
+        <v>365.08</v>
+      </c>
+      <c r="E882" t="n">
+        <v>365.08</v>
+      </c>
+      <c r="F882" t="n">
+        <v>365.08</v>
+      </c>
+      <c r="G882" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="883">
+      <c r="A883" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="B883" t="inlineStr">
+        <is>
+          <t>AVAH</t>
+        </is>
+      </c>
+      <c r="C883" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="884">
+      <c r="A884" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="B884" t="inlineStr">
+        <is>
+          <t>DH</t>
+        </is>
+      </c>
+      <c r="C884" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="885">
+      <c r="A885" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="B885" t="inlineStr">
+        <is>
+          <t>FATN</t>
+        </is>
+      </c>
+      <c r="C885" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="886">
+      <c r="A886" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="B886" t="inlineStr">
+        <is>
+          <t>GPRO</t>
+        </is>
+      </c>
+      <c r="C886" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="887">
+      <c r="A887" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="B887" t="inlineStr">
+        <is>
+          <t>HOWL</t>
+        </is>
+      </c>
+      <c r="C887" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="888">
+      <c r="A888" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="B888" t="inlineStr">
+        <is>
+          <t>OSCR</t>
+        </is>
+      </c>
+      <c r="C888" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="889">
+      <c r="A889" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="B889" t="inlineStr">
+        <is>
+          <t>RDIB</t>
+        </is>
+      </c>
+      <c r="C889" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="890">
+      <c r="A890" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="B890" t="inlineStr">
+        <is>
+          <t>UTZ</t>
+        </is>
+      </c>
+      <c r="C890" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="891">
+      <c r="A891" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="B891" t="inlineStr">
+        <is>
+          <t>VSTM</t>
+        </is>
+      </c>
+      <c r="C891" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="892">
+      <c r="A892" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="B892" t="inlineStr">
+        <is>
+          <t>ZSTK</t>
+        </is>
+      </c>
+      <c r="C892" t="inlineStr">
         <is>
           <t>Dropped</t>
         </is>
@@ -20658,7 +20857,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G917"/>
+  <dimension ref="A1:G937"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -41758,6 +41957,502 @@
         </is>
       </c>
       <c r="C917" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="918">
+      <c r="A918" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="B918" t="inlineStr">
+        <is>
+          <t>AVAT</t>
+        </is>
+      </c>
+      <c r="C918" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D918" t="n">
+        <v>1.58</v>
+      </c>
+      <c r="E918" t="n">
+        <v>1.38</v>
+      </c>
+      <c r="F918" t="n">
+        <v>1.98</v>
+      </c>
+      <c r="G918" t="n">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="919">
+      <c r="A919" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="B919" t="inlineStr">
+        <is>
+          <t>CISS</t>
+        </is>
+      </c>
+      <c r="C919" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D919" t="n">
+        <v>1.58</v>
+      </c>
+      <c r="E919" t="n">
+        <v>1.22</v>
+      </c>
+      <c r="F919" t="n">
+        <v>2.3</v>
+      </c>
+      <c r="G919" t="n">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="920">
+      <c r="A920" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="B920" t="inlineStr">
+        <is>
+          <t>GLND</t>
+        </is>
+      </c>
+      <c r="C920" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D920" t="n">
+        <v>3.03</v>
+      </c>
+      <c r="E920" t="n">
+        <v>2.65</v>
+      </c>
+      <c r="F920" t="n">
+        <v>3.79</v>
+      </c>
+      <c r="G920" t="n">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="921">
+      <c r="A921" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="B921" t="inlineStr">
+        <is>
+          <t>GRAL</t>
+        </is>
+      </c>
+      <c r="C921" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D921" t="n">
+        <v>101.57</v>
+      </c>
+      <c r="E921" t="n">
+        <v>92</v>
+      </c>
+      <c r="F921" t="n">
+        <v>120.71</v>
+      </c>
+      <c r="G921" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="922">
+      <c r="A922" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="B922" t="inlineStr">
+        <is>
+          <t>GRML</t>
+        </is>
+      </c>
+      <c r="C922" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D922" t="n">
+        <v>7.9</v>
+      </c>
+      <c r="E922" t="n">
+        <v>6.63</v>
+      </c>
+      <c r="F922" t="n">
+        <v>10.44</v>
+      </c>
+      <c r="G922" t="n">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="923">
+      <c r="A923" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="B923" t="inlineStr">
+        <is>
+          <t>INV</t>
+        </is>
+      </c>
+      <c r="C923" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D923" t="n">
+        <v>0.82</v>
+      </c>
+      <c r="E923" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="F923" t="n">
+        <v>1.06</v>
+      </c>
+      <c r="G923" t="n">
+        <v>417</v>
+      </c>
+    </row>
+    <row r="924">
+      <c r="A924" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="B924" t="inlineStr">
+        <is>
+          <t>MX</t>
+        </is>
+      </c>
+      <c r="C924" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D924" t="n">
+        <v>3.49</v>
+      </c>
+      <c r="E924" t="n">
+        <v>3.09</v>
+      </c>
+      <c r="F924" t="n">
+        <v>4.29</v>
+      </c>
+      <c r="G924" t="n">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="925">
+      <c r="A925" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="B925" t="inlineStr">
+        <is>
+          <t>NUAI</t>
+        </is>
+      </c>
+      <c r="C925" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D925" t="n">
+        <v>7.54</v>
+      </c>
+      <c r="E925" t="n">
+        <v>6.75</v>
+      </c>
+      <c r="F925" t="n">
+        <v>9.119999999999999</v>
+      </c>
+      <c r="G925" t="n">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="926">
+      <c r="A926" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="B926" t="inlineStr">
+        <is>
+          <t>OPTX</t>
+        </is>
+      </c>
+      <c r="C926" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D926" t="n">
+        <v>8.23</v>
+      </c>
+      <c r="E926" t="n">
+        <v>7.8</v>
+      </c>
+      <c r="F926" t="n">
+        <v>9.09</v>
+      </c>
+      <c r="G926" t="n">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="927">
+      <c r="A927" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="B927" t="inlineStr">
+        <is>
+          <t>PRTH</t>
+        </is>
+      </c>
+      <c r="C927" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D927" t="n">
+        <v>7.8</v>
+      </c>
+      <c r="E927" t="n">
+        <v>7.76</v>
+      </c>
+      <c r="F927" t="n">
+        <v>7.88</v>
+      </c>
+      <c r="G927" t="n">
+        <v>1250</v>
+      </c>
+    </row>
+    <row r="928">
+      <c r="A928" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="B928" t="inlineStr">
+        <is>
+          <t>SPRU</t>
+        </is>
+      </c>
+      <c r="C928" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D928" t="n">
+        <v>2.31</v>
+      </c>
+      <c r="E928" t="n">
+        <v>2</v>
+      </c>
+      <c r="F928" t="n">
+        <v>2.93</v>
+      </c>
+      <c r="G928" t="n">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="929">
+      <c r="A929" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="B929" t="inlineStr">
+        <is>
+          <t>SUIG</t>
+        </is>
+      </c>
+      <c r="C929" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D929" t="n">
+        <v>1.43</v>
+      </c>
+      <c r="E929" t="n">
+        <v>1.35</v>
+      </c>
+      <c r="F929" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="G929" t="n">
+        <v>588</v>
+      </c>
+    </row>
+    <row r="930">
+      <c r="A930" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="B930" t="inlineStr">
+        <is>
+          <t>VEEE</t>
+        </is>
+      </c>
+      <c r="C930" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D930" t="n">
+        <v>16.32</v>
+      </c>
+      <c r="E930" t="n">
+        <v>13.68</v>
+      </c>
+      <c r="F930" t="n">
+        <v>21.6</v>
+      </c>
+      <c r="G930" t="n">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="931">
+      <c r="A931" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="B931" t="inlineStr">
+        <is>
+          <t>BENF</t>
+        </is>
+      </c>
+      <c r="C931" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="932">
+      <c r="A932" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="B932" t="inlineStr">
+        <is>
+          <t>CTNT</t>
+        </is>
+      </c>
+      <c r="C932" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="933">
+      <c r="A933" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="B933" t="inlineStr">
+        <is>
+          <t>DSP</t>
+        </is>
+      </c>
+      <c r="C933" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="934">
+      <c r="A934" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="B934" t="inlineStr">
+        <is>
+          <t>FTCI</t>
+        </is>
+      </c>
+      <c r="C934" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="935">
+      <c r="A935" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="B935" t="inlineStr">
+        <is>
+          <t>GIPR</t>
+        </is>
+      </c>
+      <c r="C935" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="936">
+      <c r="A936" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="B936" t="inlineStr">
+        <is>
+          <t>TRUG</t>
+        </is>
+      </c>
+      <c r="C936" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="937">
+      <c r="A937" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="B937" t="inlineStr">
+        <is>
+          <t>USDE</t>
+        </is>
+      </c>
+      <c r="C937" t="inlineStr">
         <is>
           <t>Dropped</t>
         </is>

</xml_diff>

<commit_message>
Daily screener update: 2026-09-24
</commit_message>
<xml_diff>
--- a/screener_history.xlsx
+++ b/screener_history.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G904"/>
+  <dimension ref="A1:G916"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -21177,6 +21177,246 @@
         </is>
       </c>
       <c r="C904" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="905">
+      <c r="A905" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="B905" t="inlineStr">
+        <is>
+          <t>CHPT</t>
+        </is>
+      </c>
+      <c r="C905" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D905" t="n">
+        <v>10.72</v>
+      </c>
+      <c r="E905" t="n">
+        <v>8.56</v>
+      </c>
+      <c r="F905" t="n">
+        <v>15.04</v>
+      </c>
+      <c r="G905" t="n">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="906">
+      <c r="A906" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="B906" t="inlineStr">
+        <is>
+          <t>HELP</t>
+        </is>
+      </c>
+      <c r="C906" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D906" t="n">
+        <v>15.15</v>
+      </c>
+      <c r="E906" t="n">
+        <v>12.1</v>
+      </c>
+      <c r="F906" t="n">
+        <v>21.26</v>
+      </c>
+      <c r="G906" t="n">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="907">
+      <c r="A907" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="B907" t="inlineStr">
+        <is>
+          <t>PLSE</t>
+        </is>
+      </c>
+      <c r="C907" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D907" t="n">
+        <v>58.9</v>
+      </c>
+      <c r="E907" t="n">
+        <v>48.43</v>
+      </c>
+      <c r="F907" t="n">
+        <v>79.84999999999999</v>
+      </c>
+      <c r="G907" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="908">
+      <c r="A908" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="B908" t="inlineStr">
+        <is>
+          <t>AMLX</t>
+        </is>
+      </c>
+      <c r="C908" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="909">
+      <c r="A909" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="B909" t="inlineStr">
+        <is>
+          <t>ATER</t>
+        </is>
+      </c>
+      <c r="C909" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="910">
+      <c r="A910" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="B910" t="inlineStr">
+        <is>
+          <t>HOWL</t>
+        </is>
+      </c>
+      <c r="C910" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="911">
+      <c r="A911" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="B911" t="inlineStr">
+        <is>
+          <t>KPLT</t>
+        </is>
+      </c>
+      <c r="C911" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="912">
+      <c r="A912" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="B912" t="inlineStr">
+        <is>
+          <t>LHAI</t>
+        </is>
+      </c>
+      <c r="C912" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="913">
+      <c r="A913" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="B913" t="inlineStr">
+        <is>
+          <t>PEPG</t>
+        </is>
+      </c>
+      <c r="C913" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="914">
+      <c r="A914" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="B914" t="inlineStr">
+        <is>
+          <t>PYXS</t>
+        </is>
+      </c>
+      <c r="C914" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="915">
+      <c r="A915" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="B915" t="inlineStr">
+        <is>
+          <t>SST</t>
+        </is>
+      </c>
+      <c r="C915" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="916">
+      <c r="A916" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="B916" t="inlineStr">
+        <is>
+          <t>XPON</t>
+        </is>
+      </c>
+      <c r="C916" t="inlineStr">
         <is>
           <t>Dropped</t>
         </is>
@@ -21193,7 +21433,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G959"/>
+  <dimension ref="A1:G979"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -43259,6 +43499,502 @@
         </is>
       </c>
       <c r="C959" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="960">
+      <c r="A960" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="B960" t="inlineStr">
+        <is>
+          <t>BENF</t>
+        </is>
+      </c>
+      <c r="C960" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D960" t="n">
+        <v>3.03</v>
+      </c>
+      <c r="E960" t="n">
+        <v>1.44</v>
+      </c>
+      <c r="F960" t="n">
+        <v>6.21</v>
+      </c>
+      <c r="G960" t="n">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="961">
+      <c r="A961" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="B961" t="inlineStr">
+        <is>
+          <t>BFRG</t>
+        </is>
+      </c>
+      <c r="C961" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D961" t="n">
+        <v>0.79</v>
+      </c>
+      <c r="E961" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="F961" t="n">
+        <v>0.96</v>
+      </c>
+      <c r="G961" t="n">
+        <v>589</v>
+      </c>
+    </row>
+    <row r="962">
+      <c r="A962" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="B962" t="inlineStr">
+        <is>
+          <t>CAPS</t>
+        </is>
+      </c>
+      <c r="C962" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D962" t="n">
+        <v>0.23</v>
+      </c>
+      <c r="E962" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="F962" t="n">
+        <v>0.38</v>
+      </c>
+      <c r="G962" t="n">
+        <v>651</v>
+      </c>
+    </row>
+    <row r="963">
+      <c r="A963" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="B963" t="inlineStr">
+        <is>
+          <t>GRAL</t>
+        </is>
+      </c>
+      <c r="C963" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D963" t="n">
+        <v>107.15</v>
+      </c>
+      <c r="E963" t="n">
+        <v>104</v>
+      </c>
+      <c r="F963" t="n">
+        <v>113.45</v>
+      </c>
+      <c r="G963" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="964">
+      <c r="A964" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="B964" t="inlineStr">
+        <is>
+          <t>GURE</t>
+        </is>
+      </c>
+      <c r="C964" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D964" t="n">
+        <v>3.83</v>
+      </c>
+      <c r="E964" t="n">
+        <v>3.12</v>
+      </c>
+      <c r="F964" t="n">
+        <v>5.25</v>
+      </c>
+      <c r="G964" t="n">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="965">
+      <c r="A965" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="B965" t="inlineStr">
+        <is>
+          <t>HCTI</t>
+        </is>
+      </c>
+      <c r="C965" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D965" t="n">
+        <v>1.28</v>
+      </c>
+      <c r="E965" t="n">
+        <v>0.89</v>
+      </c>
+      <c r="F965" t="n">
+        <v>2.06</v>
+      </c>
+      <c r="G965" t="n">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="966">
+      <c r="A966" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="B966" t="inlineStr">
+        <is>
+          <t>IONQ</t>
+        </is>
+      </c>
+      <c r="C966" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D966" t="n">
+        <v>46.05</v>
+      </c>
+      <c r="E966" t="n">
+        <v>41.63</v>
+      </c>
+      <c r="F966" t="n">
+        <v>54.89</v>
+      </c>
+      <c r="G966" t="n">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="967">
+      <c r="A967" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="B967" t="inlineStr">
+        <is>
+          <t>MAZE</t>
+        </is>
+      </c>
+      <c r="C967" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D967" t="n">
+        <v>29.31</v>
+      </c>
+      <c r="E967" t="n">
+        <v>27.53</v>
+      </c>
+      <c r="F967" t="n">
+        <v>32.87</v>
+      </c>
+      <c r="G967" t="n">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="968">
+      <c r="A968" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="B968" t="inlineStr">
+        <is>
+          <t>MSS</t>
+        </is>
+      </c>
+      <c r="C968" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D968" t="n">
+        <v>2.32</v>
+      </c>
+      <c r="E968" t="n">
+        <v>1.81</v>
+      </c>
+      <c r="F968" t="n">
+        <v>3.34</v>
+      </c>
+      <c r="G968" t="n">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="969">
+      <c r="A969" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="B969" t="inlineStr">
+        <is>
+          <t>NNBR</t>
+        </is>
+      </c>
+      <c r="C969" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D969" t="n">
+        <v>3.75</v>
+      </c>
+      <c r="E969" t="n">
+        <v>3.55</v>
+      </c>
+      <c r="F969" t="n">
+        <v>4.15</v>
+      </c>
+      <c r="G969" t="n">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="970">
+      <c r="A970" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="B970" t="inlineStr">
+        <is>
+          <t>TLSI</t>
+        </is>
+      </c>
+      <c r="C970" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D970" t="n">
+        <v>5.83</v>
+      </c>
+      <c r="E970" t="n">
+        <v>4.92</v>
+      </c>
+      <c r="F970" t="n">
+        <v>7.65</v>
+      </c>
+      <c r="G970" t="n">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="971">
+      <c r="A971" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="B971" t="inlineStr">
+        <is>
+          <t>VTGN</t>
+        </is>
+      </c>
+      <c r="C971" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D971" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="E971" t="n">
+        <v>0.34</v>
+      </c>
+      <c r="F971" t="n">
+        <v>0.54</v>
+      </c>
+      <c r="G971" t="n">
+        <v>720</v>
+      </c>
+    </row>
+    <row r="972">
+      <c r="A972" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="B972" t="inlineStr">
+        <is>
+          <t>WHLR</t>
+        </is>
+      </c>
+      <c r="C972" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D972" t="n">
+        <v>6.14</v>
+      </c>
+      <c r="E972" t="n">
+        <v>4.75</v>
+      </c>
+      <c r="F972" t="n">
+        <v>8.92</v>
+      </c>
+      <c r="G972" t="n">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="973">
+      <c r="A973" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="B973" t="inlineStr">
+        <is>
+          <t>FLNA</t>
+        </is>
+      </c>
+      <c r="C973" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="974">
+      <c r="A974" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="B974" t="inlineStr">
+        <is>
+          <t>GDC</t>
+        </is>
+      </c>
+      <c r="C974" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="975">
+      <c r="A975" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="B975" t="inlineStr">
+        <is>
+          <t>OPENL</t>
+        </is>
+      </c>
+      <c r="C975" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="976">
+      <c r="A976" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="B976" t="inlineStr">
+        <is>
+          <t>OPENZ</t>
+        </is>
+      </c>
+      <c r="C976" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="977">
+      <c r="A977" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="B977" t="inlineStr">
+        <is>
+          <t>SPRO</t>
+        </is>
+      </c>
+      <c r="C977" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="978">
+      <c r="A978" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="B978" t="inlineStr">
+        <is>
+          <t>VKTX</t>
+        </is>
+      </c>
+      <c r="C978" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="979">
+      <c r="A979" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="B979" t="inlineStr">
+        <is>
+          <t>ZEO</t>
+        </is>
+      </c>
+      <c r="C979" t="inlineStr">
         <is>
           <t>Dropped</t>
         </is>

</xml_diff>

<commit_message>
Daily screener update: 2026-09-25
</commit_message>
<xml_diff>
--- a/screener_history.xlsx
+++ b/screener_history.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G916"/>
+  <dimension ref="A1:G924"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -21417,6 +21417,178 @@
         </is>
       </c>
       <c r="C916" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="917">
+      <c r="A917" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="B917" t="inlineStr">
+        <is>
+          <t>AGPU</t>
+        </is>
+      </c>
+      <c r="C917" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D917" t="n">
+        <v>13.48</v>
+      </c>
+      <c r="E917" t="n">
+        <v>10.46</v>
+      </c>
+      <c r="F917" t="n">
+        <v>19.52</v>
+      </c>
+      <c r="G917" t="n">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="918">
+      <c r="A918" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="B918" t="inlineStr">
+        <is>
+          <t>ATER</t>
+        </is>
+      </c>
+      <c r="C918" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D918" t="n">
+        <v>0.92</v>
+      </c>
+      <c r="E918" t="n">
+        <v>0.63</v>
+      </c>
+      <c r="F918" t="n">
+        <v>1.49</v>
+      </c>
+      <c r="G918" t="n">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="919">
+      <c r="A919" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="B919" t="inlineStr">
+        <is>
+          <t>RDIB</t>
+        </is>
+      </c>
+      <c r="C919" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D919" t="n">
+        <v>19.36</v>
+      </c>
+      <c r="E919" t="n">
+        <v>14.33</v>
+      </c>
+      <c r="F919" t="n">
+        <v>29.42</v>
+      </c>
+      <c r="G919" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="920">
+      <c r="A920" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="B920" t="inlineStr">
+        <is>
+          <t>CHPT</t>
+        </is>
+      </c>
+      <c r="C920" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="921">
+      <c r="A921" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="B921" t="inlineStr">
+        <is>
+          <t>GPRO</t>
+        </is>
+      </c>
+      <c r="C921" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="922">
+      <c r="A922" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="B922" t="inlineStr">
+        <is>
+          <t>HELP</t>
+        </is>
+      </c>
+      <c r="C922" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="923">
+      <c r="A923" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="B923" t="inlineStr">
+        <is>
+          <t>PLSE</t>
+        </is>
+      </c>
+      <c r="C923" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="924">
+      <c r="A924" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="B924" t="inlineStr">
+        <is>
+          <t>UTZ</t>
+        </is>
+      </c>
+      <c r="C924" t="inlineStr">
         <is>
           <t>Dropped</t>
         </is>
@@ -21433,7 +21605,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G979"/>
+  <dimension ref="A1:G1002"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -43995,6 +44167,493 @@
         </is>
       </c>
       <c r="C979" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="980">
+      <c r="A980" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="B980" t="inlineStr">
+        <is>
+          <t>GCTK</t>
+        </is>
+      </c>
+      <c r="C980" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D980" t="n">
+        <v>2.92</v>
+      </c>
+      <c r="E980" t="n">
+        <v>2.38</v>
+      </c>
+      <c r="F980" t="n">
+        <v>4</v>
+      </c>
+      <c r="G980" t="n">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="981">
+      <c r="A981" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="B981" t="inlineStr">
+        <is>
+          <t>GLND</t>
+        </is>
+      </c>
+      <c r="C981" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D981" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="E981" t="n">
+        <v>3.19</v>
+      </c>
+      <c r="F981" t="n">
+        <v>4.12</v>
+      </c>
+      <c r="G981" t="n">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="982">
+      <c r="A982" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="B982" t="inlineStr">
+        <is>
+          <t>KYTX</t>
+        </is>
+      </c>
+      <c r="C982" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D982" t="n">
+        <v>7.82</v>
+      </c>
+      <c r="E982" t="n">
+        <v>6.68</v>
+      </c>
+      <c r="F982" t="n">
+        <v>10.1</v>
+      </c>
+      <c r="G982" t="n">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="983">
+      <c r="A983" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="B983" t="inlineStr">
+        <is>
+          <t>LITS</t>
+        </is>
+      </c>
+      <c r="C983" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D983" t="n">
+        <v>1.48</v>
+      </c>
+      <c r="E983" t="n">
+        <v>1.31</v>
+      </c>
+      <c r="F983" t="n">
+        <v>1.82</v>
+      </c>
+      <c r="G983" t="n">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="984">
+      <c r="A984" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="B984" t="inlineStr">
+        <is>
+          <t>PFSA</t>
+        </is>
+      </c>
+      <c r="C984" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D984" t="n">
+        <v>4.13</v>
+      </c>
+      <c r="E984" t="n">
+        <v>2.39</v>
+      </c>
+      <c r="F984" t="n">
+        <v>7.61</v>
+      </c>
+      <c r="G984" t="n">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="985">
+      <c r="A985" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="B985" t="inlineStr">
+        <is>
+          <t>SKYQ</t>
+        </is>
+      </c>
+      <c r="C985" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D985" t="n">
+        <v>3.1</v>
+      </c>
+      <c r="E985" t="n">
+        <v>2.68</v>
+      </c>
+      <c r="F985" t="n">
+        <v>3.94</v>
+      </c>
+      <c r="G985" t="n">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="986">
+      <c r="A986" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="B986" t="inlineStr">
+        <is>
+          <t>SRZN</t>
+        </is>
+      </c>
+      <c r="C986" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D986" t="n">
+        <v>35.04</v>
+      </c>
+      <c r="E986" t="n">
+        <v>29.1</v>
+      </c>
+      <c r="F986" t="n">
+        <v>46.92</v>
+      </c>
+      <c r="G986" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="987">
+      <c r="A987" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="B987" t="inlineStr">
+        <is>
+          <t>VRME</t>
+        </is>
+      </c>
+      <c r="C987" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D987" t="n">
+        <v>1.31</v>
+      </c>
+      <c r="E987" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="F987" t="n">
+        <v>1.73</v>
+      </c>
+      <c r="G987" t="n">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="988">
+      <c r="A988" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="B988" t="inlineStr">
+        <is>
+          <t>BENF</t>
+        </is>
+      </c>
+      <c r="C988" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="989">
+      <c r="A989" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="B989" t="inlineStr">
+        <is>
+          <t>BFRG</t>
+        </is>
+      </c>
+      <c r="C989" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="990">
+      <c r="A990" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="B990" t="inlineStr">
+        <is>
+          <t>CAPS</t>
+        </is>
+      </c>
+      <c r="C990" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="991">
+      <c r="A991" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="B991" t="inlineStr">
+        <is>
+          <t>DCOY</t>
+        </is>
+      </c>
+      <c r="C991" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="992">
+      <c r="A992" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="B992" t="inlineStr">
+        <is>
+          <t>GRAL</t>
+        </is>
+      </c>
+      <c r="C992" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="993">
+      <c r="A993" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="B993" t="inlineStr">
+        <is>
+          <t>GURE</t>
+        </is>
+      </c>
+      <c r="C993" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="994">
+      <c r="A994" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="B994" t="inlineStr">
+        <is>
+          <t>HCTI</t>
+        </is>
+      </c>
+      <c r="C994" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="995">
+      <c r="A995" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="B995" t="inlineStr">
+        <is>
+          <t>IONQ</t>
+        </is>
+      </c>
+      <c r="C995" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="996">
+      <c r="A996" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="B996" t="inlineStr">
+        <is>
+          <t>MAZE</t>
+        </is>
+      </c>
+      <c r="C996" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="997">
+      <c r="A997" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="B997" t="inlineStr">
+        <is>
+          <t>MSS</t>
+        </is>
+      </c>
+      <c r="C997" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="998">
+      <c r="A998" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="B998" t="inlineStr">
+        <is>
+          <t>NNBR</t>
+        </is>
+      </c>
+      <c r="C998" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="999">
+      <c r="A999" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="B999" t="inlineStr">
+        <is>
+          <t>SVRN</t>
+        </is>
+      </c>
+      <c r="C999" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="1000">
+      <c r="A1000" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="B1000" t="inlineStr">
+        <is>
+          <t>TLSI</t>
+        </is>
+      </c>
+      <c r="C1000" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="1001">
+      <c r="A1001" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="B1001" t="inlineStr">
+        <is>
+          <t>VTGN</t>
+        </is>
+      </c>
+      <c r="C1001" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="1002">
+      <c r="A1002" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="B1002" t="inlineStr">
+        <is>
+          <t>WHLR</t>
+        </is>
+      </c>
+      <c r="C1002" t="inlineStr">
         <is>
           <t>Dropped</t>
         </is>

</xml_diff>

<commit_message>
Daily screener update: 2026-09-26
</commit_message>
<xml_diff>
--- a/screener_history.xlsx
+++ b/screener_history.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G924"/>
+  <dimension ref="A1:G929"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -21589,6 +21589,115 @@
         </is>
       </c>
       <c r="C924" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="925">
+      <c r="A925" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+      <c r="B925" t="inlineStr">
+        <is>
+          <t>BIO-B</t>
+        </is>
+      </c>
+      <c r="C925" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D925" t="n">
+        <v>365.08</v>
+      </c>
+      <c r="E925" t="n">
+        <v>365.08</v>
+      </c>
+      <c r="F925" t="n">
+        <v>365.08</v>
+      </c>
+      <c r="G925" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="926">
+      <c r="A926" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+      <c r="B926" t="inlineStr">
+        <is>
+          <t>BYFC</t>
+        </is>
+      </c>
+      <c r="C926" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D926" t="n">
+        <v>12.15</v>
+      </c>
+      <c r="E926" t="n">
+        <v>11.79</v>
+      </c>
+      <c r="F926" t="n">
+        <v>12.87</v>
+      </c>
+      <c r="G926" t="n">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="927">
+      <c r="A927" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+      <c r="B927" t="inlineStr">
+        <is>
+          <t>AGPU</t>
+        </is>
+      </c>
+      <c r="C927" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="928">
+      <c r="A928" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+      <c r="B928" t="inlineStr">
+        <is>
+          <t>ATER</t>
+        </is>
+      </c>
+      <c r="C928" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="929">
+      <c r="A929" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+      <c r="B929" t="inlineStr">
+        <is>
+          <t>RDIB</t>
+        </is>
+      </c>
+      <c r="C929" t="inlineStr">
         <is>
           <t>Dropped</t>
         </is>
@@ -21605,7 +21714,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G1002"/>
+  <dimension ref="A1:G1019"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -44654,6 +44763,403 @@
         </is>
       </c>
       <c r="C1002" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="1003">
+      <c r="A1003" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+      <c r="B1003" t="inlineStr">
+        <is>
+          <t>AESI</t>
+        </is>
+      </c>
+      <c r="C1003" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D1003" t="n">
+        <v>12.4</v>
+      </c>
+      <c r="E1003" t="n">
+        <v>12.25</v>
+      </c>
+      <c r="F1003" t="n">
+        <v>12.7</v>
+      </c>
+      <c r="G1003" t="n">
+        <v>333</v>
+      </c>
+    </row>
+    <row r="1004">
+      <c r="A1004" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+      <c r="B1004" t="inlineStr">
+        <is>
+          <t>AIFF</t>
+        </is>
+      </c>
+      <c r="C1004" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D1004" t="n">
+        <v>1.77</v>
+      </c>
+      <c r="E1004" t="n">
+        <v>1.48</v>
+      </c>
+      <c r="F1004" t="n">
+        <v>2.35</v>
+      </c>
+      <c r="G1004" t="n">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="1005">
+      <c r="A1005" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+      <c r="B1005" t="inlineStr">
+        <is>
+          <t>AKAM</t>
+        </is>
+      </c>
+      <c r="C1005" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D1005" t="n">
+        <v>128.35</v>
+      </c>
+      <c r="E1005" t="n">
+        <v>113.84</v>
+      </c>
+      <c r="F1005" t="n">
+        <v>157.37</v>
+      </c>
+      <c r="G1005" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="1006">
+      <c r="A1006" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+      <c r="B1006" t="inlineStr">
+        <is>
+          <t>CNET</t>
+        </is>
+      </c>
+      <c r="C1006" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D1006" t="n">
+        <v>2.3</v>
+      </c>
+      <c r="E1006" t="n">
+        <v>1.53</v>
+      </c>
+      <c r="F1006" t="n">
+        <v>3.84</v>
+      </c>
+      <c r="G1006" t="n">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="1007">
+      <c r="A1007" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+      <c r="B1007" t="inlineStr">
+        <is>
+          <t>FTHM</t>
+        </is>
+      </c>
+      <c r="C1007" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D1007" t="n">
+        <v>0.64</v>
+      </c>
+      <c r="E1007" t="n">
+        <v>0.5600000000000001</v>
+      </c>
+      <c r="F1007" t="n">
+        <v>0.8100000000000001</v>
+      </c>
+      <c r="G1007" t="n">
+        <v>580</v>
+      </c>
+    </row>
+    <row r="1008">
+      <c r="A1008" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+      <c r="B1008" t="inlineStr">
+        <is>
+          <t>JAGX</t>
+        </is>
+      </c>
+      <c r="C1008" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D1008" t="n">
+        <v>9.859999999999999</v>
+      </c>
+      <c r="E1008" t="n">
+        <v>6.8</v>
+      </c>
+      <c r="F1008" t="n">
+        <v>15.98</v>
+      </c>
+      <c r="G1008" t="n">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="1009">
+      <c r="A1009" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+      <c r="B1009" t="inlineStr">
+        <is>
+          <t>ONCO</t>
+        </is>
+      </c>
+      <c r="C1009" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D1009" t="n">
+        <v>1.12</v>
+      </c>
+      <c r="E1009" t="n">
+        <v>1</v>
+      </c>
+      <c r="F1009" t="n">
+        <v>1.36</v>
+      </c>
+      <c r="G1009" t="n">
+        <v>416</v>
+      </c>
+    </row>
+    <row r="1010">
+      <c r="A1010" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+      <c r="B1010" t="inlineStr">
+        <is>
+          <t>STEM</t>
+        </is>
+      </c>
+      <c r="C1010" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D1010" t="n">
+        <v>4.45</v>
+      </c>
+      <c r="E1010" t="n">
+        <v>4.25</v>
+      </c>
+      <c r="F1010" t="n">
+        <v>4.85</v>
+      </c>
+      <c r="G1010" t="n">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="1011">
+      <c r="A1011" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+      <c r="B1011" t="inlineStr">
+        <is>
+          <t>WHLR</t>
+        </is>
+      </c>
+      <c r="C1011" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D1011" t="n">
+        <v>4.86</v>
+      </c>
+      <c r="E1011" t="n">
+        <v>4.38</v>
+      </c>
+      <c r="F1011" t="n">
+        <v>5.82</v>
+      </c>
+      <c r="G1011" t="n">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="1012">
+      <c r="A1012" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+      <c r="B1012" t="inlineStr">
+        <is>
+          <t>GCTK</t>
+        </is>
+      </c>
+      <c r="C1012" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="1013">
+      <c r="A1013" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+      <c r="B1013" t="inlineStr">
+        <is>
+          <t>GRML</t>
+        </is>
+      </c>
+      <c r="C1013" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="1014">
+      <c r="A1014" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+      <c r="B1014" t="inlineStr">
+        <is>
+          <t>KYTX</t>
+        </is>
+      </c>
+      <c r="C1014" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="1015">
+      <c r="A1015" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+      <c r="B1015" t="inlineStr">
+        <is>
+          <t>LITS</t>
+        </is>
+      </c>
+      <c r="C1015" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="1016">
+      <c r="A1016" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+      <c r="B1016" t="inlineStr">
+        <is>
+          <t>PFSA</t>
+        </is>
+      </c>
+      <c r="C1016" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="1017">
+      <c r="A1017" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+      <c r="B1017" t="inlineStr">
+        <is>
+          <t>SKYQ</t>
+        </is>
+      </c>
+      <c r="C1017" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="1018">
+      <c r="A1018" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+      <c r="B1018" t="inlineStr">
+        <is>
+          <t>SRZN</t>
+        </is>
+      </c>
+      <c r="C1018" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="1019">
+      <c r="A1019" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+      <c r="B1019" t="inlineStr">
+        <is>
+          <t>VRME</t>
+        </is>
+      </c>
+      <c r="C1019" t="inlineStr">
         <is>
           <t>Dropped</t>
         </is>

</xml_diff>

<commit_message>
Daily screener update: 2026-09-29
</commit_message>
<xml_diff>
--- a/screener_history.xlsx
+++ b/screener_history.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G929"/>
+  <dimension ref="A1:G932"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -21698,6 +21698,81 @@
         </is>
       </c>
       <c r="C929" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="930">
+      <c r="A930" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="B930" t="inlineStr">
+        <is>
+          <t>EFSI</t>
+        </is>
+      </c>
+      <c r="C930" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D930" t="n">
+        <v>48.17</v>
+      </c>
+      <c r="E930" t="n">
+        <v>45.36</v>
+      </c>
+      <c r="F930" t="n">
+        <v>53.79</v>
+      </c>
+      <c r="G930" t="n">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="931">
+      <c r="A931" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="B931" t="inlineStr">
+        <is>
+          <t>RDIB</t>
+        </is>
+      </c>
+      <c r="C931" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D931" t="n">
+        <v>19.36</v>
+      </c>
+      <c r="E931" t="n">
+        <v>14.57</v>
+      </c>
+      <c r="F931" t="n">
+        <v>28.94</v>
+      </c>
+      <c r="G931" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="932">
+      <c r="A932" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="B932" t="inlineStr">
+        <is>
+          <t>BYFC</t>
+        </is>
+      </c>
+      <c r="C932" t="inlineStr">
         <is>
           <t>Dropped</t>
         </is>
@@ -21714,7 +21789,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G1019"/>
+  <dimension ref="A1:G1034"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -45160,6 +45235,333 @@
         </is>
       </c>
       <c r="C1019" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="1020">
+      <c r="A1020" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="B1020" t="inlineStr">
+        <is>
+          <t>ARAY</t>
+        </is>
+      </c>
+      <c r="C1020" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D1020" t="n">
+        <v>0.33</v>
+      </c>
+      <c r="E1020" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="F1020" t="n">
+        <v>0.41</v>
+      </c>
+      <c r="G1020" t="n">
+        <v>1190</v>
+      </c>
+    </row>
+    <row r="1021">
+      <c r="A1021" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="B1021" t="inlineStr">
+        <is>
+          <t>CLRO</t>
+        </is>
+      </c>
+      <c r="C1021" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D1021" t="n">
+        <v>6</v>
+      </c>
+      <c r="E1021" t="n">
+        <v>4.19</v>
+      </c>
+      <c r="F1021" t="n">
+        <v>9.619999999999999</v>
+      </c>
+      <c r="G1021" t="n">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="1022">
+      <c r="A1022" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="B1022" t="inlineStr">
+        <is>
+          <t>KOD</t>
+        </is>
+      </c>
+      <c r="C1022" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D1022" t="n">
+        <v>69.98999999999999</v>
+      </c>
+      <c r="E1022" t="n">
+        <v>60.5</v>
+      </c>
+      <c r="F1022" t="n">
+        <v>88.97</v>
+      </c>
+      <c r="G1022" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="1023">
+      <c r="A1023" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="B1023" t="inlineStr">
+        <is>
+          <t>LABT</t>
+        </is>
+      </c>
+      <c r="C1023" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D1023" t="n">
+        <v>2.13</v>
+      </c>
+      <c r="E1023" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="F1023" t="n">
+        <v>4.19</v>
+      </c>
+      <c r="G1023" t="n">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="1024">
+      <c r="A1024" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="B1024" t="inlineStr">
+        <is>
+          <t>LFCR</t>
+        </is>
+      </c>
+      <c r="C1024" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D1024" t="n">
+        <v>6.65</v>
+      </c>
+      <c r="E1024" t="n">
+        <v>6.4</v>
+      </c>
+      <c r="F1024" t="n">
+        <v>7.14</v>
+      </c>
+      <c r="G1024" t="n">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="1025">
+      <c r="A1025" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="B1025" t="inlineStr">
+        <is>
+          <t>MX</t>
+        </is>
+      </c>
+      <c r="C1025" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D1025" t="n">
+        <v>4.02</v>
+      </c>
+      <c r="E1025" t="n">
+        <v>3.66</v>
+      </c>
+      <c r="F1025" t="n">
+        <v>4.74</v>
+      </c>
+      <c r="G1025" t="n">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="1026">
+      <c r="A1026" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="B1026" t="inlineStr">
+        <is>
+          <t>AESI</t>
+        </is>
+      </c>
+      <c r="C1026" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="1027">
+      <c r="A1027" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="B1027" t="inlineStr">
+        <is>
+          <t>AIFF</t>
+        </is>
+      </c>
+      <c r="C1027" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="1028">
+      <c r="A1028" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="B1028" t="inlineStr">
+        <is>
+          <t>AKAM</t>
+        </is>
+      </c>
+      <c r="C1028" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="1029">
+      <c r="A1029" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="B1029" t="inlineStr">
+        <is>
+          <t>CNET</t>
+        </is>
+      </c>
+      <c r="C1029" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="1030">
+      <c r="A1030" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="B1030" t="inlineStr">
+        <is>
+          <t>FTHM</t>
+        </is>
+      </c>
+      <c r="C1030" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="1031">
+      <c r="A1031" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="B1031" t="inlineStr">
+        <is>
+          <t>GLND</t>
+        </is>
+      </c>
+      <c r="C1031" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="1032">
+      <c r="A1032" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="B1032" t="inlineStr">
+        <is>
+          <t>JAGX</t>
+        </is>
+      </c>
+      <c r="C1032" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="1033">
+      <c r="A1033" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="B1033" t="inlineStr">
+        <is>
+          <t>STEM</t>
+        </is>
+      </c>
+      <c r="C1033" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="1034">
+      <c r="A1034" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="B1034" t="inlineStr">
+        <is>
+          <t>WHLR</t>
+        </is>
+      </c>
+      <c r="C1034" t="inlineStr">
         <is>
           <t>Dropped</t>
         </is>

</xml_diff>

<commit_message>
Daily screener update: 2026-09-30
</commit_message>
<xml_diff>
--- a/screener_history.xlsx
+++ b/screener_history.xlsx
@@ -21789,7 +21789,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G1034"/>
+  <dimension ref="A1:G1045"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -45562,6 +45562,241 @@
         </is>
       </c>
       <c r="C1034" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="1035">
+      <c r="A1035" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="B1035" t="inlineStr">
+        <is>
+          <t>IOVA</t>
+        </is>
+      </c>
+      <c r="C1035" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D1035" t="n">
+        <v>13.26</v>
+      </c>
+      <c r="E1035" t="n">
+        <v>12.78</v>
+      </c>
+      <c r="F1035" t="n">
+        <v>14.22</v>
+      </c>
+      <c r="G1035" t="n">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="1036">
+      <c r="A1036" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="B1036" t="inlineStr">
+        <is>
+          <t>JELD</t>
+        </is>
+      </c>
+      <c r="C1036" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D1036" t="n">
+        <v>2.11</v>
+      </c>
+      <c r="E1036" t="n">
+        <v>1.82</v>
+      </c>
+      <c r="F1036" t="n">
+        <v>2.7</v>
+      </c>
+      <c r="G1036" t="n">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="1037">
+      <c r="A1037" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="B1037" t="inlineStr">
+        <is>
+          <t>SMMT</t>
+        </is>
+      </c>
+      <c r="C1037" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D1037" t="n">
+        <v>19.07</v>
+      </c>
+      <c r="E1037" t="n">
+        <v>16.15</v>
+      </c>
+      <c r="F1037" t="n">
+        <v>24.91</v>
+      </c>
+      <c r="G1037" t="n">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="1038">
+      <c r="A1038" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="B1038" t="inlineStr">
+        <is>
+          <t>SSTI</t>
+        </is>
+      </c>
+      <c r="C1038" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D1038" t="n">
+        <v>8.43</v>
+      </c>
+      <c r="E1038" t="n">
+        <v>8.18</v>
+      </c>
+      <c r="F1038" t="n">
+        <v>8.93</v>
+      </c>
+      <c r="G1038" t="n">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="1039">
+      <c r="A1039" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="B1039" t="inlineStr">
+        <is>
+          <t>ARAY</t>
+        </is>
+      </c>
+      <c r="C1039" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="1040">
+      <c r="A1040" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="B1040" t="inlineStr">
+        <is>
+          <t>CLRO</t>
+        </is>
+      </c>
+      <c r="C1040" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="1041">
+      <c r="A1041" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="B1041" t="inlineStr">
+        <is>
+          <t>KOD</t>
+        </is>
+      </c>
+      <c r="C1041" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="1042">
+      <c r="A1042" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="B1042" t="inlineStr">
+        <is>
+          <t>LABT</t>
+        </is>
+      </c>
+      <c r="C1042" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="1043">
+      <c r="A1043" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="B1043" t="inlineStr">
+        <is>
+          <t>LFCR</t>
+        </is>
+      </c>
+      <c r="C1043" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="1044">
+      <c r="A1044" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="B1044" t="inlineStr">
+        <is>
+          <t>MX</t>
+        </is>
+      </c>
+      <c r="C1044" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="1045">
+      <c r="A1045" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="B1045" t="inlineStr">
+        <is>
+          <t>ONCO</t>
+        </is>
+      </c>
+      <c r="C1045" t="inlineStr">
         <is>
           <t>Dropped</t>
         </is>

</xml_diff>

<commit_message>
Daily screener update: 2026-10-01
</commit_message>
<xml_diff>
--- a/screener_history.xlsx
+++ b/screener_history.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G932"/>
+  <dimension ref="A1:G934"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -21773,6 +21773,52 @@
         </is>
       </c>
       <c r="C932" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="933">
+      <c r="A933" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="B933" t="inlineStr">
+        <is>
+          <t>KF</t>
+        </is>
+      </c>
+      <c r="C933" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D933" t="n">
+        <v>68.98</v>
+      </c>
+      <c r="E933" t="n">
+        <v>63.85</v>
+      </c>
+      <c r="F933" t="n">
+        <v>79.23999999999999</v>
+      </c>
+      <c r="G933" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="934">
+      <c r="A934" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="B934" t="inlineStr">
+        <is>
+          <t>RDIB</t>
+        </is>
+      </c>
+      <c r="C934" t="inlineStr">
         <is>
           <t>Dropped</t>
         </is>
@@ -21789,7 +21835,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G1045"/>
+  <dimension ref="A1:G1054"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -45797,6 +45843,219 @@
         </is>
       </c>
       <c r="C1045" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="1046">
+      <c r="A1046" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="B1046" t="inlineStr">
+        <is>
+          <t>AMSS</t>
+        </is>
+      </c>
+      <c r="C1046" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D1046" t="n">
+        <v>0.48</v>
+      </c>
+      <c r="E1046" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="F1046" t="n">
+        <v>0.57</v>
+      </c>
+      <c r="G1046" t="n">
+        <v>1136</v>
+      </c>
+    </row>
+    <row r="1047">
+      <c r="A1047" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="B1047" t="inlineStr">
+        <is>
+          <t>FNGR</t>
+        </is>
+      </c>
+      <c r="C1047" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D1047" t="n">
+        <v>0.16</v>
+      </c>
+      <c r="E1047" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="F1047" t="n">
+        <v>0.17</v>
+      </c>
+      <c r="G1047" t="n">
+        <v>7462</v>
+      </c>
+    </row>
+    <row r="1048">
+      <c r="A1048" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="B1048" t="inlineStr">
+        <is>
+          <t>SGMT</t>
+        </is>
+      </c>
+      <c r="C1048" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D1048" t="n">
+        <v>10.92</v>
+      </c>
+      <c r="E1048" t="n">
+        <v>9.460000000000001</v>
+      </c>
+      <c r="F1048" t="n">
+        <v>13.84</v>
+      </c>
+      <c r="G1048" t="n">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="1049">
+      <c r="A1049" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="B1049" t="inlineStr">
+        <is>
+          <t>SOTK</t>
+        </is>
+      </c>
+      <c r="C1049" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D1049" t="n">
+        <v>6.2</v>
+      </c>
+      <c r="E1049" t="n">
+        <v>5.3</v>
+      </c>
+      <c r="F1049" t="n">
+        <v>8</v>
+      </c>
+      <c r="G1049" t="n">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="1050">
+      <c r="A1050" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="B1050" t="inlineStr">
+        <is>
+          <t>VBIO</t>
+        </is>
+      </c>
+      <c r="C1050" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D1050" t="n">
+        <v>4.39</v>
+      </c>
+      <c r="E1050" t="n">
+        <v>2.53</v>
+      </c>
+      <c r="F1050" t="n">
+        <v>8.109999999999999</v>
+      </c>
+      <c r="G1050" t="n">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="1051">
+      <c r="A1051" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="B1051" t="inlineStr">
+        <is>
+          <t>IOVA</t>
+        </is>
+      </c>
+      <c r="C1051" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="1052">
+      <c r="A1052" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="B1052" t="inlineStr">
+        <is>
+          <t>JELD</t>
+        </is>
+      </c>
+      <c r="C1052" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="1053">
+      <c r="A1053" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="B1053" t="inlineStr">
+        <is>
+          <t>SMMT</t>
+        </is>
+      </c>
+      <c r="C1053" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="1054">
+      <c r="A1054" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="B1054" t="inlineStr">
+        <is>
+          <t>SSTI</t>
+        </is>
+      </c>
+      <c r="C1054" t="inlineStr">
         <is>
           <t>Dropped</t>
         </is>

</xml_diff>

<commit_message>
Daily screener update: 2026-10-02
</commit_message>
<xml_diff>
--- a/screener_history.xlsx
+++ b/screener_history.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G934"/>
+  <dimension ref="A1:G938"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -21819,6 +21819,86 @@
         </is>
       </c>
       <c r="C934" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="935">
+      <c r="A935" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+      <c r="B935" t="inlineStr">
+        <is>
+          <t>RDIB</t>
+        </is>
+      </c>
+      <c r="C935" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D935" t="n">
+        <v>19.36</v>
+      </c>
+      <c r="E935" t="n">
+        <v>14.57</v>
+      </c>
+      <c r="F935" t="n">
+        <v>28.94</v>
+      </c>
+      <c r="G935" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="936">
+      <c r="A936" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+      <c r="B936" t="inlineStr">
+        <is>
+          <t>BIO-B</t>
+        </is>
+      </c>
+      <c r="C936" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="937">
+      <c r="A937" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+      <c r="B937" t="inlineStr">
+        <is>
+          <t>EFSI</t>
+        </is>
+      </c>
+      <c r="C937" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="938">
+      <c r="A938" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+      <c r="B938" t="inlineStr">
+        <is>
+          <t>KF</t>
+        </is>
+      </c>
+      <c r="C938" t="inlineStr">
         <is>
           <t>Dropped</t>
         </is>
@@ -21835,7 +21915,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G1054"/>
+  <dimension ref="A1:G1065"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -46056,6 +46136,265 @@
         </is>
       </c>
       <c r="C1054" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="1055">
+      <c r="A1055" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+      <c r="B1055" t="inlineStr">
+        <is>
+          <t>AIXC</t>
+        </is>
+      </c>
+      <c r="C1055" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D1055" t="n">
+        <v>1.79</v>
+      </c>
+      <c r="E1055" t="n">
+        <v>0.97</v>
+      </c>
+      <c r="F1055" t="n">
+        <v>3.43</v>
+      </c>
+      <c r="G1055" t="n">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="1056">
+      <c r="A1056" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+      <c r="B1056" t="inlineStr">
+        <is>
+          <t>GIPR</t>
+        </is>
+      </c>
+      <c r="C1056" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D1056" t="n">
+        <v>0.58</v>
+      </c>
+      <c r="E1056" t="n">
+        <v>0.42</v>
+      </c>
+      <c r="F1056" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="G1056" t="n">
+        <v>307</v>
+      </c>
+    </row>
+    <row r="1057">
+      <c r="A1057" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+      <c r="B1057" t="inlineStr">
+        <is>
+          <t>NXL</t>
+        </is>
+      </c>
+      <c r="C1057" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D1057" t="n">
+        <v>9.109999999999999</v>
+      </c>
+      <c r="E1057" t="n">
+        <v>6.8</v>
+      </c>
+      <c r="F1057" t="n">
+        <v>13.73</v>
+      </c>
+      <c r="G1057" t="n">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="1058">
+      <c r="A1058" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+      <c r="B1058" t="inlineStr">
+        <is>
+          <t>QSI</t>
+        </is>
+      </c>
+      <c r="C1058" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D1058" t="n">
+        <v>1.21</v>
+      </c>
+      <c r="E1058" t="n">
+        <v>1.15</v>
+      </c>
+      <c r="F1058" t="n">
+        <v>1.33</v>
+      </c>
+      <c r="G1058" t="n">
+        <v>833</v>
+      </c>
+    </row>
+    <row r="1059">
+      <c r="A1059" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+      <c r="B1059" t="inlineStr">
+        <is>
+          <t>SCKT</t>
+        </is>
+      </c>
+      <c r="C1059" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D1059" t="n">
+        <v>0.51</v>
+      </c>
+      <c r="E1059" t="n">
+        <v>0.48</v>
+      </c>
+      <c r="F1059" t="n">
+        <v>0.58</v>
+      </c>
+      <c r="G1059" t="n">
+        <v>1510</v>
+      </c>
+    </row>
+    <row r="1060">
+      <c r="A1060" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+      <c r="B1060" t="inlineStr">
+        <is>
+          <t>VEEA</t>
+        </is>
+      </c>
+      <c r="C1060" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D1060" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="E1060" t="n">
+        <v>2.92</v>
+      </c>
+      <c r="F1060" t="n">
+        <v>4.66</v>
+      </c>
+      <c r="G1060" t="n">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="1061">
+      <c r="A1061" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+      <c r="B1061" t="inlineStr">
+        <is>
+          <t>AMSS</t>
+        </is>
+      </c>
+      <c r="C1061" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="1062">
+      <c r="A1062" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+      <c r="B1062" t="inlineStr">
+        <is>
+          <t>FNGR</t>
+        </is>
+      </c>
+      <c r="C1062" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="1063">
+      <c r="A1063" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+      <c r="B1063" t="inlineStr">
+        <is>
+          <t>SGMT</t>
+        </is>
+      </c>
+      <c r="C1063" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="1064">
+      <c r="A1064" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+      <c r="B1064" t="inlineStr">
+        <is>
+          <t>SOTK</t>
+        </is>
+      </c>
+      <c r="C1064" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="1065">
+      <c r="A1065" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+      <c r="B1065" t="inlineStr">
+        <is>
+          <t>VBIO</t>
+        </is>
+      </c>
+      <c r="C1065" t="inlineStr">
         <is>
           <t>Dropped</t>
         </is>

</xml_diff>

<commit_message>
Daily screener update: 2026-10-03
</commit_message>
<xml_diff>
--- a/screener_history.xlsx
+++ b/screener_history.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G938"/>
+  <dimension ref="A1:G942"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -21899,6 +21899,110 @@
         </is>
       </c>
       <c r="C938" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="939">
+      <c r="A939" t="inlineStr">
+        <is>
+          <t>2026-10-03</t>
+        </is>
+      </c>
+      <c r="B939" t="inlineStr">
+        <is>
+          <t>BIO-B</t>
+        </is>
+      </c>
+      <c r="C939" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D939" t="n">
+        <v>365.08</v>
+      </c>
+      <c r="E939" t="n">
+        <v>365.08</v>
+      </c>
+      <c r="F939" t="n">
+        <v>365.08</v>
+      </c>
+      <c r="G939" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="940">
+      <c r="A940" t="inlineStr">
+        <is>
+          <t>2026-10-03</t>
+        </is>
+      </c>
+      <c r="B940" t="inlineStr">
+        <is>
+          <t>EFSI</t>
+        </is>
+      </c>
+      <c r="C940" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D940" t="n">
+        <v>46.72</v>
+      </c>
+      <c r="E940" t="n">
+        <v>45</v>
+      </c>
+      <c r="F940" t="n">
+        <v>50.16</v>
+      </c>
+      <c r="G940" t="n">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="941">
+      <c r="A941" t="inlineStr">
+        <is>
+          <t>2026-10-03</t>
+        </is>
+      </c>
+      <c r="B941" t="inlineStr">
+        <is>
+          <t>TMS</t>
+        </is>
+      </c>
+      <c r="C941" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D941" t="n">
+        <v>9.359999999999999</v>
+      </c>
+      <c r="E941" t="n">
+        <v>6.96</v>
+      </c>
+      <c r="F941" t="n">
+        <v>14.16</v>
+      </c>
+      <c r="G941" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="942">
+      <c r="A942" t="inlineStr">
+        <is>
+          <t>2026-10-03</t>
+        </is>
+      </c>
+      <c r="B942" t="inlineStr">
+        <is>
+          <t>RDIB</t>
+        </is>
+      </c>
+      <c r="C942" t="inlineStr">
         <is>
           <t>Dropped</t>
         </is>
@@ -21915,7 +22019,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G1065"/>
+  <dimension ref="A1:G1074"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -46395,6 +46499,207 @@
         </is>
       </c>
       <c r="C1065" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="1066">
+      <c r="A1066" t="inlineStr">
+        <is>
+          <t>2026-10-03</t>
+        </is>
+      </c>
+      <c r="B1066" t="inlineStr">
+        <is>
+          <t>AMOD</t>
+        </is>
+      </c>
+      <c r="C1066" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D1066" t="n">
+        <v>3.97</v>
+      </c>
+      <c r="E1066" t="n">
+        <v>3.08</v>
+      </c>
+      <c r="F1066" t="n">
+        <v>5.75</v>
+      </c>
+      <c r="G1066" t="n">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="1067">
+      <c r="A1067" t="inlineStr">
+        <is>
+          <t>2026-10-03</t>
+        </is>
+      </c>
+      <c r="B1067" t="inlineStr">
+        <is>
+          <t>CYCU</t>
+        </is>
+      </c>
+      <c r="C1067" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D1067" t="n">
+        <v>3.02</v>
+      </c>
+      <c r="E1067" t="n">
+        <v>2.64</v>
+      </c>
+      <c r="F1067" t="n">
+        <v>3.78</v>
+      </c>
+      <c r="G1067" t="n">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="1068">
+      <c r="A1068" t="inlineStr">
+        <is>
+          <t>2026-10-03</t>
+        </is>
+      </c>
+      <c r="B1068" t="inlineStr">
+        <is>
+          <t>SCNX</t>
+        </is>
+      </c>
+      <c r="C1068" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D1068" t="n">
+        <v>0.21</v>
+      </c>
+      <c r="E1068" t="n">
+        <v>0.14</v>
+      </c>
+      <c r="F1068" t="n">
+        <v>0.37</v>
+      </c>
+      <c r="G1068" t="n">
+        <v>639</v>
+      </c>
+    </row>
+    <row r="1069">
+      <c r="A1069" t="inlineStr">
+        <is>
+          <t>2026-10-03</t>
+        </is>
+      </c>
+      <c r="B1069" t="inlineStr">
+        <is>
+          <t>SYNA</t>
+        </is>
+      </c>
+      <c r="C1069" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D1069" t="n">
+        <v>121.98</v>
+      </c>
+      <c r="E1069" t="n">
+        <v>119.91</v>
+      </c>
+      <c r="F1069" t="n">
+        <v>126.12</v>
+      </c>
+      <c r="G1069" t="n">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="1070">
+      <c r="A1070" t="inlineStr">
+        <is>
+          <t>2026-10-03</t>
+        </is>
+      </c>
+      <c r="B1070" t="inlineStr">
+        <is>
+          <t>AIXC</t>
+        </is>
+      </c>
+      <c r="C1070" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="1071">
+      <c r="A1071" t="inlineStr">
+        <is>
+          <t>2026-10-03</t>
+        </is>
+      </c>
+      <c r="B1071" t="inlineStr">
+        <is>
+          <t>GIPR</t>
+        </is>
+      </c>
+      <c r="C1071" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="1072">
+      <c r="A1072" t="inlineStr">
+        <is>
+          <t>2026-10-03</t>
+        </is>
+      </c>
+      <c r="B1072" t="inlineStr">
+        <is>
+          <t>NXL</t>
+        </is>
+      </c>
+      <c r="C1072" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="1073">
+      <c r="A1073" t="inlineStr">
+        <is>
+          <t>2026-10-03</t>
+        </is>
+      </c>
+      <c r="B1073" t="inlineStr">
+        <is>
+          <t>QSI</t>
+        </is>
+      </c>
+      <c r="C1073" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="1074">
+      <c r="A1074" t="inlineStr">
+        <is>
+          <t>2026-10-03</t>
+        </is>
+      </c>
+      <c r="B1074" t="inlineStr">
+        <is>
+          <t>VEEA</t>
+        </is>
+      </c>
+      <c r="C1074" t="inlineStr">
         <is>
           <t>Dropped</t>
         </is>

</xml_diff>

<commit_message>
Daily screener update: 2026-10-06
</commit_message>
<xml_diff>
--- a/screener_history.xlsx
+++ b/screener_history.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G942"/>
+  <dimension ref="A1:G971"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -22003,6 +22003,811 @@
         </is>
       </c>
       <c r="C942" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="943">
+      <c r="A943" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B943" t="inlineStr">
+        <is>
+          <t>ACVA</t>
+        </is>
+      </c>
+      <c r="C943" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D943" t="n">
+        <v>10.5</v>
+      </c>
+      <c r="E943" t="n">
+        <v>10.41</v>
+      </c>
+      <c r="F943" t="n">
+        <v>10.68</v>
+      </c>
+      <c r="G943" t="n">
+        <v>555</v>
+      </c>
+    </row>
+    <row r="944">
+      <c r="A944" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B944" t="inlineStr">
+        <is>
+          <t>AEMD</t>
+        </is>
+      </c>
+      <c r="C944" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D944" t="n">
+        <v>7.21</v>
+      </c>
+      <c r="E944" t="n">
+        <v>5.95</v>
+      </c>
+      <c r="F944" t="n">
+        <v>9.73</v>
+      </c>
+      <c r="G944" t="n">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="945">
+      <c r="A945" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B945" t="inlineStr">
+        <is>
+          <t>ALP</t>
+        </is>
+      </c>
+      <c r="C945" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D945" t="n">
+        <v>5.79</v>
+      </c>
+      <c r="E945" t="n">
+        <v>4.2</v>
+      </c>
+      <c r="F945" t="n">
+        <v>8.970000000000001</v>
+      </c>
+      <c r="G945" t="n">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="946">
+      <c r="A946" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B946" t="inlineStr">
+        <is>
+          <t>AVAT</t>
+        </is>
+      </c>
+      <c r="C946" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D946" t="n">
+        <v>2.58</v>
+      </c>
+      <c r="E946" t="n">
+        <v>1.58</v>
+      </c>
+      <c r="F946" t="n">
+        <v>4.58</v>
+      </c>
+      <c r="G946" t="n">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="947">
+      <c r="A947" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B947" t="inlineStr">
+        <is>
+          <t>BMNR</t>
+        </is>
+      </c>
+      <c r="C947" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D947" t="n">
+        <v>28.86</v>
+      </c>
+      <c r="E947" t="n">
+        <v>25.92</v>
+      </c>
+      <c r="F947" t="n">
+        <v>34.74</v>
+      </c>
+      <c r="G947" t="n">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="948">
+      <c r="A948" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B948" t="inlineStr">
+        <is>
+          <t>BNC</t>
+        </is>
+      </c>
+      <c r="C948" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D948" t="n">
+        <v>6.41</v>
+      </c>
+      <c r="E948" t="n">
+        <v>5.55</v>
+      </c>
+      <c r="F948" t="n">
+        <v>8.130000000000001</v>
+      </c>
+      <c r="G948" t="n">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="949">
+      <c r="A949" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B949" t="inlineStr">
+        <is>
+          <t>BRTX</t>
+        </is>
+      </c>
+      <c r="C949" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D949" t="n">
+        <v>2.93</v>
+      </c>
+      <c r="E949" t="n">
+        <v>2.01</v>
+      </c>
+      <c r="F949" t="n">
+        <v>4.77</v>
+      </c>
+      <c r="G949" t="n">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="950">
+      <c r="A950" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B950" t="inlineStr">
+        <is>
+          <t>COSM</t>
+        </is>
+      </c>
+      <c r="C950" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D950" t="n">
+        <v>0.48</v>
+      </c>
+      <c r="E950" t="n">
+        <v>0.33</v>
+      </c>
+      <c r="F950" t="n">
+        <v>0.78</v>
+      </c>
+      <c r="G950" t="n">
+        <v>335</v>
+      </c>
+    </row>
+    <row r="951">
+      <c r="A951" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B951" t="inlineStr">
+        <is>
+          <t>CYPH</t>
+        </is>
+      </c>
+      <c r="C951" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D951" t="n">
+        <v>4.19</v>
+      </c>
+      <c r="E951" t="n">
+        <v>2.88</v>
+      </c>
+      <c r="F951" t="n">
+        <v>6.81</v>
+      </c>
+      <c r="G951" t="n">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="952">
+      <c r="A952" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B952" t="inlineStr">
+        <is>
+          <t>DFDV</t>
+        </is>
+      </c>
+      <c r="C952" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D952" t="n">
+        <v>6.57</v>
+      </c>
+      <c r="E952" t="n">
+        <v>5.14</v>
+      </c>
+      <c r="F952" t="n">
+        <v>9.44</v>
+      </c>
+      <c r="G952" t="n">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="953">
+      <c r="A953" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B953" t="inlineStr">
+        <is>
+          <t>ETS</t>
+        </is>
+      </c>
+      <c r="C953" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D953" t="n">
+        <v>2.08</v>
+      </c>
+      <c r="E953" t="n">
+        <v>1.42</v>
+      </c>
+      <c r="F953" t="n">
+        <v>3.4</v>
+      </c>
+      <c r="G953" t="n">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="954">
+      <c r="A954" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B954" t="inlineStr">
+        <is>
+          <t>FEIM</t>
+        </is>
+      </c>
+      <c r="C954" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D954" t="n">
+        <v>89.59</v>
+      </c>
+      <c r="E954" t="n">
+        <v>81.58</v>
+      </c>
+      <c r="F954" t="n">
+        <v>105.61</v>
+      </c>
+      <c r="G954" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="955">
+      <c r="A955" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B955" t="inlineStr">
+        <is>
+          <t>FWDI</t>
+        </is>
+      </c>
+      <c r="C955" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D955" t="n">
+        <v>8.76</v>
+      </c>
+      <c r="E955" t="n">
+        <v>7.65</v>
+      </c>
+      <c r="F955" t="n">
+        <v>10.98</v>
+      </c>
+      <c r="G955" t="n">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="956">
+      <c r="A956" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B956" t="inlineStr">
+        <is>
+          <t>GTBP</t>
+        </is>
+      </c>
+      <c r="C956" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D956" t="n">
+        <v>7.28</v>
+      </c>
+      <c r="E956" t="n">
+        <v>6</v>
+      </c>
+      <c r="F956" t="n">
+        <v>9.83</v>
+      </c>
+      <c r="G956" t="n">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="957">
+      <c r="A957" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B957" t="inlineStr">
+        <is>
+          <t>HHS</t>
+        </is>
+      </c>
+      <c r="C957" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D957" t="n">
+        <v>4.67</v>
+      </c>
+      <c r="E957" t="n">
+        <v>4.51</v>
+      </c>
+      <c r="F957" t="n">
+        <v>4.99</v>
+      </c>
+      <c r="G957" t="n">
+        <v>312</v>
+      </c>
+    </row>
+    <row r="958">
+      <c r="A958" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B958" t="inlineStr">
+        <is>
+          <t>HURN</t>
+        </is>
+      </c>
+      <c r="C958" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D958" t="n">
+        <v>169.45</v>
+      </c>
+      <c r="E958" t="n">
+        <v>155.05</v>
+      </c>
+      <c r="F958" t="n">
+        <v>198.25</v>
+      </c>
+      <c r="G958" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="959">
+      <c r="A959" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B959" t="inlineStr">
+        <is>
+          <t>MU</t>
+        </is>
+      </c>
+      <c r="C959" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D959" t="n">
+        <v>1108.72</v>
+      </c>
+      <c r="E959" t="n">
+        <v>1022.9</v>
+      </c>
+      <c r="F959" t="n">
+        <v>1280.36</v>
+      </c>
+      <c r="G959" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="960">
+      <c r="A960" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B960" t="inlineStr">
+        <is>
+          <t>NFE</t>
+        </is>
+      </c>
+      <c r="C960" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D960" t="n">
+        <v>10.68</v>
+      </c>
+      <c r="E960" t="n">
+        <v>5.45</v>
+      </c>
+      <c r="F960" t="n">
+        <v>21.15</v>
+      </c>
+      <c r="G960" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="961">
+      <c r="A961" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B961" t="inlineStr">
+        <is>
+          <t>OMER</t>
+        </is>
+      </c>
+      <c r="C961" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D961" t="n">
+        <v>21.24</v>
+      </c>
+      <c r="E961" t="n">
+        <v>18.22</v>
+      </c>
+      <c r="F961" t="n">
+        <v>27.28</v>
+      </c>
+      <c r="G961" t="n">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="962">
+      <c r="A962" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B962" t="inlineStr">
+        <is>
+          <t>PRTH</t>
+        </is>
+      </c>
+      <c r="C962" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D962" t="n">
+        <v>7.82</v>
+      </c>
+      <c r="E962" t="n">
+        <v>7.76</v>
+      </c>
+      <c r="F962" t="n">
+        <v>7.94</v>
+      </c>
+      <c r="G962" t="n">
+        <v>833</v>
+      </c>
+    </row>
+    <row r="963">
+      <c r="A963" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B963" t="inlineStr">
+        <is>
+          <t>PSNL</t>
+        </is>
+      </c>
+      <c r="C963" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D963" t="n">
+        <v>16.77</v>
+      </c>
+      <c r="E963" t="n">
+        <v>16</v>
+      </c>
+      <c r="F963" t="n">
+        <v>18.31</v>
+      </c>
+      <c r="G963" t="n">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="964">
+      <c r="A964" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B964" t="inlineStr">
+        <is>
+          <t>RXT</t>
+        </is>
+      </c>
+      <c r="C964" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D964" t="n">
+        <v>4.29</v>
+      </c>
+      <c r="E964" t="n">
+        <v>3.7</v>
+      </c>
+      <c r="F964" t="n">
+        <v>5.47</v>
+      </c>
+      <c r="G964" t="n">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="965">
+      <c r="A965" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B965" t="inlineStr">
+        <is>
+          <t>SBET</t>
+        </is>
+      </c>
+      <c r="C965" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D965" t="n">
+        <v>10.4</v>
+      </c>
+      <c r="E965" t="n">
+        <v>9.23</v>
+      </c>
+      <c r="F965" t="n">
+        <v>12.74</v>
+      </c>
+      <c r="G965" t="n">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="966">
+      <c r="A966" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B966" t="inlineStr">
+        <is>
+          <t>TELA</t>
+        </is>
+      </c>
+      <c r="C966" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D966" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="E966" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="F966" t="n">
+        <v>2.3</v>
+      </c>
+      <c r="G966" t="n">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="967">
+      <c r="A967" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B967" t="inlineStr">
+        <is>
+          <t>UMC</t>
+        </is>
+      </c>
+      <c r="C967" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D967" t="n">
+        <v>26.37</v>
+      </c>
+      <c r="E967" t="n">
+        <v>23.26</v>
+      </c>
+      <c r="F967" t="n">
+        <v>32.59</v>
+      </c>
+      <c r="G967" t="n">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="968">
+      <c r="A968" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B968" t="inlineStr">
+        <is>
+          <t>VREX</t>
+        </is>
+      </c>
+      <c r="C968" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D968" t="n">
+        <v>18.51</v>
+      </c>
+      <c r="E968" t="n">
+        <v>18.42</v>
+      </c>
+      <c r="F968" t="n">
+        <v>18.69</v>
+      </c>
+      <c r="G968" t="n">
+        <v>555</v>
+      </c>
+    </row>
+    <row r="969">
+      <c r="A969" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B969" t="inlineStr">
+        <is>
+          <t>BIO-B</t>
+        </is>
+      </c>
+      <c r="C969" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="970">
+      <c r="A970" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B970" t="inlineStr">
+        <is>
+          <t>EFSI</t>
+        </is>
+      </c>
+      <c r="C970" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="971">
+      <c r="A971" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B971" t="inlineStr">
+        <is>
+          <t>TMS</t>
+        </is>
+      </c>
+      <c r="C971" t="inlineStr">
         <is>
           <t>Dropped</t>
         </is>
@@ -22019,7 +22824,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G1074"/>
+  <dimension ref="A1:G1089"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -46700,6 +47505,393 @@
         </is>
       </c>
       <c r="C1074" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="1075">
+      <c r="A1075" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B1075" t="inlineStr">
+        <is>
+          <t>ALEC</t>
+        </is>
+      </c>
+      <c r="C1075" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D1075" t="n">
+        <v>2.73</v>
+      </c>
+      <c r="E1075" t="n">
+        <v>1.96</v>
+      </c>
+      <c r="F1075" t="n">
+        <v>4.27</v>
+      </c>
+      <c r="G1075" t="n">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="1076">
+      <c r="A1076" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B1076" t="inlineStr">
+        <is>
+          <t>BEAT</t>
+        </is>
+      </c>
+      <c r="C1076" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D1076" t="n">
+        <v>0.88</v>
+      </c>
+      <c r="E1076" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="F1076" t="n">
+        <v>1.44</v>
+      </c>
+      <c r="G1076" t="n">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="1077">
+      <c r="A1077" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B1077" t="inlineStr">
+        <is>
+          <t>JAGX</t>
+        </is>
+      </c>
+      <c r="C1077" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D1077" t="n">
+        <v>4.27</v>
+      </c>
+      <c r="E1077" t="n">
+        <v>4.1</v>
+      </c>
+      <c r="F1077" t="n">
+        <v>4.61</v>
+      </c>
+      <c r="G1077" t="n">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="1078">
+      <c r="A1078" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B1078" t="inlineStr">
+        <is>
+          <t>NAUT</t>
+        </is>
+      </c>
+      <c r="C1078" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D1078" t="n">
+        <v>2.2</v>
+      </c>
+      <c r="E1078" t="n">
+        <v>1.81</v>
+      </c>
+      <c r="F1078" t="n">
+        <v>2.98</v>
+      </c>
+      <c r="G1078" t="n">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="1079">
+      <c r="A1079" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B1079" t="inlineStr">
+        <is>
+          <t>PCVX</t>
+        </is>
+      </c>
+      <c r="C1079" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D1079" t="n">
+        <v>90.75</v>
+      </c>
+      <c r="E1079" t="n">
+        <v>71.59999999999999</v>
+      </c>
+      <c r="F1079" t="n">
+        <v>129.05</v>
+      </c>
+      <c r="G1079" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="1080">
+      <c r="A1080" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B1080" t="inlineStr">
+        <is>
+          <t>PTC</t>
+        </is>
+      </c>
+      <c r="C1080" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D1080" t="n">
+        <v>196</v>
+      </c>
+      <c r="E1080" t="n">
+        <v>192.07</v>
+      </c>
+      <c r="F1080" t="n">
+        <v>203.86</v>
+      </c>
+      <c r="G1080" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="1081">
+      <c r="A1081" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B1081" t="inlineStr">
+        <is>
+          <t>RXO</t>
+        </is>
+      </c>
+      <c r="C1081" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D1081" t="n">
+        <v>29.04</v>
+      </c>
+      <c r="E1081" t="n">
+        <v>28.03</v>
+      </c>
+      <c r="F1081" t="n">
+        <v>31.06</v>
+      </c>
+      <c r="G1081" t="n">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="1082">
+      <c r="A1082" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B1082" t="inlineStr">
+        <is>
+          <t>SID</t>
+        </is>
+      </c>
+      <c r="C1082" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D1082" t="n">
+        <v>1.33</v>
+      </c>
+      <c r="E1082" t="n">
+        <v>1.22</v>
+      </c>
+      <c r="F1082" t="n">
+        <v>1.56</v>
+      </c>
+      <c r="G1082" t="n">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="1083">
+      <c r="A1083" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B1083" t="inlineStr">
+        <is>
+          <t>SXTP</t>
+        </is>
+      </c>
+      <c r="C1083" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D1083" t="n">
+        <v>1.56</v>
+      </c>
+      <c r="E1083" t="n">
+        <v>1.36</v>
+      </c>
+      <c r="F1083" t="n">
+        <v>1.96</v>
+      </c>
+      <c r="G1083" t="n">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="1084">
+      <c r="A1084" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B1084" t="inlineStr">
+        <is>
+          <t>VEEA</t>
+        </is>
+      </c>
+      <c r="C1084" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D1084" t="n">
+        <v>5.43</v>
+      </c>
+      <c r="E1084" t="n">
+        <v>4.66</v>
+      </c>
+      <c r="F1084" t="n">
+        <v>6.97</v>
+      </c>
+      <c r="G1084" t="n">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="1085">
+      <c r="A1085" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B1085" t="inlineStr">
+        <is>
+          <t>XP</t>
+        </is>
+      </c>
+      <c r="C1085" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D1085" t="n">
+        <v>28.17</v>
+      </c>
+      <c r="E1085" t="n">
+        <v>25.84</v>
+      </c>
+      <c r="F1085" t="n">
+        <v>32.84</v>
+      </c>
+      <c r="G1085" t="n">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="1086">
+      <c r="A1086" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B1086" t="inlineStr">
+        <is>
+          <t>CYCU</t>
+        </is>
+      </c>
+      <c r="C1086" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="1087">
+      <c r="A1087" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B1087" t="inlineStr">
+        <is>
+          <t>SCKT</t>
+        </is>
+      </c>
+      <c r="C1087" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="1088">
+      <c r="A1088" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B1088" t="inlineStr">
+        <is>
+          <t>SCNX</t>
+        </is>
+      </c>
+      <c r="C1088" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="1089">
+      <c r="A1089" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B1089" t="inlineStr">
+        <is>
+          <t>SYNA</t>
+        </is>
+      </c>
+      <c r="C1089" t="inlineStr">
         <is>
           <t>Dropped</t>
         </is>

</xml_diff>

<commit_message>
Daily screener update: 2026-10-07
</commit_message>
<xml_diff>
--- a/screener_history.xlsx
+++ b/screener_history.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G971"/>
+  <dimension ref="A1:G996"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -22808,6 +22808,467 @@
         </is>
       </c>
       <c r="C971" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="972">
+      <c r="A972" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B972" t="inlineStr">
+        <is>
+          <t>OESX</t>
+        </is>
+      </c>
+      <c r="C972" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D972" t="n">
+        <v>31.65</v>
+      </c>
+      <c r="E972" t="n">
+        <v>28.1</v>
+      </c>
+      <c r="F972" t="n">
+        <v>38.75</v>
+      </c>
+      <c r="G972" t="n">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="973">
+      <c r="A973" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B973" t="inlineStr">
+        <is>
+          <t>REFR</t>
+        </is>
+      </c>
+      <c r="C973" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D973" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="E973" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="F973" t="n">
+        <v>1.25</v>
+      </c>
+      <c r="G973" t="n">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="974">
+      <c r="A974" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B974" t="inlineStr">
+        <is>
+          <t>TISI</t>
+        </is>
+      </c>
+      <c r="C974" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D974" t="n">
+        <v>29.57</v>
+      </c>
+      <c r="E974" t="n">
+        <v>27.12</v>
+      </c>
+      <c r="F974" t="n">
+        <v>34.47</v>
+      </c>
+      <c r="G974" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="975">
+      <c r="A975" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B975" t="inlineStr">
+        <is>
+          <t>ACVA</t>
+        </is>
+      </c>
+      <c r="C975" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="976">
+      <c r="A976" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B976" t="inlineStr">
+        <is>
+          <t>ALP</t>
+        </is>
+      </c>
+      <c r="C976" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="977">
+      <c r="A977" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B977" t="inlineStr">
+        <is>
+          <t>AVAT</t>
+        </is>
+      </c>
+      <c r="C977" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="978">
+      <c r="A978" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B978" t="inlineStr">
+        <is>
+          <t>BMNR</t>
+        </is>
+      </c>
+      <c r="C978" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="979">
+      <c r="A979" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B979" t="inlineStr">
+        <is>
+          <t>BNC</t>
+        </is>
+      </c>
+      <c r="C979" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="980">
+      <c r="A980" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B980" t="inlineStr">
+        <is>
+          <t>BRTX</t>
+        </is>
+      </c>
+      <c r="C980" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="981">
+      <c r="A981" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B981" t="inlineStr">
+        <is>
+          <t>COSM</t>
+        </is>
+      </c>
+      <c r="C981" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="982">
+      <c r="A982" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B982" t="inlineStr">
+        <is>
+          <t>CYPH</t>
+        </is>
+      </c>
+      <c r="C982" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="983">
+      <c r="A983" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B983" t="inlineStr">
+        <is>
+          <t>DFDV</t>
+        </is>
+      </c>
+      <c r="C983" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="984">
+      <c r="A984" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B984" t="inlineStr">
+        <is>
+          <t>ETS</t>
+        </is>
+      </c>
+      <c r="C984" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="985">
+      <c r="A985" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B985" t="inlineStr">
+        <is>
+          <t>FEIM</t>
+        </is>
+      </c>
+      <c r="C985" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="986">
+      <c r="A986" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B986" t="inlineStr">
+        <is>
+          <t>GTBP</t>
+        </is>
+      </c>
+      <c r="C986" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="987">
+      <c r="A987" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B987" t="inlineStr">
+        <is>
+          <t>HHS</t>
+        </is>
+      </c>
+      <c r="C987" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="988">
+      <c r="A988" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B988" t="inlineStr">
+        <is>
+          <t>HURN</t>
+        </is>
+      </c>
+      <c r="C988" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="989">
+      <c r="A989" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B989" t="inlineStr">
+        <is>
+          <t>NFE</t>
+        </is>
+      </c>
+      <c r="C989" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="990">
+      <c r="A990" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B990" t="inlineStr">
+        <is>
+          <t>OMER</t>
+        </is>
+      </c>
+      <c r="C990" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="991">
+      <c r="A991" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B991" t="inlineStr">
+        <is>
+          <t>PRTH</t>
+        </is>
+      </c>
+      <c r="C991" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="992">
+      <c r="A992" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B992" t="inlineStr">
+        <is>
+          <t>PSNL</t>
+        </is>
+      </c>
+      <c r="C992" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="993">
+      <c r="A993" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B993" t="inlineStr">
+        <is>
+          <t>RXT</t>
+        </is>
+      </c>
+      <c r="C993" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="994">
+      <c r="A994" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B994" t="inlineStr">
+        <is>
+          <t>TELA</t>
+        </is>
+      </c>
+      <c r="C994" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="995">
+      <c r="A995" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B995" t="inlineStr">
+        <is>
+          <t>UMC</t>
+        </is>
+      </c>
+      <c r="C995" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="996">
+      <c r="A996" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B996" t="inlineStr">
+        <is>
+          <t>VREX</t>
+        </is>
+      </c>
+      <c r="C996" t="inlineStr">
         <is>
           <t>Dropped</t>
         </is>
@@ -22824,7 +23285,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G1089"/>
+  <dimension ref="A1:G1107"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -47892,6 +48353,396 @@
         </is>
       </c>
       <c r="C1089" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="1090">
+      <c r="A1090" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B1090" t="inlineStr">
+        <is>
+          <t>AIFA</t>
+        </is>
+      </c>
+      <c r="C1090" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D1090" t="n">
+        <v>7.47</v>
+      </c>
+      <c r="E1090" t="n">
+        <v>6.7</v>
+      </c>
+      <c r="F1090" t="n">
+        <v>9</v>
+      </c>
+      <c r="G1090" t="n">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="1091">
+      <c r="A1091" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B1091" t="inlineStr">
+        <is>
+          <t>APOG</t>
+        </is>
+      </c>
+      <c r="C1091" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D1091" t="n">
+        <v>42.74</v>
+      </c>
+      <c r="E1091" t="n">
+        <v>37.85</v>
+      </c>
+      <c r="F1091" t="n">
+        <v>52.52</v>
+      </c>
+      <c r="G1091" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="1092">
+      <c r="A1092" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B1092" t="inlineStr">
+        <is>
+          <t>CIRC</t>
+        </is>
+      </c>
+      <c r="C1092" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D1092" t="n">
+        <v>0.64</v>
+      </c>
+      <c r="E1092" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="F1092" t="n">
+        <v>1.04</v>
+      </c>
+      <c r="G1092" t="n">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="1093">
+      <c r="A1093" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B1093" t="inlineStr">
+        <is>
+          <t>IPDN</t>
+        </is>
+      </c>
+      <c r="C1093" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D1093" t="n">
+        <v>6.78</v>
+      </c>
+      <c r="E1093" t="n">
+        <v>4.09</v>
+      </c>
+      <c r="F1093" t="n">
+        <v>12.16</v>
+      </c>
+      <c r="G1093" t="n">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="1094">
+      <c r="A1094" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B1094" t="inlineStr">
+        <is>
+          <t>OLOX</t>
+        </is>
+      </c>
+      <c r="C1094" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D1094" t="n">
+        <v>1.54</v>
+      </c>
+      <c r="E1094" t="n">
+        <v>1.25</v>
+      </c>
+      <c r="F1094" t="n">
+        <v>2.12</v>
+      </c>
+      <c r="G1094" t="n">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="1095">
+      <c r="A1095" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B1095" t="inlineStr">
+        <is>
+          <t>OPCH</t>
+        </is>
+      </c>
+      <c r="C1095" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D1095" t="n">
+        <v>31.08</v>
+      </c>
+      <c r="E1095" t="n">
+        <v>30.97</v>
+      </c>
+      <c r="F1095" t="n">
+        <v>31.31</v>
+      </c>
+      <c r="G1095" t="n">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="1096">
+      <c r="A1096" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B1096" t="inlineStr">
+        <is>
+          <t>PRME</t>
+        </is>
+      </c>
+      <c r="C1096" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D1096" t="n">
+        <v>3.7</v>
+      </c>
+      <c r="E1096" t="n">
+        <v>3.26</v>
+      </c>
+      <c r="F1096" t="n">
+        <v>4.58</v>
+      </c>
+      <c r="G1096" t="n">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="1097">
+      <c r="A1097" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B1097" t="inlineStr">
+        <is>
+          <t>ALEC</t>
+        </is>
+      </c>
+      <c r="C1097" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="1098">
+      <c r="A1098" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B1098" t="inlineStr">
+        <is>
+          <t>AMOD</t>
+        </is>
+      </c>
+      <c r="C1098" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="1099">
+      <c r="A1099" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B1099" t="inlineStr">
+        <is>
+          <t>BEAT</t>
+        </is>
+      </c>
+      <c r="C1099" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="1100">
+      <c r="A1100" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B1100" t="inlineStr">
+        <is>
+          <t>NAUT</t>
+        </is>
+      </c>
+      <c r="C1100" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="1101">
+      <c r="A1101" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B1101" t="inlineStr">
+        <is>
+          <t>PCVX</t>
+        </is>
+      </c>
+      <c r="C1101" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="1102">
+      <c r="A1102" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B1102" t="inlineStr">
+        <is>
+          <t>PTC</t>
+        </is>
+      </c>
+      <c r="C1102" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="1103">
+      <c r="A1103" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B1103" t="inlineStr">
+        <is>
+          <t>RXO</t>
+        </is>
+      </c>
+      <c r="C1103" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="1104">
+      <c r="A1104" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B1104" t="inlineStr">
+        <is>
+          <t>SID</t>
+        </is>
+      </c>
+      <c r="C1104" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="1105">
+      <c r="A1105" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B1105" t="inlineStr">
+        <is>
+          <t>SXTP</t>
+        </is>
+      </c>
+      <c r="C1105" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="1106">
+      <c r="A1106" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B1106" t="inlineStr">
+        <is>
+          <t>VEEA</t>
+        </is>
+      </c>
+      <c r="C1106" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="1107">
+      <c r="A1107" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B1107" t="inlineStr">
+        <is>
+          <t>XP</t>
+        </is>
+      </c>
+      <c r="C1107" t="inlineStr">
         <is>
           <t>Dropped</t>
         </is>

</xml_diff>

<commit_message>
Daily screener update: 2026-10-08
</commit_message>
<xml_diff>
--- a/screener_history.xlsx
+++ b/screener_history.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G996"/>
+  <dimension ref="A1:G1005"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -23269,6 +23269,183 @@
         </is>
       </c>
       <c r="C996" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="997">
+      <c r="A997" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B997" t="inlineStr">
+        <is>
+          <t>BIO-B</t>
+        </is>
+      </c>
+      <c r="C997" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D997" t="n">
+        <v>365.08</v>
+      </c>
+      <c r="E997" t="n">
+        <v>365.08</v>
+      </c>
+      <c r="F997" t="n">
+        <v>365.08</v>
+      </c>
+      <c r="G997" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="998">
+      <c r="A998" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B998" t="inlineStr">
+        <is>
+          <t>EFSI</t>
+        </is>
+      </c>
+      <c r="C998" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D998" t="n">
+        <v>46.39</v>
+      </c>
+      <c r="E998" t="n">
+        <v>45</v>
+      </c>
+      <c r="F998" t="n">
+        <v>49.17</v>
+      </c>
+      <c r="G998" t="n">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="999">
+      <c r="A999" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B999" t="inlineStr">
+        <is>
+          <t>AEMD</t>
+        </is>
+      </c>
+      <c r="C999" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="1000">
+      <c r="A1000" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B1000" t="inlineStr">
+        <is>
+          <t>FWDI</t>
+        </is>
+      </c>
+      <c r="C1000" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="1001">
+      <c r="A1001" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B1001" t="inlineStr">
+        <is>
+          <t>MU</t>
+        </is>
+      </c>
+      <c r="C1001" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="1002">
+      <c r="A1002" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B1002" t="inlineStr">
+        <is>
+          <t>OESX</t>
+        </is>
+      </c>
+      <c r="C1002" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="1003">
+      <c r="A1003" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B1003" t="inlineStr">
+        <is>
+          <t>REFR</t>
+        </is>
+      </c>
+      <c r="C1003" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="1004">
+      <c r="A1004" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B1004" t="inlineStr">
+        <is>
+          <t>SBET</t>
+        </is>
+      </c>
+      <c r="C1004" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="1005">
+      <c r="A1005" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B1005" t="inlineStr">
+        <is>
+          <t>TISI</t>
+        </is>
+      </c>
+      <c r="C1005" t="inlineStr">
         <is>
           <t>Dropped</t>
         </is>
@@ -23285,7 +23462,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G1107"/>
+  <dimension ref="A1:G1119"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -48743,6 +48920,258 @@
         </is>
       </c>
       <c r="C1107" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="1108">
+      <c r="A1108" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B1108" t="inlineStr">
+        <is>
+          <t>BFRG</t>
+        </is>
+      </c>
+      <c r="C1108" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D1108" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="E1108" t="n">
+        <v>0.66</v>
+      </c>
+      <c r="F1108" t="n">
+        <v>1.07</v>
+      </c>
+      <c r="G1108" t="n">
+        <v>359</v>
+      </c>
+    </row>
+    <row r="1109">
+      <c r="A1109" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B1109" t="inlineStr">
+        <is>
+          <t>GIPR</t>
+        </is>
+      </c>
+      <c r="C1109" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D1109" t="n">
+        <v>0.57</v>
+      </c>
+      <c r="E1109" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="F1109" t="n">
+        <v>0.8100000000000001</v>
+      </c>
+      <c r="G1109" t="n">
+        <v>416</v>
+      </c>
+    </row>
+    <row r="1110">
+      <c r="A1110" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B1110" t="inlineStr">
+        <is>
+          <t>LPCN</t>
+        </is>
+      </c>
+      <c r="C1110" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D1110" t="n">
+        <v>3.14</v>
+      </c>
+      <c r="E1110" t="n">
+        <v>2.07</v>
+      </c>
+      <c r="F1110" t="n">
+        <v>5.28</v>
+      </c>
+      <c r="G1110" t="n">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="1111">
+      <c r="A1111" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B1111" t="inlineStr">
+        <is>
+          <t>QETA</t>
+        </is>
+      </c>
+      <c r="C1111" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D1111" t="n">
+        <v>15.5</v>
+      </c>
+      <c r="E1111" t="n">
+        <v>12.21</v>
+      </c>
+      <c r="F1111" t="n">
+        <v>22.08</v>
+      </c>
+      <c r="G1111" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="1112">
+      <c r="A1112" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B1112" t="inlineStr">
+        <is>
+          <t>AIFA</t>
+        </is>
+      </c>
+      <c r="C1112" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="1113">
+      <c r="A1113" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B1113" t="inlineStr">
+        <is>
+          <t>APOG</t>
+        </is>
+      </c>
+      <c r="C1113" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="1114">
+      <c r="A1114" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B1114" t="inlineStr">
+        <is>
+          <t>CIRC</t>
+        </is>
+      </c>
+      <c r="C1114" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="1115">
+      <c r="A1115" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B1115" t="inlineStr">
+        <is>
+          <t>IPDN</t>
+        </is>
+      </c>
+      <c r="C1115" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="1116">
+      <c r="A1116" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B1116" t="inlineStr">
+        <is>
+          <t>JAGX</t>
+        </is>
+      </c>
+      <c r="C1116" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="1117">
+      <c r="A1117" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B1117" t="inlineStr">
+        <is>
+          <t>OLOX</t>
+        </is>
+      </c>
+      <c r="C1117" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="1118">
+      <c r="A1118" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B1118" t="inlineStr">
+        <is>
+          <t>OPCH</t>
+        </is>
+      </c>
+      <c r="C1118" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="1119">
+      <c r="A1119" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B1119" t="inlineStr">
+        <is>
+          <t>PRME</t>
+        </is>
+      </c>
+      <c r="C1119" t="inlineStr">
         <is>
           <t>Dropped</t>
         </is>

</xml_diff>

<commit_message>
Daily screener update: 2026-10-09
</commit_message>
<xml_diff>
--- a/screener_history.xlsx
+++ b/screener_history.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G1005"/>
+  <dimension ref="A1:G1020"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -23446,6 +23446,417 @@
         </is>
       </c>
       <c r="C1005" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="1006">
+      <c r="A1006" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="B1006" t="inlineStr">
+        <is>
+          <t>BALY</t>
+        </is>
+      </c>
+      <c r="C1006" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D1006" t="n">
+        <v>14.51</v>
+      </c>
+      <c r="E1006" t="n">
+        <v>13.38</v>
+      </c>
+      <c r="F1006" t="n">
+        <v>16.77</v>
+      </c>
+      <c r="G1006" t="n">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="1007">
+      <c r="A1007" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="B1007" t="inlineStr">
+        <is>
+          <t>CDNA</t>
+        </is>
+      </c>
+      <c r="C1007" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D1007" t="n">
+        <v>72.51000000000001</v>
+      </c>
+      <c r="E1007" t="n">
+        <v>60.51</v>
+      </c>
+      <c r="F1007" t="n">
+        <v>96.51000000000001</v>
+      </c>
+      <c r="G1007" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="1008">
+      <c r="A1008" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="B1008" t="inlineStr">
+        <is>
+          <t>EMBC</t>
+        </is>
+      </c>
+      <c r="C1008" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D1008" t="n">
+        <v>6.16</v>
+      </c>
+      <c r="E1008" t="n">
+        <v>5.49</v>
+      </c>
+      <c r="F1008" t="n">
+        <v>7.5</v>
+      </c>
+      <c r="G1008" t="n">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="1009">
+      <c r="A1009" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="B1009" t="inlineStr">
+        <is>
+          <t>FIRY</t>
+        </is>
+      </c>
+      <c r="C1009" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D1009" t="n">
+        <v>13</v>
+      </c>
+      <c r="E1009" t="n">
+        <v>11.61</v>
+      </c>
+      <c r="F1009" t="n">
+        <v>15.77</v>
+      </c>
+      <c r="G1009" t="n">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="1010">
+      <c r="A1010" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="B1010" t="inlineStr">
+        <is>
+          <t>HHS</t>
+        </is>
+      </c>
+      <c r="C1010" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D1010" t="n">
+        <v>4.67</v>
+      </c>
+      <c r="E1010" t="n">
+        <v>4.38</v>
+      </c>
+      <c r="F1010" t="n">
+        <v>5.25</v>
+      </c>
+      <c r="G1010" t="n">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="1011">
+      <c r="A1011" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="B1011" t="inlineStr">
+        <is>
+          <t>MNTK</t>
+        </is>
+      </c>
+      <c r="C1011" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D1011" t="n">
+        <v>3.28</v>
+      </c>
+      <c r="E1011" t="n">
+        <v>2.6</v>
+      </c>
+      <c r="F1011" t="n">
+        <v>4.64</v>
+      </c>
+      <c r="G1011" t="n">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="1012">
+      <c r="A1012" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="B1012" t="inlineStr">
+        <is>
+          <t>MYGN</t>
+        </is>
+      </c>
+      <c r="C1012" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D1012" t="n">
+        <v>4.83</v>
+      </c>
+      <c r="E1012" t="n">
+        <v>4.05</v>
+      </c>
+      <c r="F1012" t="n">
+        <v>6.39</v>
+      </c>
+      <c r="G1012" t="n">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="1013">
+      <c r="A1013" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="B1013" t="inlineStr">
+        <is>
+          <t>NCPL</t>
+        </is>
+      </c>
+      <c r="C1013" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D1013" t="n">
+        <v>1.86</v>
+      </c>
+      <c r="E1013" t="n">
+        <v>1.07</v>
+      </c>
+      <c r="F1013" t="n">
+        <v>3.44</v>
+      </c>
+      <c r="G1013" t="n">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="1014">
+      <c r="A1014" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="B1014" t="inlineStr">
+        <is>
+          <t>PRTH</t>
+        </is>
+      </c>
+      <c r="C1014" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D1014" t="n">
+        <v>7.8</v>
+      </c>
+      <c r="E1014" t="n">
+        <v>7.76</v>
+      </c>
+      <c r="F1014" t="n">
+        <v>7.88</v>
+      </c>
+      <c r="G1014" t="n">
+        <v>1250</v>
+      </c>
+    </row>
+    <row r="1015">
+      <c r="A1015" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="B1015" t="inlineStr">
+        <is>
+          <t>SRFM</t>
+        </is>
+      </c>
+      <c r="C1015" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D1015" t="n">
+        <v>1.34</v>
+      </c>
+      <c r="E1015" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="F1015" t="n">
+        <v>2.32</v>
+      </c>
+      <c r="G1015" t="n">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="1016">
+      <c r="A1016" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="B1016" t="inlineStr">
+        <is>
+          <t>SVRN</t>
+        </is>
+      </c>
+      <c r="C1016" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D1016" t="n">
+        <v>74.73999999999999</v>
+      </c>
+      <c r="E1016" t="n">
+        <v>35.77</v>
+      </c>
+      <c r="F1016" t="n">
+        <v>152.68</v>
+      </c>
+      <c r="G1016" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1017">
+      <c r="A1017" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="B1017" t="inlineStr">
+        <is>
+          <t>TKNO</t>
+        </is>
+      </c>
+      <c r="C1017" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D1017" t="n">
+        <v>9.48</v>
+      </c>
+      <c r="E1017" t="n">
+        <v>8.34</v>
+      </c>
+      <c r="F1017" t="n">
+        <v>11.76</v>
+      </c>
+      <c r="G1017" t="n">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="1018">
+      <c r="A1018" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="B1018" t="inlineStr">
+        <is>
+          <t>XGN</t>
+        </is>
+      </c>
+      <c r="C1018" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D1018" t="n">
+        <v>8.890000000000001</v>
+      </c>
+      <c r="E1018" t="n">
+        <v>7.78</v>
+      </c>
+      <c r="F1018" t="n">
+        <v>11.11</v>
+      </c>
+      <c r="G1018" t="n">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="1019">
+      <c r="A1019" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="B1019" t="inlineStr">
+        <is>
+          <t>BIO-B</t>
+        </is>
+      </c>
+      <c r="C1019" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="1020">
+      <c r="A1020" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="B1020" t="inlineStr">
+        <is>
+          <t>EFSI</t>
+        </is>
+      </c>
+      <c r="C1020" t="inlineStr">
         <is>
           <t>Dropped</t>
         </is>
@@ -23462,7 +23873,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G1119"/>
+  <dimension ref="A1:G1133"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -49172,6 +49583,364 @@
         </is>
       </c>
       <c r="C1119" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="1120">
+      <c r="A1120" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="B1120" t="inlineStr">
+        <is>
+          <t>FLYE</t>
+        </is>
+      </c>
+      <c r="C1120" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D1120" t="n">
+        <v>3.47</v>
+      </c>
+      <c r="E1120" t="n">
+        <v>1.95</v>
+      </c>
+      <c r="F1120" t="n">
+        <v>6.51</v>
+      </c>
+      <c r="G1120" t="n">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="1121">
+      <c r="A1121" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="B1121" t="inlineStr">
+        <is>
+          <t>HAE</t>
+        </is>
+      </c>
+      <c r="C1121" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D1121" t="n">
+        <v>116.85</v>
+      </c>
+      <c r="E1121" t="n">
+        <v>111.66</v>
+      </c>
+      <c r="F1121" t="n">
+        <v>127.23</v>
+      </c>
+      <c r="G1121" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="1122">
+      <c r="A1122" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="B1122" t="inlineStr">
+        <is>
+          <t>HELE</t>
+        </is>
+      </c>
+      <c r="C1122" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D1122" t="n">
+        <v>31.94</v>
+      </c>
+      <c r="E1122" t="n">
+        <v>26.2</v>
+      </c>
+      <c r="F1122" t="n">
+        <v>43.42</v>
+      </c>
+      <c r="G1122" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="1123">
+      <c r="A1123" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="B1123" t="inlineStr">
+        <is>
+          <t>HYPR</t>
+        </is>
+      </c>
+      <c r="C1123" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D1123" t="n">
+        <v>0.99</v>
+      </c>
+      <c r="E1123" t="n">
+        <v>0.84</v>
+      </c>
+      <c r="F1123" t="n">
+        <v>1.29</v>
+      </c>
+      <c r="G1123" t="n">
+        <v>334</v>
+      </c>
+    </row>
+    <row r="1124">
+      <c r="A1124" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="B1124" t="inlineStr">
+        <is>
+          <t>IPW</t>
+        </is>
+      </c>
+      <c r="C1124" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D1124" t="n">
+        <v>1.41</v>
+      </c>
+      <c r="E1124" t="n">
+        <v>0.92</v>
+      </c>
+      <c r="F1124" t="n">
+        <v>2.39</v>
+      </c>
+      <c r="G1124" t="n">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="1125">
+      <c r="A1125" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="B1125" t="inlineStr">
+        <is>
+          <t>OLB</t>
+        </is>
+      </c>
+      <c r="C1125" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D1125" t="n">
+        <v>0.57</v>
+      </c>
+      <c r="E1125" t="n">
+        <v>0.46</v>
+      </c>
+      <c r="F1125" t="n">
+        <v>0.78</v>
+      </c>
+      <c r="G1125" t="n">
+        <v>464</v>
+      </c>
+    </row>
+    <row r="1126">
+      <c r="A1126" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="B1126" t="inlineStr">
+        <is>
+          <t>PCRX</t>
+        </is>
+      </c>
+      <c r="C1126" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D1126" t="n">
+        <v>36.33</v>
+      </c>
+      <c r="E1126" t="n">
+        <v>36.27</v>
+      </c>
+      <c r="F1126" t="n">
+        <v>36.45</v>
+      </c>
+      <c r="G1126" t="n">
+        <v>833</v>
+      </c>
+    </row>
+    <row r="1127">
+      <c r="A1127" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="B1127" t="inlineStr">
+        <is>
+          <t>PROF</t>
+        </is>
+      </c>
+      <c r="C1127" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D1127" t="n">
+        <v>6.53</v>
+      </c>
+      <c r="E1127" t="n">
+        <v>6.04</v>
+      </c>
+      <c r="F1127" t="n">
+        <v>7.5</v>
+      </c>
+      <c r="G1127" t="n">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="1128">
+      <c r="A1128" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="B1128" t="inlineStr">
+        <is>
+          <t>VHUB</t>
+        </is>
+      </c>
+      <c r="C1128" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D1128" t="n">
+        <v>0.53</v>
+      </c>
+      <c r="E1128" t="n">
+        <v>0.39</v>
+      </c>
+      <c r="F1128" t="n">
+        <v>0.8100000000000001</v>
+      </c>
+      <c r="G1128" t="n">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="1129">
+      <c r="A1129" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="B1129" t="inlineStr">
+        <is>
+          <t>WOLF</t>
+        </is>
+      </c>
+      <c r="C1129" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D1129" t="n">
+        <v>35.94</v>
+      </c>
+      <c r="E1129" t="n">
+        <v>29.52</v>
+      </c>
+      <c r="F1129" t="n">
+        <v>48.78</v>
+      </c>
+      <c r="G1129" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="1130">
+      <c r="A1130" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="B1130" t="inlineStr">
+        <is>
+          <t>BFRG</t>
+        </is>
+      </c>
+      <c r="C1130" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="1131">
+      <c r="A1131" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="B1131" t="inlineStr">
+        <is>
+          <t>GIPR</t>
+        </is>
+      </c>
+      <c r="C1131" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="1132">
+      <c r="A1132" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="B1132" t="inlineStr">
+        <is>
+          <t>LPCN</t>
+        </is>
+      </c>
+      <c r="C1132" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="1133">
+      <c r="A1133" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="B1133" t="inlineStr">
+        <is>
+          <t>QETA</t>
+        </is>
+      </c>
+      <c r="C1133" t="inlineStr">
         <is>
           <t>Dropped</t>
         </is>

</xml_diff>

<commit_message>
Daily screener update: 2026-10-10
</commit_message>
<xml_diff>
--- a/screener_history.xlsx
+++ b/screener_history.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G1020"/>
+  <dimension ref="A1:G1034"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -23857,6 +23857,256 @@
         </is>
       </c>
       <c r="C1020" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="1021">
+      <c r="A1021" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="B1021" t="inlineStr">
+        <is>
+          <t>BIO-B</t>
+        </is>
+      </c>
+      <c r="C1021" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D1021" t="n">
+        <v>365.08</v>
+      </c>
+      <c r="E1021" t="n">
+        <v>365.08</v>
+      </c>
+      <c r="F1021" t="n">
+        <v>365.08</v>
+      </c>
+      <c r="G1021" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="1022">
+      <c r="A1022" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="B1022" t="inlineStr">
+        <is>
+          <t>BALY</t>
+        </is>
+      </c>
+      <c r="C1022" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="1023">
+      <c r="A1023" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="B1023" t="inlineStr">
+        <is>
+          <t>CDNA</t>
+        </is>
+      </c>
+      <c r="C1023" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="1024">
+      <c r="A1024" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="B1024" t="inlineStr">
+        <is>
+          <t>EMBC</t>
+        </is>
+      </c>
+      <c r="C1024" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="1025">
+      <c r="A1025" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="B1025" t="inlineStr">
+        <is>
+          <t>FIRY</t>
+        </is>
+      </c>
+      <c r="C1025" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="1026">
+      <c r="A1026" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="B1026" t="inlineStr">
+        <is>
+          <t>HHS</t>
+        </is>
+      </c>
+      <c r="C1026" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="1027">
+      <c r="A1027" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="B1027" t="inlineStr">
+        <is>
+          <t>MNTK</t>
+        </is>
+      </c>
+      <c r="C1027" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="1028">
+      <c r="A1028" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="B1028" t="inlineStr">
+        <is>
+          <t>MYGN</t>
+        </is>
+      </c>
+      <c r="C1028" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="1029">
+      <c r="A1029" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="B1029" t="inlineStr">
+        <is>
+          <t>NCPL</t>
+        </is>
+      </c>
+      <c r="C1029" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="1030">
+      <c r="A1030" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="B1030" t="inlineStr">
+        <is>
+          <t>PRTH</t>
+        </is>
+      </c>
+      <c r="C1030" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="1031">
+      <c r="A1031" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="B1031" t="inlineStr">
+        <is>
+          <t>SRFM</t>
+        </is>
+      </c>
+      <c r="C1031" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="1032">
+      <c r="A1032" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="B1032" t="inlineStr">
+        <is>
+          <t>SVRN</t>
+        </is>
+      </c>
+      <c r="C1032" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="1033">
+      <c r="A1033" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="B1033" t="inlineStr">
+        <is>
+          <t>TKNO</t>
+        </is>
+      </c>
+      <c r="C1033" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="1034">
+      <c r="A1034" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="B1034" t="inlineStr">
+        <is>
+          <t>XGN</t>
+        </is>
+      </c>
+      <c r="C1034" t="inlineStr">
         <is>
           <t>Dropped</t>
         </is>
@@ -23873,7 +24123,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G1133"/>
+  <dimension ref="A1:G1146"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -49941,6 +50191,275 @@
         </is>
       </c>
       <c r="C1133" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="1134">
+      <c r="A1134" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="B1134" t="inlineStr">
+        <is>
+          <t>HUM</t>
+        </is>
+      </c>
+      <c r="C1134" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D1134" t="n">
+        <v>453.5</v>
+      </c>
+      <c r="E1134" t="n">
+        <v>428.45</v>
+      </c>
+      <c r="F1134" t="n">
+        <v>503.61</v>
+      </c>
+      <c r="G1134" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1135">
+      <c r="A1135" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="B1135" t="inlineStr">
+        <is>
+          <t>QETA</t>
+        </is>
+      </c>
+      <c r="C1135" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D1135" t="n">
+        <v>14.22</v>
+      </c>
+      <c r="E1135" t="n">
+        <v>12.01</v>
+      </c>
+      <c r="F1135" t="n">
+        <v>18.64</v>
+      </c>
+      <c r="G1135" t="n">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="1136">
+      <c r="A1136" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="B1136" t="inlineStr">
+        <is>
+          <t>VEEA</t>
+        </is>
+      </c>
+      <c r="C1136" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D1136" t="n">
+        <v>6.04</v>
+      </c>
+      <c r="E1136" t="n">
+        <v>5.3</v>
+      </c>
+      <c r="F1136" t="n">
+        <v>7.52</v>
+      </c>
+      <c r="G1136" t="n">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="1137">
+      <c r="A1137" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="B1137" t="inlineStr">
+        <is>
+          <t>VIVK</t>
+        </is>
+      </c>
+      <c r="C1137" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D1137" t="n">
+        <v>8.300000000000001</v>
+      </c>
+      <c r="E1137" t="n">
+        <v>3.66</v>
+      </c>
+      <c r="F1137" t="n">
+        <v>17.58</v>
+      </c>
+      <c r="G1137" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="1138">
+      <c r="A1138" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="B1138" t="inlineStr">
+        <is>
+          <t>FLYE</t>
+        </is>
+      </c>
+      <c r="C1138" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="1139">
+      <c r="A1139" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="B1139" t="inlineStr">
+        <is>
+          <t>HAE</t>
+        </is>
+      </c>
+      <c r="C1139" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="1140">
+      <c r="A1140" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="B1140" t="inlineStr">
+        <is>
+          <t>HELE</t>
+        </is>
+      </c>
+      <c r="C1140" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="1141">
+      <c r="A1141" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="B1141" t="inlineStr">
+        <is>
+          <t>HYPR</t>
+        </is>
+      </c>
+      <c r="C1141" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="1142">
+      <c r="A1142" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="B1142" t="inlineStr">
+        <is>
+          <t>IPW</t>
+        </is>
+      </c>
+      <c r="C1142" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="1143">
+      <c r="A1143" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="B1143" t="inlineStr">
+        <is>
+          <t>PCRX</t>
+        </is>
+      </c>
+      <c r="C1143" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="1144">
+      <c r="A1144" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="B1144" t="inlineStr">
+        <is>
+          <t>PROF</t>
+        </is>
+      </c>
+      <c r="C1144" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="1145">
+      <c r="A1145" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="B1145" t="inlineStr">
+        <is>
+          <t>VHUB</t>
+        </is>
+      </c>
+      <c r="C1145" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="1146">
+      <c r="A1146" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="B1146" t="inlineStr">
+        <is>
+          <t>WOLF</t>
+        </is>
+      </c>
+      <c r="C1146" t="inlineStr">
         <is>
           <t>Dropped</t>
         </is>

</xml_diff>

<commit_message>
Daily screener update: 2026-10-13
</commit_message>
<xml_diff>
--- a/screener_history.xlsx
+++ b/screener_history.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G1034"/>
+  <dimension ref="A1:G1047"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -24107,6 +24107,371 @@
         </is>
       </c>
       <c r="C1034" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="1035">
+      <c r="A1035" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="B1035" t="inlineStr">
+        <is>
+          <t>ACVA</t>
+        </is>
+      </c>
+      <c r="C1035" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D1035" t="n">
+        <v>10.5</v>
+      </c>
+      <c r="E1035" t="n">
+        <v>10.43</v>
+      </c>
+      <c r="F1035" t="n">
+        <v>10.65</v>
+      </c>
+      <c r="G1035" t="n">
+        <v>666</v>
+      </c>
+    </row>
+    <row r="1036">
+      <c r="A1036" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="B1036" t="inlineStr">
+        <is>
+          <t>AEMD</t>
+        </is>
+      </c>
+      <c r="C1036" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D1036" t="n">
+        <v>6.69</v>
+      </c>
+      <c r="E1036" t="n">
+        <v>5.82</v>
+      </c>
+      <c r="F1036" t="n">
+        <v>8.43</v>
+      </c>
+      <c r="G1036" t="n">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="1037">
+      <c r="A1037" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="B1037" t="inlineStr">
+        <is>
+          <t>BALY</t>
+        </is>
+      </c>
+      <c r="C1037" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D1037" t="n">
+        <v>14.51</v>
+      </c>
+      <c r="E1037" t="n">
+        <v>13.38</v>
+      </c>
+      <c r="F1037" t="n">
+        <v>16.77</v>
+      </c>
+      <c r="G1037" t="n">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="1038">
+      <c r="A1038" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="B1038" t="inlineStr">
+        <is>
+          <t>CDNA</t>
+        </is>
+      </c>
+      <c r="C1038" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D1038" t="n">
+        <v>72.51000000000001</v>
+      </c>
+      <c r="E1038" t="n">
+        <v>61.19</v>
+      </c>
+      <c r="F1038" t="n">
+        <v>95.15000000000001</v>
+      </c>
+      <c r="G1038" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="1039">
+      <c r="A1039" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="B1039" t="inlineStr">
+        <is>
+          <t>CRWD</t>
+        </is>
+      </c>
+      <c r="C1039" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D1039" t="n">
+        <v>286.99</v>
+      </c>
+      <c r="E1039" t="n">
+        <v>255.76</v>
+      </c>
+      <c r="F1039" t="n">
+        <v>349.46</v>
+      </c>
+      <c r="G1039" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1040">
+      <c r="A1040" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="B1040" t="inlineStr">
+        <is>
+          <t>FIRY</t>
+        </is>
+      </c>
+      <c r="C1040" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D1040" t="n">
+        <v>12.95</v>
+      </c>
+      <c r="E1040" t="n">
+        <v>11.73</v>
+      </c>
+      <c r="F1040" t="n">
+        <v>15.39</v>
+      </c>
+      <c r="G1040" t="n">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="1041">
+      <c r="A1041" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="B1041" t="inlineStr">
+        <is>
+          <t>GRAL</t>
+        </is>
+      </c>
+      <c r="C1041" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D1041" t="n">
+        <v>166.48</v>
+      </c>
+      <c r="E1041" t="n">
+        <v>127.46</v>
+      </c>
+      <c r="F1041" t="n">
+        <v>244.51</v>
+      </c>
+      <c r="G1041" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1042">
+      <c r="A1042" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="B1042" t="inlineStr">
+        <is>
+          <t>LFCR</t>
+        </is>
+      </c>
+      <c r="C1042" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D1042" t="n">
+        <v>6.61</v>
+      </c>
+      <c r="E1042" t="n">
+        <v>6.42</v>
+      </c>
+      <c r="F1042" t="n">
+        <v>6.99</v>
+      </c>
+      <c r="G1042" t="n">
+        <v>263</v>
+      </c>
+    </row>
+    <row r="1043">
+      <c r="A1043" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="B1043" t="inlineStr">
+        <is>
+          <t>PRTH</t>
+        </is>
+      </c>
+      <c r="C1043" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D1043" t="n">
+        <v>7.81</v>
+      </c>
+      <c r="E1043" t="n">
+        <v>7.76</v>
+      </c>
+      <c r="F1043" t="n">
+        <v>7.91</v>
+      </c>
+      <c r="G1043" t="n">
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="1044">
+      <c r="A1044" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="B1044" t="inlineStr">
+        <is>
+          <t>SSTI</t>
+        </is>
+      </c>
+      <c r="C1044" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D1044" t="n">
+        <v>8.779999999999999</v>
+      </c>
+      <c r="E1044" t="n">
+        <v>8.18</v>
+      </c>
+      <c r="F1044" t="n">
+        <v>9.98</v>
+      </c>
+      <c r="G1044" t="n">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="1045">
+      <c r="A1045" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="B1045" t="inlineStr">
+        <is>
+          <t>SUIG</t>
+        </is>
+      </c>
+      <c r="C1045" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D1045" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="E1045" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="F1045" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="G1045" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="1046">
+      <c r="A1046" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="B1046" t="inlineStr">
+        <is>
+          <t>TKNO</t>
+        </is>
+      </c>
+      <c r="C1046" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D1046" t="n">
+        <v>9.41</v>
+      </c>
+      <c r="E1046" t="n">
+        <v>8.34</v>
+      </c>
+      <c r="F1046" t="n">
+        <v>11.56</v>
+      </c>
+      <c r="G1046" t="n">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="1047">
+      <c r="A1047" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="B1047" t="inlineStr">
+        <is>
+          <t>BIO-B</t>
+        </is>
+      </c>
+      <c r="C1047" t="inlineStr">
         <is>
           <t>Dropped</t>
         </is>
@@ -24123,7 +24488,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G1146"/>
+  <dimension ref="A1:G1153"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -50460,6 +50825,149 @@
         </is>
       </c>
       <c r="C1146" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="1147">
+      <c r="A1147" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="B1147" t="inlineStr">
+        <is>
+          <t>IPW</t>
+        </is>
+      </c>
+      <c r="C1147" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D1147" t="n">
+        <v>0.83</v>
+      </c>
+      <c r="E1147" t="n">
+        <v>0.51</v>
+      </c>
+      <c r="F1147" t="n">
+        <v>1.48</v>
+      </c>
+      <c r="G1147" t="n">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="1148">
+      <c r="A1148" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="B1148" t="inlineStr">
+        <is>
+          <t>SKYA</t>
+        </is>
+      </c>
+      <c r="C1148" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D1148" t="n">
+        <v>2.44</v>
+      </c>
+      <c r="E1148" t="n">
+        <v>2.3</v>
+      </c>
+      <c r="F1148" t="n">
+        <v>2.72</v>
+      </c>
+      <c r="G1148" t="n">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="1149">
+      <c r="A1149" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="B1149" t="inlineStr">
+        <is>
+          <t>HUM</t>
+        </is>
+      </c>
+      <c r="C1149" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="1150">
+      <c r="A1150" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="B1150" t="inlineStr">
+        <is>
+          <t>OLB</t>
+        </is>
+      </c>
+      <c r="C1150" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="1151">
+      <c r="A1151" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="B1151" t="inlineStr">
+        <is>
+          <t>QETA</t>
+        </is>
+      </c>
+      <c r="C1151" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="1152">
+      <c r="A1152" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="B1152" t="inlineStr">
+        <is>
+          <t>VEEA</t>
+        </is>
+      </c>
+      <c r="C1152" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="1153">
+      <c r="A1153" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="B1153" t="inlineStr">
+        <is>
+          <t>VIVK</t>
+        </is>
+      </c>
+      <c r="C1153" t="inlineStr">
         <is>
           <t>Dropped</t>
         </is>

</xml_diff>

<commit_message>
Daily screener update: 2026-10-14
</commit_message>
<xml_diff>
--- a/screener_history.xlsx
+++ b/screener_history.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G1047"/>
+  <dimension ref="A1:G1061"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -24472,6 +24472,268 @@
         </is>
       </c>
       <c r="C1047" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="1048">
+      <c r="A1048" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B1048" t="inlineStr">
+        <is>
+          <t>BIO-B</t>
+        </is>
+      </c>
+      <c r="C1048" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D1048" t="n">
+        <v>365.08</v>
+      </c>
+      <c r="E1048" t="n">
+        <v>365.08</v>
+      </c>
+      <c r="F1048" t="n">
+        <v>365.08</v>
+      </c>
+      <c r="G1048" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="1049">
+      <c r="A1049" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B1049" t="inlineStr">
+        <is>
+          <t>TWN</t>
+        </is>
+      </c>
+      <c r="C1049" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D1049" t="n">
+        <v>108.27</v>
+      </c>
+      <c r="E1049" t="n">
+        <v>99.41</v>
+      </c>
+      <c r="F1049" t="n">
+        <v>125.99</v>
+      </c>
+      <c r="G1049" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="1050">
+      <c r="A1050" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B1050" t="inlineStr">
+        <is>
+          <t>ACVA</t>
+        </is>
+      </c>
+      <c r="C1050" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="1051">
+      <c r="A1051" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B1051" t="inlineStr">
+        <is>
+          <t>AEMD</t>
+        </is>
+      </c>
+      <c r="C1051" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="1052">
+      <c r="A1052" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B1052" t="inlineStr">
+        <is>
+          <t>BALY</t>
+        </is>
+      </c>
+      <c r="C1052" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="1053">
+      <c r="A1053" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B1053" t="inlineStr">
+        <is>
+          <t>CDNA</t>
+        </is>
+      </c>
+      <c r="C1053" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="1054">
+      <c r="A1054" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B1054" t="inlineStr">
+        <is>
+          <t>CRWD</t>
+        </is>
+      </c>
+      <c r="C1054" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="1055">
+      <c r="A1055" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B1055" t="inlineStr">
+        <is>
+          <t>FIRY</t>
+        </is>
+      </c>
+      <c r="C1055" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="1056">
+      <c r="A1056" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B1056" t="inlineStr">
+        <is>
+          <t>GRAL</t>
+        </is>
+      </c>
+      <c r="C1056" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="1057">
+      <c r="A1057" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B1057" t="inlineStr">
+        <is>
+          <t>LFCR</t>
+        </is>
+      </c>
+      <c r="C1057" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="1058">
+      <c r="A1058" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B1058" t="inlineStr">
+        <is>
+          <t>PRTH</t>
+        </is>
+      </c>
+      <c r="C1058" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="1059">
+      <c r="A1059" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B1059" t="inlineStr">
+        <is>
+          <t>SSTI</t>
+        </is>
+      </c>
+      <c r="C1059" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="1060">
+      <c r="A1060" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B1060" t="inlineStr">
+        <is>
+          <t>SUIG</t>
+        </is>
+      </c>
+      <c r="C1060" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="1061">
+      <c r="A1061" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B1061" t="inlineStr">
+        <is>
+          <t>TKNO</t>
+        </is>
+      </c>
+      <c r="C1061" t="inlineStr">
         <is>
           <t>Dropped</t>
         </is>
@@ -24488,7 +24750,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G1153"/>
+  <dimension ref="A1:G1158"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -50968,6 +51230,127 @@
         </is>
       </c>
       <c r="C1153" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="1154">
+      <c r="A1154" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B1154" t="inlineStr">
+        <is>
+          <t>BMBL</t>
+        </is>
+      </c>
+      <c r="C1154" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D1154" t="n">
+        <v>5.98</v>
+      </c>
+      <c r="E1154" t="n">
+        <v>5.92</v>
+      </c>
+      <c r="F1154" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="G1154" t="n">
+        <v>833</v>
+      </c>
+    </row>
+    <row r="1155">
+      <c r="A1155" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B1155" t="inlineStr">
+        <is>
+          <t>FRMI</t>
+        </is>
+      </c>
+      <c r="C1155" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D1155" t="n">
+        <v>3.67</v>
+      </c>
+      <c r="E1155" t="n">
+        <v>3.48</v>
+      </c>
+      <c r="F1155" t="n">
+        <v>4.05</v>
+      </c>
+      <c r="G1155" t="n">
+        <v>263</v>
+      </c>
+    </row>
+    <row r="1156">
+      <c r="A1156" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B1156" t="inlineStr">
+        <is>
+          <t>TCRT</t>
+        </is>
+      </c>
+      <c r="C1156" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D1156" t="n">
+        <v>2.09</v>
+      </c>
+      <c r="E1156" t="n">
+        <v>1.51</v>
+      </c>
+      <c r="F1156" t="n">
+        <v>3.25</v>
+      </c>
+      <c r="G1156" t="n">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="1157">
+      <c r="A1157" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B1157" t="inlineStr">
+        <is>
+          <t>IPW</t>
+        </is>
+      </c>
+      <c r="C1157" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="1158">
+      <c r="A1158" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B1158" t="inlineStr">
+        <is>
+          <t>SKYA</t>
+        </is>
+      </c>
+      <c r="C1158" t="inlineStr">
         <is>
           <t>Dropped</t>
         </is>

</xml_diff>

<commit_message>
Daily screener update: 2026-10-15
</commit_message>
<xml_diff>
--- a/screener_history.xlsx
+++ b/screener_history.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G1061"/>
+  <dimension ref="A1:G1064"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -24734,6 +24734,69 @@
         </is>
       </c>
       <c r="C1061" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="1062">
+      <c r="A1062" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="B1062" t="inlineStr">
+        <is>
+          <t>SBFG</t>
+        </is>
+      </c>
+      <c r="C1062" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D1062" t="n">
+        <v>30.39</v>
+      </c>
+      <c r="E1062" t="n">
+        <v>28.45</v>
+      </c>
+      <c r="F1062" t="n">
+        <v>34.27</v>
+      </c>
+      <c r="G1062" t="n">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="1063">
+      <c r="A1063" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="B1063" t="inlineStr">
+        <is>
+          <t>BIO-B</t>
+        </is>
+      </c>
+      <c r="C1063" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="1064">
+      <c r="A1064" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="B1064" t="inlineStr">
+        <is>
+          <t>TWN</t>
+        </is>
+      </c>
+      <c r="C1064" t="inlineStr">
         <is>
           <t>Dropped</t>
         </is>
@@ -24750,7 +24813,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G1158"/>
+  <dimension ref="A1:G1167"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -51351,6 +51414,243 @@
         </is>
       </c>
       <c r="C1158" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="1159">
+      <c r="A1159" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="B1159" t="inlineStr">
+        <is>
+          <t>FFAI</t>
+        </is>
+      </c>
+      <c r="C1159" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D1159" t="n">
+        <v>1.29</v>
+      </c>
+      <c r="E1159" t="n">
+        <v>1.04</v>
+      </c>
+      <c r="F1159" t="n">
+        <v>1.79</v>
+      </c>
+      <c r="G1159" t="n">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="1160">
+      <c r="A1160" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="B1160" t="inlineStr">
+        <is>
+          <t>GENK</t>
+        </is>
+      </c>
+      <c r="C1160" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D1160" t="n">
+        <v>2.53</v>
+      </c>
+      <c r="E1160" t="n">
+        <v>1.58</v>
+      </c>
+      <c r="F1160" t="n">
+        <v>4.43</v>
+      </c>
+      <c r="G1160" t="n">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="1161">
+      <c r="A1161" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="B1161" t="inlineStr">
+        <is>
+          <t>GLND</t>
+        </is>
+      </c>
+      <c r="C1161" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D1161" t="n">
+        <v>4.16</v>
+      </c>
+      <c r="E1161" t="n">
+        <v>3.41</v>
+      </c>
+      <c r="F1161" t="n">
+        <v>5.66</v>
+      </c>
+      <c r="G1161" t="n">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="1162">
+      <c r="A1162" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="B1162" t="inlineStr">
+        <is>
+          <t>LESL</t>
+        </is>
+      </c>
+      <c r="C1162" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D1162" t="n">
+        <v>0.13</v>
+      </c>
+      <c r="E1162" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="F1162" t="n">
+        <v>0.18</v>
+      </c>
+      <c r="G1162" t="n">
+        <v>2008</v>
+      </c>
+    </row>
+    <row r="1163">
+      <c r="A1163" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="B1163" t="inlineStr">
+        <is>
+          <t>LQDA</t>
+        </is>
+      </c>
+      <c r="C1163" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D1163" t="n">
+        <v>37.75</v>
+      </c>
+      <c r="E1163" t="n">
+        <v>33.12</v>
+      </c>
+      <c r="F1163" t="n">
+        <v>47.01</v>
+      </c>
+      <c r="G1163" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="1164">
+      <c r="A1164" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="B1164" t="inlineStr">
+        <is>
+          <t>MXCT</t>
+        </is>
+      </c>
+      <c r="C1164" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D1164" t="n">
+        <v>1.33</v>
+      </c>
+      <c r="E1164" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="F1164" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="G1164" t="n">
+        <v>370</v>
+      </c>
+    </row>
+    <row r="1165">
+      <c r="A1165" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="B1165" t="inlineStr">
+        <is>
+          <t>TGL</t>
+        </is>
+      </c>
+      <c r="C1165" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D1165" t="n">
+        <v>0.92</v>
+      </c>
+      <c r="E1165" t="n">
+        <v>0.32</v>
+      </c>
+      <c r="F1165" t="n">
+        <v>2.11</v>
+      </c>
+      <c r="G1165" t="n">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="1166">
+      <c r="A1166" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="B1166" t="inlineStr">
+        <is>
+          <t>BMBL</t>
+        </is>
+      </c>
+      <c r="C1166" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="1167">
+      <c r="A1167" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="B1167" t="inlineStr">
+        <is>
+          <t>FRMI</t>
+        </is>
+      </c>
+      <c r="C1167" t="inlineStr">
         <is>
           <t>Dropped</t>
         </is>

</xml_diff>

<commit_message>
Daily screener update: 2026-10-16
</commit_message>
<xml_diff>
--- a/screener_history.xlsx
+++ b/screener_history.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G1080"/>
+  <dimension ref="A1:G1106"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -25249,6 +25249,640 @@
         </is>
       </c>
       <c r="C1080" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="1081">
+      <c r="A1081" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="B1081" t="inlineStr">
+        <is>
+          <t>AMPL</t>
+        </is>
+      </c>
+      <c r="C1081" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D1081" t="n">
+        <v>16.17</v>
+      </c>
+      <c r="E1081" t="n">
+        <v>14.46</v>
+      </c>
+      <c r="F1081" t="n">
+        <v>19.6</v>
+      </c>
+      <c r="G1081" t="n">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="1082">
+      <c r="A1082" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="B1082" t="inlineStr">
+        <is>
+          <t>CDNA</t>
+        </is>
+      </c>
+      <c r="C1082" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D1082" t="n">
+        <v>72.51000000000001</v>
+      </c>
+      <c r="E1082" t="n">
+        <v>61.19</v>
+      </c>
+      <c r="F1082" t="n">
+        <v>95.15000000000001</v>
+      </c>
+      <c r="G1082" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="1083">
+      <c r="A1083" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="B1083" t="inlineStr">
+        <is>
+          <t>DK</t>
+        </is>
+      </c>
+      <c r="C1083" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D1083" t="n">
+        <v>81.72</v>
+      </c>
+      <c r="E1083" t="n">
+        <v>73.06999999999999</v>
+      </c>
+      <c r="F1083" t="n">
+        <v>99.02</v>
+      </c>
+      <c r="G1083" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="1084">
+      <c r="A1084" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="B1084" t="inlineStr">
+        <is>
+          <t>ECO</t>
+        </is>
+      </c>
+      <c r="C1084" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D1084" t="n">
+        <v>100.68</v>
+      </c>
+      <c r="E1084" t="n">
+        <v>85.81</v>
+      </c>
+      <c r="F1084" t="n">
+        <v>130.43</v>
+      </c>
+      <c r="G1084" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="1085">
+      <c r="A1085" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="B1085" t="inlineStr">
+        <is>
+          <t>FOSL</t>
+        </is>
+      </c>
+      <c r="C1085" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D1085" t="n">
+        <v>7.39</v>
+      </c>
+      <c r="E1085" t="n">
+        <v>6.78</v>
+      </c>
+      <c r="F1085" t="n">
+        <v>8.609999999999999</v>
+      </c>
+      <c r="G1085" t="n">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="1086">
+      <c r="A1086" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="B1086" t="inlineStr">
+        <is>
+          <t>HNGE</t>
+        </is>
+      </c>
+      <c r="C1086" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D1086" t="n">
+        <v>107</v>
+      </c>
+      <c r="E1086" t="n">
+        <v>96.02</v>
+      </c>
+      <c r="F1086" t="n">
+        <v>128.96</v>
+      </c>
+      <c r="G1086" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="1087">
+      <c r="A1087" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="B1087" t="inlineStr">
+        <is>
+          <t>LIND</t>
+        </is>
+      </c>
+      <c r="C1087" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D1087" t="n">
+        <v>36.97</v>
+      </c>
+      <c r="E1087" t="n">
+        <v>34.17</v>
+      </c>
+      <c r="F1087" t="n">
+        <v>42.57</v>
+      </c>
+      <c r="G1087" t="n">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="1088">
+      <c r="A1088" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="B1088" t="inlineStr">
+        <is>
+          <t>LVWR</t>
+        </is>
+      </c>
+      <c r="C1088" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D1088" t="n">
+        <v>1.75</v>
+      </c>
+      <c r="E1088" t="n">
+        <v>1.45</v>
+      </c>
+      <c r="F1088" t="n">
+        <v>2.34</v>
+      </c>
+      <c r="G1088" t="n">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="1089">
+      <c r="A1089" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="B1089" t="inlineStr">
+        <is>
+          <t>OM</t>
+        </is>
+      </c>
+      <c r="C1089" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D1089" t="n">
+        <v>4.34</v>
+      </c>
+      <c r="E1089" t="n">
+        <v>3.8</v>
+      </c>
+      <c r="F1089" t="n">
+        <v>5.42</v>
+      </c>
+      <c r="G1089" t="n">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="1090">
+      <c r="A1090" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="B1090" t="inlineStr">
+        <is>
+          <t>PBF</t>
+        </is>
+      </c>
+      <c r="C1090" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D1090" t="n">
+        <v>92.45999999999999</v>
+      </c>
+      <c r="E1090" t="n">
+        <v>80.05</v>
+      </c>
+      <c r="F1090" t="n">
+        <v>117.28</v>
+      </c>
+      <c r="G1090" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="1091">
+      <c r="A1091" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="B1091" t="inlineStr">
+        <is>
+          <t>PTC</t>
+        </is>
+      </c>
+      <c r="C1091" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D1091" t="n">
+        <v>196.05</v>
+      </c>
+      <c r="E1091" t="n">
+        <v>191.92</v>
+      </c>
+      <c r="F1091" t="n">
+        <v>204.31</v>
+      </c>
+      <c r="G1091" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="1092">
+      <c r="A1092" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="B1092" t="inlineStr">
+        <is>
+          <t>RCEL</t>
+        </is>
+      </c>
+      <c r="C1092" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D1092" t="n">
+        <v>13.73</v>
+      </c>
+      <c r="E1092" t="n">
+        <v>12.39</v>
+      </c>
+      <c r="F1092" t="n">
+        <v>16.41</v>
+      </c>
+      <c r="G1092" t="n">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="1093">
+      <c r="A1093" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="B1093" t="inlineStr">
+        <is>
+          <t>RPD</t>
+        </is>
+      </c>
+      <c r="C1093" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D1093" t="n">
+        <v>13.87</v>
+      </c>
+      <c r="E1093" t="n">
+        <v>11.88</v>
+      </c>
+      <c r="F1093" t="n">
+        <v>17.85</v>
+      </c>
+      <c r="G1093" t="n">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="1094">
+      <c r="A1094" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="B1094" t="inlineStr">
+        <is>
+          <t>RXO</t>
+        </is>
+      </c>
+      <c r="C1094" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D1094" t="n">
+        <v>29.37</v>
+      </c>
+      <c r="E1094" t="n">
+        <v>28.03</v>
+      </c>
+      <c r="F1094" t="n">
+        <v>32.05</v>
+      </c>
+      <c r="G1094" t="n">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="1095">
+      <c r="A1095" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="B1095" t="inlineStr">
+        <is>
+          <t>SBC</t>
+        </is>
+      </c>
+      <c r="C1095" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D1095" t="n">
+        <v>5.61</v>
+      </c>
+      <c r="E1095" t="n">
+        <v>5.1</v>
+      </c>
+      <c r="F1095" t="n">
+        <v>6.63</v>
+      </c>
+      <c r="G1095" t="n">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="1096">
+      <c r="A1096" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="B1096" t="inlineStr">
+        <is>
+          <t>SYNA</t>
+        </is>
+      </c>
+      <c r="C1096" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D1096" t="n">
+        <v>121</v>
+      </c>
+      <c r="E1096" t="n">
+        <v>116.85</v>
+      </c>
+      <c r="F1096" t="n">
+        <v>129.3</v>
+      </c>
+      <c r="G1096" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="1097">
+      <c r="A1097" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="B1097" t="inlineStr">
+        <is>
+          <t>BALY</t>
+        </is>
+      </c>
+      <c r="C1097" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="1098">
+      <c r="A1098" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="B1098" t="inlineStr">
+        <is>
+          <t>BENF</t>
+        </is>
+      </c>
+      <c r="C1098" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="1099">
+      <c r="A1099" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="B1099" t="inlineStr">
+        <is>
+          <t>EEIQ</t>
+        </is>
+      </c>
+      <c r="C1099" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="1100">
+      <c r="A1100" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="B1100" t="inlineStr">
+        <is>
+          <t>FEAM</t>
+        </is>
+      </c>
+      <c r="C1100" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="1101">
+      <c r="A1101" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="B1101" t="inlineStr">
+        <is>
+          <t>FTNT</t>
+        </is>
+      </c>
+      <c r="C1101" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="1102">
+      <c r="A1102" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="B1102" t="inlineStr">
+        <is>
+          <t>GRAL</t>
+        </is>
+      </c>
+      <c r="C1102" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="1103">
+      <c r="A1103" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="B1103" t="inlineStr">
+        <is>
+          <t>GRML</t>
+        </is>
+      </c>
+      <c r="C1103" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="1104">
+      <c r="A1104" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="B1104" t="inlineStr">
+        <is>
+          <t>QLYS</t>
+        </is>
+      </c>
+      <c r="C1104" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="1105">
+      <c r="A1105" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="B1105" t="inlineStr">
+        <is>
+          <t>REFR</t>
+        </is>
+      </c>
+      <c r="C1105" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="1106">
+      <c r="A1106" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="B1106" t="inlineStr">
+        <is>
+          <t>SVRN</t>
+        </is>
+      </c>
+      <c r="C1106" t="inlineStr">
         <is>
           <t>Dropped</t>
         </is>
@@ -25265,7 +25899,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G1179"/>
+  <dimension ref="A1:G1187"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -52355,6 +52989,202 @@
         </is>
       </c>
       <c r="C1179" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="1180">
+      <c r="A1180" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="B1180" t="inlineStr">
+        <is>
+          <t>HODO</t>
+        </is>
+      </c>
+      <c r="C1180" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D1180" t="n">
+        <v>0.09</v>
+      </c>
+      <c r="E1180" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="F1180" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="G1180" t="n">
+        <v>3496</v>
+      </c>
+    </row>
+    <row r="1181">
+      <c r="A1181" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="B1181" t="inlineStr">
+        <is>
+          <t>MRKR</t>
+        </is>
+      </c>
+      <c r="C1181" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D1181" t="n">
+        <v>1.03</v>
+      </c>
+      <c r="E1181" t="n">
+        <v>1</v>
+      </c>
+      <c r="F1181" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="G1181" t="n">
+        <v>1428</v>
+      </c>
+    </row>
+    <row r="1182">
+      <c r="A1182" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="B1182" t="inlineStr">
+        <is>
+          <t>RUBI</t>
+        </is>
+      </c>
+      <c r="C1182" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D1182" t="n">
+        <v>0.41</v>
+      </c>
+      <c r="E1182" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="F1182" t="n">
+        <v>0.63</v>
+      </c>
+      <c r="G1182" t="n">
+        <v>449</v>
+      </c>
+    </row>
+    <row r="1183">
+      <c r="A1183" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="B1183" t="inlineStr">
+        <is>
+          <t>SITC</t>
+        </is>
+      </c>
+      <c r="C1183" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D1183" t="n">
+        <v>3.63</v>
+      </c>
+      <c r="E1183" t="n">
+        <v>3.41</v>
+      </c>
+      <c r="F1183" t="n">
+        <v>4.06</v>
+      </c>
+      <c r="G1183" t="n">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="1184">
+      <c r="A1184" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="B1184" t="inlineStr">
+        <is>
+          <t>TCRT</t>
+        </is>
+      </c>
+      <c r="C1184" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D1184" t="n">
+        <v>2.94</v>
+      </c>
+      <c r="E1184" t="n">
+        <v>2.31</v>
+      </c>
+      <c r="F1184" t="n">
+        <v>4.2</v>
+      </c>
+      <c r="G1184" t="n">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="1185">
+      <c r="A1185" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="B1185" t="inlineStr">
+        <is>
+          <t>DRMA</t>
+        </is>
+      </c>
+      <c r="C1185" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="1186">
+      <c r="A1186" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="B1186" t="inlineStr">
+        <is>
+          <t>OPK</t>
+        </is>
+      </c>
+      <c r="C1186" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="1187">
+      <c r="A1187" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="B1187" t="inlineStr">
+        <is>
+          <t>SDST</t>
+        </is>
+      </c>
+      <c r="C1187" t="inlineStr">
         <is>
           <t>Dropped</t>
         </is>

</xml_diff>

<commit_message>
Daily screener update: 2026-10-20
</commit_message>
<xml_diff>
--- a/screener_history.xlsx
+++ b/screener_history.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G1106"/>
+  <dimension ref="A1:G1127"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -25883,6 +25883,363 @@
         </is>
       </c>
       <c r="C1106" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="1107">
+      <c r="A1107" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="B1107" t="inlineStr">
+        <is>
+          <t>AMPL</t>
+        </is>
+      </c>
+      <c r="C1107" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="1108">
+      <c r="A1108" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="B1108" t="inlineStr">
+        <is>
+          <t>CDNA</t>
+        </is>
+      </c>
+      <c r="C1108" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="1109">
+      <c r="A1109" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="B1109" t="inlineStr">
+        <is>
+          <t>DK</t>
+        </is>
+      </c>
+      <c r="C1109" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="1110">
+      <c r="A1110" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="B1110" t="inlineStr">
+        <is>
+          <t>ECO</t>
+        </is>
+      </c>
+      <c r="C1110" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="1111">
+      <c r="A1111" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="B1111" t="inlineStr">
+        <is>
+          <t>FOSL</t>
+        </is>
+      </c>
+      <c r="C1111" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="1112">
+      <c r="A1112" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="B1112" t="inlineStr">
+        <is>
+          <t>HNGE</t>
+        </is>
+      </c>
+      <c r="C1112" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="1113">
+      <c r="A1113" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="B1113" t="inlineStr">
+        <is>
+          <t>KOD</t>
+        </is>
+      </c>
+      <c r="C1113" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="1114">
+      <c r="A1114" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="B1114" t="inlineStr">
+        <is>
+          <t>LFCR</t>
+        </is>
+      </c>
+      <c r="C1114" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="1115">
+      <c r="A1115" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="B1115" t="inlineStr">
+        <is>
+          <t>LIND</t>
+        </is>
+      </c>
+      <c r="C1115" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="1116">
+      <c r="A1116" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="B1116" t="inlineStr">
+        <is>
+          <t>LVWR</t>
+        </is>
+      </c>
+      <c r="C1116" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="1117">
+      <c r="A1117" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="B1117" t="inlineStr">
+        <is>
+          <t>OM</t>
+        </is>
+      </c>
+      <c r="C1117" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="1118">
+      <c r="A1118" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="B1118" t="inlineStr">
+        <is>
+          <t>PBF</t>
+        </is>
+      </c>
+      <c r="C1118" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="1119">
+      <c r="A1119" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="B1119" t="inlineStr">
+        <is>
+          <t>PRTH</t>
+        </is>
+      </c>
+      <c r="C1119" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="1120">
+      <c r="A1120" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="B1120" t="inlineStr">
+        <is>
+          <t>PTC</t>
+        </is>
+      </c>
+      <c r="C1120" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="1121">
+      <c r="A1121" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="B1121" t="inlineStr">
+        <is>
+          <t>PXS</t>
+        </is>
+      </c>
+      <c r="C1121" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="1122">
+      <c r="A1122" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="B1122" t="inlineStr">
+        <is>
+          <t>RCEL</t>
+        </is>
+      </c>
+      <c r="C1122" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="1123">
+      <c r="A1123" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="B1123" t="inlineStr">
+        <is>
+          <t>RPD</t>
+        </is>
+      </c>
+      <c r="C1123" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="1124">
+      <c r="A1124" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="B1124" t="inlineStr">
+        <is>
+          <t>RXO</t>
+        </is>
+      </c>
+      <c r="C1124" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="1125">
+      <c r="A1125" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="B1125" t="inlineStr">
+        <is>
+          <t>SBC</t>
+        </is>
+      </c>
+      <c r="C1125" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="1126">
+      <c r="A1126" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="B1126" t="inlineStr">
+        <is>
+          <t>SSTI</t>
+        </is>
+      </c>
+      <c r="C1126" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="1127">
+      <c r="A1127" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="B1127" t="inlineStr">
+        <is>
+          <t>SYNA</t>
+        </is>
+      </c>
+      <c r="C1127" t="inlineStr">
         <is>
           <t>Dropped</t>
         </is>
@@ -25899,7 +26256,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G1187"/>
+  <dimension ref="A1:G1198"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -53185,6 +53542,265 @@
         </is>
       </c>
       <c r="C1187" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="1188">
+      <c r="A1188" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="B1188" t="inlineStr">
+        <is>
+          <t>AAME</t>
+        </is>
+      </c>
+      <c r="C1188" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D1188" t="n">
+        <v>1.56</v>
+      </c>
+      <c r="E1188" t="n">
+        <v>1.18</v>
+      </c>
+      <c r="F1188" t="n">
+        <v>2.31</v>
+      </c>
+      <c r="G1188" t="n">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="1189">
+      <c r="A1189" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="B1189" t="inlineStr">
+        <is>
+          <t>CLF</t>
+        </is>
+      </c>
+      <c r="C1189" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D1189" t="n">
+        <v>14.58</v>
+      </c>
+      <c r="E1189" t="n">
+        <v>12.94</v>
+      </c>
+      <c r="F1189" t="n">
+        <v>17.86</v>
+      </c>
+      <c r="G1189" t="n">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="1190">
+      <c r="A1190" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="B1190" t="inlineStr">
+        <is>
+          <t>DWTX</t>
+        </is>
+      </c>
+      <c r="C1190" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D1190" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="E1190" t="n">
+        <v>1.18</v>
+      </c>
+      <c r="F1190" t="n">
+        <v>1.84</v>
+      </c>
+      <c r="G1190" t="n">
+        <v>227</v>
+      </c>
+    </row>
+    <row r="1191">
+      <c r="A1191" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="B1191" t="inlineStr">
+        <is>
+          <t>IRON</t>
+        </is>
+      </c>
+      <c r="C1191" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D1191" t="n">
+        <v>75.5</v>
+      </c>
+      <c r="E1191" t="n">
+        <v>69.98</v>
+      </c>
+      <c r="F1191" t="n">
+        <v>86.54000000000001</v>
+      </c>
+      <c r="G1191" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="1192">
+      <c r="A1192" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="B1192" t="inlineStr">
+        <is>
+          <t>SAFX</t>
+        </is>
+      </c>
+      <c r="C1192" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D1192" t="n">
+        <v>0.19</v>
+      </c>
+      <c r="E1192" t="n">
+        <v>0.14</v>
+      </c>
+      <c r="F1192" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="G1192" t="n">
+        <v>1103</v>
+      </c>
+    </row>
+    <row r="1193">
+      <c r="A1193" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="B1193" t="inlineStr">
+        <is>
+          <t>UPLD</t>
+        </is>
+      </c>
+      <c r="C1193" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D1193" t="n">
+        <v>3.93</v>
+      </c>
+      <c r="E1193" t="n">
+        <v>2.77</v>
+      </c>
+      <c r="F1193" t="n">
+        <v>6.25</v>
+      </c>
+      <c r="G1193" t="n">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="1194">
+      <c r="A1194" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="B1194" t="inlineStr">
+        <is>
+          <t>HODO</t>
+        </is>
+      </c>
+      <c r="C1194" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="1195">
+      <c r="A1195" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="B1195" t="inlineStr">
+        <is>
+          <t>MRKR</t>
+        </is>
+      </c>
+      <c r="C1195" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="1196">
+      <c r="A1196" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="B1196" t="inlineStr">
+        <is>
+          <t>OPENW</t>
+        </is>
+      </c>
+      <c r="C1196" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="1197">
+      <c r="A1197" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="B1197" t="inlineStr">
+        <is>
+          <t>RUBI</t>
+        </is>
+      </c>
+      <c r="C1197" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="1198">
+      <c r="A1198" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="B1198" t="inlineStr">
+        <is>
+          <t>SITC</t>
+        </is>
+      </c>
+      <c r="C1198" t="inlineStr">
         <is>
           <t>Dropped</t>
         </is>

</xml_diff>

<commit_message>
Daily screener update: 2026-10-21
</commit_message>
<xml_diff>
--- a/screener_history.xlsx
+++ b/screener_history.xlsx
@@ -26256,7 +26256,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G1198"/>
+  <dimension ref="A1:G1208"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -53801,6 +53801,212 @@
         </is>
       </c>
       <c r="C1198" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="1199">
+      <c r="A1199" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="B1199" t="inlineStr">
+        <is>
+          <t>BRZE</t>
+        </is>
+      </c>
+      <c r="C1199" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D1199" t="n">
+        <v>45.58</v>
+      </c>
+      <c r="E1199" t="n">
+        <v>45.26</v>
+      </c>
+      <c r="F1199" t="n">
+        <v>46.22</v>
+      </c>
+      <c r="G1199" t="n">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="1200">
+      <c r="A1200" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="B1200" t="inlineStr">
+        <is>
+          <t>MYGN</t>
+        </is>
+      </c>
+      <c r="C1200" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D1200" t="n">
+        <v>5.63</v>
+      </c>
+      <c r="E1200" t="n">
+        <v>5.25</v>
+      </c>
+      <c r="F1200" t="n">
+        <v>6.39</v>
+      </c>
+      <c r="G1200" t="n">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="1201">
+      <c r="A1201" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="B1201" t="inlineStr">
+        <is>
+          <t>PRSO</t>
+        </is>
+      </c>
+      <c r="C1201" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D1201" t="n">
+        <v>0.58</v>
+      </c>
+      <c r="E1201" t="n">
+        <v>0.42</v>
+      </c>
+      <c r="F1201" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="G1201" t="n">
+        <v>311</v>
+      </c>
+    </row>
+    <row r="1202">
+      <c r="A1202" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="B1202" t="inlineStr">
+        <is>
+          <t>AAME</t>
+        </is>
+      </c>
+      <c r="C1202" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="1203">
+      <c r="A1203" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="B1203" t="inlineStr">
+        <is>
+          <t>CLF</t>
+        </is>
+      </c>
+      <c r="C1203" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="1204">
+      <c r="A1204" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="B1204" t="inlineStr">
+        <is>
+          <t>DWTX</t>
+        </is>
+      </c>
+      <c r="C1204" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="1205">
+      <c r="A1205" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="B1205" t="inlineStr">
+        <is>
+          <t>IRON</t>
+        </is>
+      </c>
+      <c r="C1205" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="1206">
+      <c r="A1206" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="B1206" t="inlineStr">
+        <is>
+          <t>SAFX</t>
+        </is>
+      </c>
+      <c r="C1206" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="1207">
+      <c r="A1207" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="B1207" t="inlineStr">
+        <is>
+          <t>TCRT</t>
+        </is>
+      </c>
+      <c r="C1207" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="1208">
+      <c r="A1208" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="B1208" t="inlineStr">
+        <is>
+          <t>UPLD</t>
+        </is>
+      </c>
+      <c r="C1208" t="inlineStr">
         <is>
           <t>Dropped</t>
         </is>

</xml_diff>

<commit_message>
Daily screener update: 2026-10-22
</commit_message>
<xml_diff>
--- a/screener_history.xlsx
+++ b/screener_history.xlsx
@@ -26256,7 +26256,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G1208"/>
+  <dimension ref="A1:G1218"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -54007,6 +54007,260 @@
         </is>
       </c>
       <c r="C1208" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="1209">
+      <c r="A1209" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="B1209" t="inlineStr">
+        <is>
+          <t>AHT</t>
+        </is>
+      </c>
+      <c r="C1209" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D1209" t="n">
+        <v>2.44</v>
+      </c>
+      <c r="E1209" t="n">
+        <v>2.26</v>
+      </c>
+      <c r="F1209" t="n">
+        <v>2.81</v>
+      </c>
+      <c r="G1209" t="n">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="1210">
+      <c r="A1210" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="B1210" t="inlineStr">
+        <is>
+          <t>AMOD</t>
+        </is>
+      </c>
+      <c r="C1210" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D1210" t="n">
+        <v>1.94</v>
+      </c>
+      <c r="E1210" t="n">
+        <v>0.87</v>
+      </c>
+      <c r="F1210" t="n">
+        <v>4.08</v>
+      </c>
+      <c r="G1210" t="n">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="1211">
+      <c r="A1211" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="B1211" t="inlineStr">
+        <is>
+          <t>INVE</t>
+        </is>
+      </c>
+      <c r="C1211" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D1211" t="n">
+        <v>2.76</v>
+      </c>
+      <c r="E1211" t="n">
+        <v>2.68</v>
+      </c>
+      <c r="F1211" t="n">
+        <v>2.92</v>
+      </c>
+      <c r="G1211" t="n">
+        <v>625</v>
+      </c>
+    </row>
+    <row r="1212">
+      <c r="A1212" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="B1212" t="inlineStr">
+        <is>
+          <t>OLOX</t>
+        </is>
+      </c>
+      <c r="C1212" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D1212" t="n">
+        <v>1.19</v>
+      </c>
+      <c r="E1212" t="n">
+        <v>0.87</v>
+      </c>
+      <c r="F1212" t="n">
+        <v>1.83</v>
+      </c>
+      <c r="G1212" t="n">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="1213">
+      <c r="A1213" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="B1213" t="inlineStr">
+        <is>
+          <t>RBNE</t>
+        </is>
+      </c>
+      <c r="C1213" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D1213" t="n">
+        <v>1</v>
+      </c>
+      <c r="E1213" t="n">
+        <v>0.22</v>
+      </c>
+      <c r="F1213" t="n">
+        <v>2.57</v>
+      </c>
+      <c r="G1213" t="n">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="1214">
+      <c r="A1214" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="B1214" t="inlineStr">
+        <is>
+          <t>SHFS</t>
+        </is>
+      </c>
+      <c r="C1214" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D1214" t="n">
+        <v>0.18</v>
+      </c>
+      <c r="E1214" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="F1214" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="G1214" t="n">
+        <v>810</v>
+      </c>
+    </row>
+    <row r="1215">
+      <c r="A1215" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="B1215" t="inlineStr">
+        <is>
+          <t>WHLR</t>
+        </is>
+      </c>
+      <c r="C1215" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D1215" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="E1215" t="n">
+        <v>0.39</v>
+      </c>
+      <c r="F1215" t="n">
+        <v>0.58</v>
+      </c>
+      <c r="G1215" t="n">
+        <v>775</v>
+      </c>
+    </row>
+    <row r="1216">
+      <c r="A1216" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="B1216" t="inlineStr">
+        <is>
+          <t>BRZE</t>
+        </is>
+      </c>
+      <c r="C1216" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="1217">
+      <c r="A1217" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="B1217" t="inlineStr">
+        <is>
+          <t>MYGN</t>
+        </is>
+      </c>
+      <c r="C1217" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="1218">
+      <c r="A1218" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="B1218" t="inlineStr">
+        <is>
+          <t>PRSO</t>
+        </is>
+      </c>
+      <c r="C1218" t="inlineStr">
         <is>
           <t>Dropped</t>
         </is>

</xml_diff>

<commit_message>
Daily screener update: 2026-10-23
</commit_message>
<xml_diff>
--- a/screener_history.xlsx
+++ b/screener_history.xlsx
@@ -26256,7 +26256,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G1218"/>
+  <dimension ref="A1:G1233"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -54261,6 +54261,369 @@
         </is>
       </c>
       <c r="C1218" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="1219">
+      <c r="A1219" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="B1219" t="inlineStr">
+        <is>
+          <t>ATOM</t>
+        </is>
+      </c>
+      <c r="C1219" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D1219" t="n">
+        <v>3.56</v>
+      </c>
+      <c r="E1219" t="n">
+        <v>3.03</v>
+      </c>
+      <c r="F1219" t="n">
+        <v>4.62</v>
+      </c>
+      <c r="G1219" t="n">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="1220">
+      <c r="A1220" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="B1220" t="inlineStr">
+        <is>
+          <t>AVEX</t>
+        </is>
+      </c>
+      <c r="C1220" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D1220" t="n">
+        <v>11.1</v>
+      </c>
+      <c r="E1220" t="n">
+        <v>9.84</v>
+      </c>
+      <c r="F1220" t="n">
+        <v>13.62</v>
+      </c>
+      <c r="G1220" t="n">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="1221">
+      <c r="A1221" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="B1221" t="inlineStr">
+        <is>
+          <t>CJMB</t>
+        </is>
+      </c>
+      <c r="C1221" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D1221" t="n">
+        <v>0.59</v>
+      </c>
+      <c r="E1221" t="n">
+        <v>0.43</v>
+      </c>
+      <c r="F1221" t="n">
+        <v>0.89</v>
+      </c>
+      <c r="G1221" t="n">
+        <v>326</v>
+      </c>
+    </row>
+    <row r="1222">
+      <c r="A1222" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="B1222" t="inlineStr">
+        <is>
+          <t>LESL</t>
+        </is>
+      </c>
+      <c r="C1222" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D1222" t="n">
+        <v>0.13</v>
+      </c>
+      <c r="E1222" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="F1222" t="n">
+        <v>0.18</v>
+      </c>
+      <c r="G1222" t="n">
+        <v>2008</v>
+      </c>
+    </row>
+    <row r="1223">
+      <c r="A1223" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="B1223" t="inlineStr">
+        <is>
+          <t>PFSA</t>
+        </is>
+      </c>
+      <c r="C1223" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D1223" t="n">
+        <v>1.35</v>
+      </c>
+      <c r="E1223" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="F1223" t="n">
+        <v>2.25</v>
+      </c>
+      <c r="G1223" t="n">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="1224">
+      <c r="A1224" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="B1224" t="inlineStr">
+        <is>
+          <t>SKYQ</t>
+        </is>
+      </c>
+      <c r="C1224" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D1224" t="n">
+        <v>2.6</v>
+      </c>
+      <c r="E1224" t="n">
+        <v>2.06</v>
+      </c>
+      <c r="F1224" t="n">
+        <v>3.68</v>
+      </c>
+      <c r="G1224" t="n">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="1225">
+      <c r="A1225" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="B1225" t="inlineStr">
+        <is>
+          <t>SNAL</t>
+        </is>
+      </c>
+      <c r="C1225" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D1225" t="n">
+        <v>2.56</v>
+      </c>
+      <c r="E1225" t="n">
+        <v>1.88</v>
+      </c>
+      <c r="F1225" t="n">
+        <v>3.92</v>
+      </c>
+      <c r="G1225" t="n">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="1226">
+      <c r="A1226" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="B1226" t="inlineStr">
+        <is>
+          <t>XCUR</t>
+        </is>
+      </c>
+      <c r="C1226" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D1226" t="n">
+        <v>1.15</v>
+      </c>
+      <c r="E1226" t="n">
+        <v>1.08</v>
+      </c>
+      <c r="F1226" t="n">
+        <v>1.29</v>
+      </c>
+      <c r="G1226" t="n">
+        <v>715</v>
+      </c>
+    </row>
+    <row r="1227">
+      <c r="A1227" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="B1227" t="inlineStr">
+        <is>
+          <t>XXII</t>
+        </is>
+      </c>
+      <c r="C1227" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D1227" t="n">
+        <v>0.31</v>
+      </c>
+      <c r="E1227" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="F1227" t="n">
+        <v>0.52</v>
+      </c>
+      <c r="G1227" t="n">
+        <v>465</v>
+      </c>
+    </row>
+    <row r="1228">
+      <c r="A1228" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="B1228" t="inlineStr">
+        <is>
+          <t>AHT</t>
+        </is>
+      </c>
+      <c r="C1228" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="1229">
+      <c r="A1229" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="B1229" t="inlineStr">
+        <is>
+          <t>AMOD</t>
+        </is>
+      </c>
+      <c r="C1229" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="1230">
+      <c r="A1230" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="B1230" t="inlineStr">
+        <is>
+          <t>INVE</t>
+        </is>
+      </c>
+      <c r="C1230" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="1231">
+      <c r="A1231" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="B1231" t="inlineStr">
+        <is>
+          <t>OLOX</t>
+        </is>
+      </c>
+      <c r="C1231" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="1232">
+      <c r="A1232" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="B1232" t="inlineStr">
+        <is>
+          <t>RBNE</t>
+        </is>
+      </c>
+      <c r="C1232" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="1233">
+      <c r="A1233" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="B1233" t="inlineStr">
+        <is>
+          <t>WHLR</t>
+        </is>
+      </c>
+      <c r="C1233" t="inlineStr">
         <is>
           <t>Dropped</t>
         </is>

</xml_diff>

<commit_message>
Daily screener update: 2026-10-24
</commit_message>
<xml_diff>
--- a/screener_history.xlsx
+++ b/screener_history.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G1127"/>
+  <dimension ref="A1:G1131"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -26243,6 +26243,122 @@
         <is>
           <t>Dropped</t>
         </is>
+      </c>
+    </row>
+    <row r="1128">
+      <c r="A1128" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="B1128" t="inlineStr">
+        <is>
+          <t>ILMN</t>
+        </is>
+      </c>
+      <c r="C1128" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D1128" t="n">
+        <v>286.4</v>
+      </c>
+      <c r="E1128" t="n">
+        <v>257.14</v>
+      </c>
+      <c r="F1128" t="n">
+        <v>344.92</v>
+      </c>
+      <c r="G1128" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1129">
+      <c r="A1129" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="B1129" t="inlineStr">
+        <is>
+          <t>IOVA</t>
+        </is>
+      </c>
+      <c r="C1129" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D1129" t="n">
+        <v>15.37</v>
+      </c>
+      <c r="E1129" t="n">
+        <v>13.52</v>
+      </c>
+      <c r="F1129" t="n">
+        <v>19.07</v>
+      </c>
+      <c r="G1129" t="n">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="1130">
+      <c r="A1130" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="B1130" t="inlineStr">
+        <is>
+          <t>KOD</t>
+        </is>
+      </c>
+      <c r="C1130" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D1130" t="n">
+        <v>103.27</v>
+      </c>
+      <c r="E1130" t="n">
+        <v>79.06</v>
+      </c>
+      <c r="F1130" t="n">
+        <v>151.69</v>
+      </c>
+      <c r="G1130" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="1131">
+      <c r="A1131" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="B1131" t="inlineStr">
+        <is>
+          <t>LFCR</t>
+        </is>
+      </c>
+      <c r="C1131" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D1131" t="n">
+        <v>6.48</v>
+      </c>
+      <c r="E1131" t="n">
+        <v>6.36</v>
+      </c>
+      <c r="F1131" t="n">
+        <v>6.72</v>
+      </c>
+      <c r="G1131" t="n">
+        <v>416</v>
       </c>
     </row>
   </sheetData>
@@ -26256,7 +26372,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G1233"/>
+  <dimension ref="A1:G1248"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -54624,6 +54740,333 @@
         </is>
       </c>
       <c r="C1233" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="1234">
+      <c r="A1234" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="B1234" t="inlineStr">
+        <is>
+          <t>AMT</t>
+        </is>
+      </c>
+      <c r="C1234" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D1234" t="n">
+        <v>202.5</v>
+      </c>
+      <c r="E1234" t="n">
+        <v>185.44</v>
+      </c>
+      <c r="F1234" t="n">
+        <v>236.62</v>
+      </c>
+      <c r="G1234" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="1235">
+      <c r="A1235" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="B1235" t="inlineStr">
+        <is>
+          <t>BOLT</t>
+        </is>
+      </c>
+      <c r="C1235" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D1235" t="n">
+        <v>7.22</v>
+      </c>
+      <c r="E1235" t="n">
+        <v>5.99</v>
+      </c>
+      <c r="F1235" t="n">
+        <v>9.68</v>
+      </c>
+      <c r="G1235" t="n">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="1236">
+      <c r="A1236" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="B1236" t="inlineStr">
+        <is>
+          <t>CCI</t>
+        </is>
+      </c>
+      <c r="C1236" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D1236" t="n">
+        <v>91.45</v>
+      </c>
+      <c r="E1236" t="n">
+        <v>85</v>
+      </c>
+      <c r="F1236" t="n">
+        <v>104.35</v>
+      </c>
+      <c r="G1236" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="1237">
+      <c r="A1237" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="B1237" t="inlineStr">
+        <is>
+          <t>LUCD</t>
+        </is>
+      </c>
+      <c r="C1237" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D1237" t="n">
+        <v>0.43</v>
+      </c>
+      <c r="E1237" t="n">
+        <v>0.39</v>
+      </c>
+      <c r="F1237" t="n">
+        <v>0.53</v>
+      </c>
+      <c r="G1237" t="n">
+        <v>1070</v>
+      </c>
+    </row>
+    <row r="1238">
+      <c r="A1238" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="B1238" t="inlineStr">
+        <is>
+          <t>RHI</t>
+        </is>
+      </c>
+      <c r="C1238" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D1238" t="n">
+        <v>44.77</v>
+      </c>
+      <c r="E1238" t="n">
+        <v>41</v>
+      </c>
+      <c r="F1238" t="n">
+        <v>52.32</v>
+      </c>
+      <c r="G1238" t="n">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="1239">
+      <c r="A1239" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="B1239" t="inlineStr">
+        <is>
+          <t>RNG</t>
+        </is>
+      </c>
+      <c r="C1239" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D1239" t="n">
+        <v>98.14</v>
+      </c>
+      <c r="E1239" t="n">
+        <v>82.66</v>
+      </c>
+      <c r="F1239" t="n">
+        <v>129.1</v>
+      </c>
+      <c r="G1239" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="1240">
+      <c r="A1240" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="B1240" t="inlineStr">
+        <is>
+          <t>ATOM</t>
+        </is>
+      </c>
+      <c r="C1240" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="1241">
+      <c r="A1241" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="B1241" t="inlineStr">
+        <is>
+          <t>AVEX</t>
+        </is>
+      </c>
+      <c r="C1241" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="1242">
+      <c r="A1242" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="B1242" t="inlineStr">
+        <is>
+          <t>CJMB</t>
+        </is>
+      </c>
+      <c r="C1242" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="1243">
+      <c r="A1243" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="B1243" t="inlineStr">
+        <is>
+          <t>LESL</t>
+        </is>
+      </c>
+      <c r="C1243" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="1244">
+      <c r="A1244" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="B1244" t="inlineStr">
+        <is>
+          <t>PFSA</t>
+        </is>
+      </c>
+      <c r="C1244" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="1245">
+      <c r="A1245" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="B1245" t="inlineStr">
+        <is>
+          <t>SHFS</t>
+        </is>
+      </c>
+      <c r="C1245" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="1246">
+      <c r="A1246" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="B1246" t="inlineStr">
+        <is>
+          <t>SKYQ</t>
+        </is>
+      </c>
+      <c r="C1246" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="1247">
+      <c r="A1247" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="B1247" t="inlineStr">
+        <is>
+          <t>SNAL</t>
+        </is>
+      </c>
+      <c r="C1247" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="1248">
+      <c r="A1248" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="B1248" t="inlineStr">
+        <is>
+          <t>XCUR</t>
+        </is>
+      </c>
+      <c r="C1248" t="inlineStr">
         <is>
           <t>Dropped</t>
         </is>

</xml_diff>

<commit_message>
Daily screener update: 2026-10-27
</commit_message>
<xml_diff>
--- a/screener_history.xlsx
+++ b/screener_history.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G1131"/>
+  <dimension ref="A1:G1135"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -26359,6 +26359,74 @@
       </c>
       <c r="G1131" t="n">
         <v>416</v>
+      </c>
+    </row>
+    <row r="1132">
+      <c r="A1132" t="inlineStr">
+        <is>
+          <t>2026-10-27</t>
+        </is>
+      </c>
+      <c r="B1132" t="inlineStr">
+        <is>
+          <t>ILMN</t>
+        </is>
+      </c>
+      <c r="C1132" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="1133">
+      <c r="A1133" t="inlineStr">
+        <is>
+          <t>2026-10-27</t>
+        </is>
+      </c>
+      <c r="B1133" t="inlineStr">
+        <is>
+          <t>IOVA</t>
+        </is>
+      </c>
+      <c r="C1133" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="1134">
+      <c r="A1134" t="inlineStr">
+        <is>
+          <t>2026-10-27</t>
+        </is>
+      </c>
+      <c r="B1134" t="inlineStr">
+        <is>
+          <t>KOD</t>
+        </is>
+      </c>
+      <c r="C1134" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="1135">
+      <c r="A1135" t="inlineStr">
+        <is>
+          <t>2026-10-27</t>
+        </is>
+      </c>
+      <c r="B1135" t="inlineStr">
+        <is>
+          <t>LFCR</t>
+        </is>
+      </c>
+      <c r="C1135" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -26372,7 +26440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G1248"/>
+  <dimension ref="A1:G1263"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -55067,6 +55135,357 @@
         </is>
       </c>
       <c r="C1248" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="1249">
+      <c r="A1249" t="inlineStr">
+        <is>
+          <t>2026-10-27</t>
+        </is>
+      </c>
+      <c r="B1249" t="inlineStr">
+        <is>
+          <t>BRAI</t>
+        </is>
+      </c>
+      <c r="C1249" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D1249" t="n">
+        <v>4.72</v>
+      </c>
+      <c r="E1249" t="n">
+        <v>2.1</v>
+      </c>
+      <c r="F1249" t="n">
+        <v>9.949999999999999</v>
+      </c>
+      <c r="G1249" t="n">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="1250">
+      <c r="A1250" t="inlineStr">
+        <is>
+          <t>2026-10-27</t>
+        </is>
+      </c>
+      <c r="B1250" t="inlineStr">
+        <is>
+          <t>CLRO</t>
+        </is>
+      </c>
+      <c r="C1250" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D1250" t="n">
+        <v>4.69</v>
+      </c>
+      <c r="E1250" t="n">
+        <v>4.02</v>
+      </c>
+      <c r="F1250" t="n">
+        <v>6.03</v>
+      </c>
+      <c r="G1250" t="n">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="1251">
+      <c r="A1251" t="inlineStr">
+        <is>
+          <t>2026-10-27</t>
+        </is>
+      </c>
+      <c r="B1251" t="inlineStr">
+        <is>
+          <t>PLUR</t>
+        </is>
+      </c>
+      <c r="C1251" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D1251" t="n">
+        <v>1.18</v>
+      </c>
+      <c r="E1251" t="n">
+        <v>0.96</v>
+      </c>
+      <c r="F1251" t="n">
+        <v>1.62</v>
+      </c>
+      <c r="G1251" t="n">
+        <v>227</v>
+      </c>
+    </row>
+    <row r="1252">
+      <c r="A1252" t="inlineStr">
+        <is>
+          <t>2026-10-27</t>
+        </is>
+      </c>
+      <c r="B1252" t="inlineStr">
+        <is>
+          <t>RENT</t>
+        </is>
+      </c>
+      <c r="C1252" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D1252" t="n">
+        <v>2.98</v>
+      </c>
+      <c r="E1252" t="n">
+        <v>2.63</v>
+      </c>
+      <c r="F1252" t="n">
+        <v>3.68</v>
+      </c>
+      <c r="G1252" t="n">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="1253">
+      <c r="A1253" t="inlineStr">
+        <is>
+          <t>2026-10-27</t>
+        </is>
+      </c>
+      <c r="B1253" t="inlineStr">
+        <is>
+          <t>RRC</t>
+        </is>
+      </c>
+      <c r="C1253" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D1253" t="n">
+        <v>52.8</v>
+      </c>
+      <c r="E1253" t="n">
+        <v>50</v>
+      </c>
+      <c r="F1253" t="n">
+        <v>58.4</v>
+      </c>
+      <c r="G1253" t="n">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="1254">
+      <c r="A1254" t="inlineStr">
+        <is>
+          <t>2026-10-27</t>
+        </is>
+      </c>
+      <c r="B1254" t="inlineStr">
+        <is>
+          <t>SGRY</t>
+        </is>
+      </c>
+      <c r="C1254" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D1254" t="n">
+        <v>23.14</v>
+      </c>
+      <c r="E1254" t="n">
+        <v>22.94</v>
+      </c>
+      <c r="F1254" t="n">
+        <v>23.53</v>
+      </c>
+      <c r="G1254" t="n">
+        <v>256</v>
+      </c>
+    </row>
+    <row r="1255">
+      <c r="A1255" t="inlineStr">
+        <is>
+          <t>2026-10-27</t>
+        </is>
+      </c>
+      <c r="B1255" t="inlineStr">
+        <is>
+          <t>TGL</t>
+        </is>
+      </c>
+      <c r="C1255" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D1255" t="n">
+        <v>0.31</v>
+      </c>
+      <c r="E1255" t="n">
+        <v>0.22</v>
+      </c>
+      <c r="F1255" t="n">
+        <v>0.48</v>
+      </c>
+      <c r="G1255" t="n">
+        <v>562</v>
+      </c>
+    </row>
+    <row r="1256">
+      <c r="A1256" t="inlineStr">
+        <is>
+          <t>2026-10-27</t>
+        </is>
+      </c>
+      <c r="B1256" t="inlineStr">
+        <is>
+          <t>XNCR</t>
+        </is>
+      </c>
+      <c r="C1256" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D1256" t="n">
+        <v>33.58</v>
+      </c>
+      <c r="E1256" t="n">
+        <v>28.84</v>
+      </c>
+      <c r="F1256" t="n">
+        <v>43.06</v>
+      </c>
+      <c r="G1256" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="1257">
+      <c r="A1257" t="inlineStr">
+        <is>
+          <t>2026-10-27</t>
+        </is>
+      </c>
+      <c r="B1257" t="inlineStr">
+        <is>
+          <t>AMT</t>
+        </is>
+      </c>
+      <c r="C1257" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="1258">
+      <c r="A1258" t="inlineStr">
+        <is>
+          <t>2026-10-27</t>
+        </is>
+      </c>
+      <c r="B1258" t="inlineStr">
+        <is>
+          <t>BOLT</t>
+        </is>
+      </c>
+      <c r="C1258" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="1259">
+      <c r="A1259" t="inlineStr">
+        <is>
+          <t>2026-10-27</t>
+        </is>
+      </c>
+      <c r="B1259" t="inlineStr">
+        <is>
+          <t>CCI</t>
+        </is>
+      </c>
+      <c r="C1259" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="1260">
+      <c r="A1260" t="inlineStr">
+        <is>
+          <t>2026-10-27</t>
+        </is>
+      </c>
+      <c r="B1260" t="inlineStr">
+        <is>
+          <t>LUCD</t>
+        </is>
+      </c>
+      <c r="C1260" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="1261">
+      <c r="A1261" t="inlineStr">
+        <is>
+          <t>2026-10-27</t>
+        </is>
+      </c>
+      <c r="B1261" t="inlineStr">
+        <is>
+          <t>RHI</t>
+        </is>
+      </c>
+      <c r="C1261" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="1262">
+      <c r="A1262" t="inlineStr">
+        <is>
+          <t>2026-10-27</t>
+        </is>
+      </c>
+      <c r="B1262" t="inlineStr">
+        <is>
+          <t>RNG</t>
+        </is>
+      </c>
+      <c r="C1262" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="1263">
+      <c r="A1263" t="inlineStr">
+        <is>
+          <t>2026-10-27</t>
+        </is>
+      </c>
+      <c r="B1263" t="inlineStr">
+        <is>
+          <t>XXII</t>
+        </is>
+      </c>
+      <c r="C1263" t="inlineStr">
         <is>
           <t>Dropped</t>
         </is>

</xml_diff>

<commit_message>
Daily screener update: 2026-10-28
</commit_message>
<xml_diff>
--- a/screener_history.xlsx
+++ b/screener_history.xlsx
@@ -26440,7 +26440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G1263"/>
+  <dimension ref="A1:G1272"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -55486,6 +55486,195 @@
         </is>
       </c>
       <c r="C1263" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="1264">
+      <c r="A1264" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="B1264" t="inlineStr">
+        <is>
+          <t>OPENZ</t>
+        </is>
+      </c>
+      <c r="C1264" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D1264" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="E1264" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="F1264" t="n">
+        <v>0.13</v>
+      </c>
+      <c r="G1264" t="n">
+        <v>2164</v>
+      </c>
+    </row>
+    <row r="1265">
+      <c r="A1265" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="B1265" t="inlineStr">
+        <is>
+          <t>SOFI</t>
+        </is>
+      </c>
+      <c r="C1265" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D1265" t="n">
+        <v>16.17</v>
+      </c>
+      <c r="E1265" t="n">
+        <v>15.67</v>
+      </c>
+      <c r="F1265" t="n">
+        <v>17.17</v>
+      </c>
+      <c r="G1265" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="1266">
+      <c r="A1266" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="B1266" t="inlineStr">
+        <is>
+          <t>XXII</t>
+        </is>
+      </c>
+      <c r="C1266" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D1266" t="n">
+        <v>0.13</v>
+      </c>
+      <c r="E1266" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="F1266" t="n">
+        <v>0.18</v>
+      </c>
+      <c r="G1266" t="n">
+        <v>1736</v>
+      </c>
+    </row>
+    <row r="1267">
+      <c r="A1267" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="B1267" t="inlineStr">
+        <is>
+          <t>PLUR</t>
+        </is>
+      </c>
+      <c r="C1267" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="1268">
+      <c r="A1268" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="B1268" t="inlineStr">
+        <is>
+          <t>RENT</t>
+        </is>
+      </c>
+      <c r="C1268" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="1269">
+      <c r="A1269" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="B1269" t="inlineStr">
+        <is>
+          <t>RRC</t>
+        </is>
+      </c>
+      <c r="C1269" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="1270">
+      <c r="A1270" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="B1270" t="inlineStr">
+        <is>
+          <t>SGRY</t>
+        </is>
+      </c>
+      <c r="C1270" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="1271">
+      <c r="A1271" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="B1271" t="inlineStr">
+        <is>
+          <t>TGL</t>
+        </is>
+      </c>
+      <c r="C1271" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="1272">
+      <c r="A1272" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="B1272" t="inlineStr">
+        <is>
+          <t>XNCR</t>
+        </is>
+      </c>
+      <c r="C1272" t="inlineStr">
         <is>
           <t>Dropped</t>
         </is>

</xml_diff>

<commit_message>
Daily screener update: 2026-10-29
</commit_message>
<xml_diff>
--- a/screener_history.xlsx
+++ b/screener_history.xlsx
@@ -26440,7 +26440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G1272"/>
+  <dimension ref="A1:G1285"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -55675,6 +55675,335 @@
         </is>
       </c>
       <c r="C1272" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="1273">
+      <c r="A1273" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="B1273" t="inlineStr">
+        <is>
+          <t>AXGN</t>
+        </is>
+      </c>
+      <c r="C1273" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D1273" t="n">
+        <v>46.15</v>
+      </c>
+      <c r="E1273" t="n">
+        <v>43.5</v>
+      </c>
+      <c r="F1273" t="n">
+        <v>51.45</v>
+      </c>
+      <c r="G1273" t="n">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="1274">
+      <c r="A1274" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="B1274" t="inlineStr">
+        <is>
+          <t>BOOM</t>
+        </is>
+      </c>
+      <c r="C1274" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D1274" t="n">
+        <v>7.05</v>
+      </c>
+      <c r="E1274" t="n">
+        <v>6.62</v>
+      </c>
+      <c r="F1274" t="n">
+        <v>7.92</v>
+      </c>
+      <c r="G1274" t="n">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="1275">
+      <c r="A1275" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="B1275" t="inlineStr">
+        <is>
+          <t>CDT</t>
+        </is>
+      </c>
+      <c r="C1275" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D1275" t="n">
+        <v>0.09</v>
+      </c>
+      <c r="E1275" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="F1275" t="n">
+        <v>0.14</v>
+      </c>
+      <c r="G1275" t="n">
+        <v>1937</v>
+      </c>
+    </row>
+    <row r="1276">
+      <c r="A1276" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="B1276" t="inlineStr">
+        <is>
+          <t>GCTK</t>
+        </is>
+      </c>
+      <c r="C1276" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D1276" t="n">
+        <v>2.12</v>
+      </c>
+      <c r="E1276" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="F1276" t="n">
+        <v>2.76</v>
+      </c>
+      <c r="G1276" t="n">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="1277">
+      <c r="A1277" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="B1277" t="inlineStr">
+        <is>
+          <t>LUNG</t>
+        </is>
+      </c>
+      <c r="C1277" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D1277" t="n">
+        <v>2.59</v>
+      </c>
+      <c r="E1277" t="n">
+        <v>2.31</v>
+      </c>
+      <c r="F1277" t="n">
+        <v>3.14</v>
+      </c>
+      <c r="G1277" t="n">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="1278">
+      <c r="A1278" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="B1278" t="inlineStr">
+        <is>
+          <t>SSP</t>
+        </is>
+      </c>
+      <c r="C1278" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D1278" t="n">
+        <v>2.49</v>
+      </c>
+      <c r="E1278" t="n">
+        <v>2.26</v>
+      </c>
+      <c r="F1278" t="n">
+        <v>2.95</v>
+      </c>
+      <c r="G1278" t="n">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="1279">
+      <c r="A1279" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="B1279" t="inlineStr">
+        <is>
+          <t>ULBI</t>
+        </is>
+      </c>
+      <c r="C1279" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D1279" t="n">
+        <v>15.66</v>
+      </c>
+      <c r="E1279" t="n">
+        <v>15.6</v>
+      </c>
+      <c r="F1279" t="n">
+        <v>15.78</v>
+      </c>
+      <c r="G1279" t="n">
+        <v>833</v>
+      </c>
+    </row>
+    <row r="1280">
+      <c r="A1280" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="B1280" t="inlineStr">
+        <is>
+          <t>VRT</t>
+        </is>
+      </c>
+      <c r="C1280" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D1280" t="n">
+        <v>243</v>
+      </c>
+      <c r="E1280" t="n">
+        <v>228.81</v>
+      </c>
+      <c r="F1280" t="n">
+        <v>271.38</v>
+      </c>
+      <c r="G1280" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="1281">
+      <c r="A1281" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="B1281" t="inlineStr">
+        <is>
+          <t>WEN</t>
+        </is>
+      </c>
+      <c r="C1281" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D1281" t="n">
+        <v>7.15</v>
+      </c>
+      <c r="E1281" t="n">
+        <v>6.97</v>
+      </c>
+      <c r="F1281" t="n">
+        <v>7.51</v>
+      </c>
+      <c r="G1281" t="n">
+        <v>277</v>
+      </c>
+    </row>
+    <row r="1282">
+      <c r="A1282" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="B1282" t="inlineStr">
+        <is>
+          <t>CLRO</t>
+        </is>
+      </c>
+      <c r="C1282" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="1283">
+      <c r="A1283" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="B1283" t="inlineStr">
+        <is>
+          <t>OPENZ</t>
+        </is>
+      </c>
+      <c r="C1283" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="1284">
+      <c r="A1284" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="B1284" t="inlineStr">
+        <is>
+          <t>SOFI</t>
+        </is>
+      </c>
+      <c r="C1284" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="1285">
+      <c r="A1285" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="B1285" t="inlineStr">
+        <is>
+          <t>XXII</t>
+        </is>
+      </c>
+      <c r="C1285" t="inlineStr">
         <is>
           <t>Dropped</t>
         </is>

</xml_diff>

<commit_message>
Daily screener update: 2026-10-30
</commit_message>
<xml_diff>
--- a/screener_history.xlsx
+++ b/screener_history.xlsx
@@ -26440,7 +26440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G1285"/>
+  <dimension ref="A1:G1304"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -56004,6 +56004,437 @@
         </is>
       </c>
       <c r="C1285" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="1286">
+      <c r="A1286" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
+      <c r="B1286" t="inlineStr">
+        <is>
+          <t>ADT</t>
+        </is>
+      </c>
+      <c r="C1286" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D1286" t="n">
+        <v>9.970000000000001</v>
+      </c>
+      <c r="E1286" t="n">
+        <v>9.390000000000001</v>
+      </c>
+      <c r="F1286" t="n">
+        <v>11.13</v>
+      </c>
+      <c r="G1286" t="n">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="1287">
+      <c r="A1287" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
+      <c r="B1287" t="inlineStr">
+        <is>
+          <t>BHC</t>
+        </is>
+      </c>
+      <c r="C1287" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D1287" t="n">
+        <v>8.359999999999999</v>
+      </c>
+      <c r="E1287" t="n">
+        <v>7.58</v>
+      </c>
+      <c r="F1287" t="n">
+        <v>9.92</v>
+      </c>
+      <c r="G1287" t="n">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="1288">
+      <c r="A1288" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
+      <c r="B1288" t="inlineStr">
+        <is>
+          <t>CROX</t>
+        </is>
+      </c>
+      <c r="C1288" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D1288" t="n">
+        <v>144.52</v>
+      </c>
+      <c r="E1288" t="n">
+        <v>139.32</v>
+      </c>
+      <c r="F1288" t="n">
+        <v>154.91</v>
+      </c>
+      <c r="G1288" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="1289">
+      <c r="A1289" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
+      <c r="B1289" t="inlineStr">
+        <is>
+          <t>GKOS</t>
+        </is>
+      </c>
+      <c r="C1289" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D1289" t="n">
+        <v>221.52</v>
+      </c>
+      <c r="E1289" t="n">
+        <v>207.41</v>
+      </c>
+      <c r="F1289" t="n">
+        <v>249.74</v>
+      </c>
+      <c r="G1289" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="1290">
+      <c r="A1290" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
+      <c r="B1290" t="inlineStr">
+        <is>
+          <t>INSM</t>
+        </is>
+      </c>
+      <c r="C1290" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D1290" t="n">
+        <v>109.26</v>
+      </c>
+      <c r="E1290" t="n">
+        <v>103.78</v>
+      </c>
+      <c r="F1290" t="n">
+        <v>120.21</v>
+      </c>
+      <c r="G1290" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="1291">
+      <c r="A1291" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
+      <c r="B1291" t="inlineStr">
+        <is>
+          <t>MAX</t>
+        </is>
+      </c>
+      <c r="C1291" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D1291" t="n">
+        <v>14.4</v>
+      </c>
+      <c r="E1291" t="n">
+        <v>13.28</v>
+      </c>
+      <c r="F1291" t="n">
+        <v>16.64</v>
+      </c>
+      <c r="G1291" t="n">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="1292">
+      <c r="A1292" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
+      <c r="B1292" t="inlineStr">
+        <is>
+          <t>NUWE</t>
+        </is>
+      </c>
+      <c r="C1292" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D1292" t="n">
+        <v>7.15</v>
+      </c>
+      <c r="E1292" t="n">
+        <v>5.61</v>
+      </c>
+      <c r="F1292" t="n">
+        <v>10.23</v>
+      </c>
+      <c r="G1292" t="n">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="1293">
+      <c r="A1293" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
+      <c r="B1293" t="inlineStr">
+        <is>
+          <t>PRCH</t>
+        </is>
+      </c>
+      <c r="C1293" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D1293" t="n">
+        <v>20.88</v>
+      </c>
+      <c r="E1293" t="n">
+        <v>18.75</v>
+      </c>
+      <c r="F1293" t="n">
+        <v>25.14</v>
+      </c>
+      <c r="G1293" t="n">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="1294">
+      <c r="A1294" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
+      <c r="B1294" t="inlineStr">
+        <is>
+          <t>TDOC</t>
+        </is>
+      </c>
+      <c r="C1294" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D1294" t="n">
+        <v>8.779999999999999</v>
+      </c>
+      <c r="E1294" t="n">
+        <v>7.9</v>
+      </c>
+      <c r="F1294" t="n">
+        <v>10.54</v>
+      </c>
+      <c r="G1294" t="n">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="1295">
+      <c r="A1295" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
+      <c r="B1295" t="inlineStr">
+        <is>
+          <t>AXGN</t>
+        </is>
+      </c>
+      <c r="C1295" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="1296">
+      <c r="A1296" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
+      <c r="B1296" t="inlineStr">
+        <is>
+          <t>BOOM</t>
+        </is>
+      </c>
+      <c r="C1296" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="1297">
+      <c r="A1297" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
+      <c r="B1297" t="inlineStr">
+        <is>
+          <t>BRAI</t>
+        </is>
+      </c>
+      <c r="C1297" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="1298">
+      <c r="A1298" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
+      <c r="B1298" t="inlineStr">
+        <is>
+          <t>CDT</t>
+        </is>
+      </c>
+      <c r="C1298" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="1299">
+      <c r="A1299" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
+      <c r="B1299" t="inlineStr">
+        <is>
+          <t>GCTK</t>
+        </is>
+      </c>
+      <c r="C1299" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="1300">
+      <c r="A1300" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
+      <c r="B1300" t="inlineStr">
+        <is>
+          <t>LUNG</t>
+        </is>
+      </c>
+      <c r="C1300" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="1301">
+      <c r="A1301" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
+      <c r="B1301" t="inlineStr">
+        <is>
+          <t>SSP</t>
+        </is>
+      </c>
+      <c r="C1301" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="1302">
+      <c r="A1302" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
+      <c r="B1302" t="inlineStr">
+        <is>
+          <t>ULBI</t>
+        </is>
+      </c>
+      <c r="C1302" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="1303">
+      <c r="A1303" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
+      <c r="B1303" t="inlineStr">
+        <is>
+          <t>VRT</t>
+        </is>
+      </c>
+      <c r="C1303" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="1304">
+      <c r="A1304" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
+      <c r="B1304" t="inlineStr">
+        <is>
+          <t>WEN</t>
+        </is>
+      </c>
+      <c r="C1304" t="inlineStr">
         <is>
           <t>Dropped</t>
         </is>

</xml_diff>

<commit_message>
Daily screener update: 2026-10-31
</commit_message>
<xml_diff>
--- a/screener_history.xlsx
+++ b/screener_history.xlsx
@@ -26440,7 +26440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G1304"/>
+  <dimension ref="A1:G1322"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -56435,6 +56435,420 @@
         </is>
       </c>
       <c r="C1304" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="1305">
+      <c r="A1305" t="inlineStr">
+        <is>
+          <t>2026-10-31</t>
+        </is>
+      </c>
+      <c r="B1305" t="inlineStr">
+        <is>
+          <t>ACCO</t>
+        </is>
+      </c>
+      <c r="C1305" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D1305" t="n">
+        <v>5.46</v>
+      </c>
+      <c r="E1305" t="n">
+        <v>4.97</v>
+      </c>
+      <c r="F1305" t="n">
+        <v>6.44</v>
+      </c>
+      <c r="G1305" t="n">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="1306">
+      <c r="A1306" t="inlineStr">
+        <is>
+          <t>2026-10-31</t>
+        </is>
+      </c>
+      <c r="B1306" t="inlineStr">
+        <is>
+          <t>ASUR</t>
+        </is>
+      </c>
+      <c r="C1306" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D1306" t="n">
+        <v>9.199999999999999</v>
+      </c>
+      <c r="E1306" t="n">
+        <v>8.449999999999999</v>
+      </c>
+      <c r="F1306" t="n">
+        <v>10.69</v>
+      </c>
+      <c r="G1306" t="n">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="1307">
+      <c r="A1307" t="inlineStr">
+        <is>
+          <t>2026-10-31</t>
+        </is>
+      </c>
+      <c r="B1307" t="inlineStr">
+        <is>
+          <t>FMC</t>
+        </is>
+      </c>
+      <c r="C1307" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D1307" t="n">
+        <v>5.46</v>
+      </c>
+      <c r="E1307" t="n">
+        <v>5.16</v>
+      </c>
+      <c r="F1307" t="n">
+        <v>6.06</v>
+      </c>
+      <c r="G1307" t="n">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="1308">
+      <c r="A1308" t="inlineStr">
+        <is>
+          <t>2026-10-31</t>
+        </is>
+      </c>
+      <c r="B1308" t="inlineStr">
+        <is>
+          <t>INO</t>
+        </is>
+      </c>
+      <c r="C1308" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D1308" t="n">
+        <v>0.86</v>
+      </c>
+      <c r="E1308" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="F1308" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="G1308" t="n">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="1309">
+      <c r="A1309" t="inlineStr">
+        <is>
+          <t>2026-10-31</t>
+        </is>
+      </c>
+      <c r="B1309" t="inlineStr">
+        <is>
+          <t>OSPN</t>
+        </is>
+      </c>
+      <c r="C1309" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D1309" t="n">
+        <v>25.96</v>
+      </c>
+      <c r="E1309" t="n">
+        <v>24.41</v>
+      </c>
+      <c r="F1309" t="n">
+        <v>29.06</v>
+      </c>
+      <c r="G1309" t="n">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="1310">
+      <c r="A1310" t="inlineStr">
+        <is>
+          <t>2026-10-31</t>
+        </is>
+      </c>
+      <c r="B1310" t="inlineStr">
+        <is>
+          <t>RMNI</t>
+        </is>
+      </c>
+      <c r="C1310" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D1310" t="n">
+        <v>4.84</v>
+      </c>
+      <c r="E1310" t="n">
+        <v>4.7</v>
+      </c>
+      <c r="F1310" t="n">
+        <v>5.12</v>
+      </c>
+      <c r="G1310" t="n">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="1311">
+      <c r="A1311" t="inlineStr">
+        <is>
+          <t>2026-10-31</t>
+        </is>
+      </c>
+      <c r="B1311" t="inlineStr">
+        <is>
+          <t>ULH</t>
+        </is>
+      </c>
+      <c r="C1311" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D1311" t="n">
+        <v>19.72</v>
+      </c>
+      <c r="E1311" t="n">
+        <v>18.75</v>
+      </c>
+      <c r="F1311" t="n">
+        <v>21.65</v>
+      </c>
+      <c r="G1311" t="n">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="1312">
+      <c r="A1312" t="inlineStr">
+        <is>
+          <t>2026-10-31</t>
+        </is>
+      </c>
+      <c r="B1312" t="inlineStr">
+        <is>
+          <t>VIVK</t>
+        </is>
+      </c>
+      <c r="C1312" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D1312" t="n">
+        <v>1.75</v>
+      </c>
+      <c r="E1312" t="n">
+        <v>0.86</v>
+      </c>
+      <c r="F1312" t="n">
+        <v>3.53</v>
+      </c>
+      <c r="G1312" t="n">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="1313">
+      <c r="A1313" t="inlineStr">
+        <is>
+          <t>2026-10-31</t>
+        </is>
+      </c>
+      <c r="B1313" t="inlineStr">
+        <is>
+          <t>WKHS</t>
+        </is>
+      </c>
+      <c r="C1313" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="D1313" t="n">
+        <v>2.97</v>
+      </c>
+      <c r="E1313" t="n">
+        <v>2.75</v>
+      </c>
+      <c r="F1313" t="n">
+        <v>3.41</v>
+      </c>
+      <c r="G1313" t="n">
+        <v>227</v>
+      </c>
+    </row>
+    <row r="1314">
+      <c r="A1314" t="inlineStr">
+        <is>
+          <t>2026-10-31</t>
+        </is>
+      </c>
+      <c r="B1314" t="inlineStr">
+        <is>
+          <t>ADT</t>
+        </is>
+      </c>
+      <c r="C1314" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="1315">
+      <c r="A1315" t="inlineStr">
+        <is>
+          <t>2026-10-31</t>
+        </is>
+      </c>
+      <c r="B1315" t="inlineStr">
+        <is>
+          <t>BHC</t>
+        </is>
+      </c>
+      <c r="C1315" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="1316">
+      <c r="A1316" t="inlineStr">
+        <is>
+          <t>2026-10-31</t>
+        </is>
+      </c>
+      <c r="B1316" t="inlineStr">
+        <is>
+          <t>CROX</t>
+        </is>
+      </c>
+      <c r="C1316" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="1317">
+      <c r="A1317" t="inlineStr">
+        <is>
+          <t>2026-10-31</t>
+        </is>
+      </c>
+      <c r="B1317" t="inlineStr">
+        <is>
+          <t>GKOS</t>
+        </is>
+      </c>
+      <c r="C1317" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="1318">
+      <c r="A1318" t="inlineStr">
+        <is>
+          <t>2026-10-31</t>
+        </is>
+      </c>
+      <c r="B1318" t="inlineStr">
+        <is>
+          <t>INSM</t>
+        </is>
+      </c>
+      <c r="C1318" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="1319">
+      <c r="A1319" t="inlineStr">
+        <is>
+          <t>2026-10-31</t>
+        </is>
+      </c>
+      <c r="B1319" t="inlineStr">
+        <is>
+          <t>MAX</t>
+        </is>
+      </c>
+      <c r="C1319" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="1320">
+      <c r="A1320" t="inlineStr">
+        <is>
+          <t>2026-10-31</t>
+        </is>
+      </c>
+      <c r="B1320" t="inlineStr">
+        <is>
+          <t>NUWE</t>
+        </is>
+      </c>
+      <c r="C1320" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="1321">
+      <c r="A1321" t="inlineStr">
+        <is>
+          <t>2026-10-31</t>
+        </is>
+      </c>
+      <c r="B1321" t="inlineStr">
+        <is>
+          <t>PRCH</t>
+        </is>
+      </c>
+      <c r="C1321" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="1322">
+      <c r="A1322" t="inlineStr">
+        <is>
+          <t>2026-10-31</t>
+        </is>
+      </c>
+      <c r="B1322" t="inlineStr">
+        <is>
+          <t>TDOC</t>
+        </is>
+      </c>
+      <c r="C1322" t="inlineStr">
         <is>
           <t>Dropped</t>
         </is>

</xml_diff>